<commit_message>
feat(portal-web): GSAP storytelling landing 首頁 + 市集移至 /discover
- 新增 LandingView（/）：品牌 hero 進場動畫、三大商品類型
  pin 換頁區（ScrollTrigger + snap，reduced-motion 退化為直排）、
  待補充佔位區塊 x2、創作者/消費者雙 CTA
- MarketView 更名 DiscoverView，路徑 / → /discover，
  麵包屑與 CTA 連結同步更新
- landing i18n 文案（zh-TW / en）並同步 i18n.xlsx

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/portal-web/i18n.xlsx
+++ b/apps/portal-web/i18n.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="514">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="637">
   <si>
     <t>key</t>
   </si>
@@ -1553,6 +1553,375 @@
   </si>
   <si>
     <t>{storeName}: {title}</t>
+  </si>
+  <si>
+    <t>landing.screenLabel</t>
+  </si>
+  <si>
+    <t>品牌故事</t>
+  </si>
+  <si>
+    <t>Brand story</t>
+  </si>
+  <si>
+    <t>landing.hero.eyebrow</t>
+  </si>
+  <si>
+    <t>landing.hero.title1</t>
+  </si>
+  <si>
+    <t>把你的創作，</t>
+  </si>
+  <si>
+    <t>Put your creations</t>
+  </si>
+  <si>
+    <t>landing.hero.title2</t>
+  </si>
+  <si>
+    <t>交到{hl}手上</t>
+  </si>
+  <si>
+    <t>into {hl} hands</t>
+  </si>
+  <si>
+    <t>landing.hero.hl</t>
+  </si>
+  <si>
+    <t>對的人</t>
+  </si>
+  <si>
+    <t>the right</t>
+  </si>
+  <si>
+    <t>landing.hero.lede</t>
+  </si>
+  <si>
+    <t>Open Jam 是台灣創作者的數位商品平台。用自己的子網域開一間小店，上架音樂、攝影與電子書；買家免註冊，一個信箱就能把作品帶回家。</t>
+  </si>
+  <si>
+    <t>Open Jam is a digital goods platform for creators in Taiwan. Open a shop on your own subdomain and sell music, photography and e-books — buyers need no account, just an email to take your work home.</t>
+  </si>
+  <si>
+    <t>landing.hero.scrollHint</t>
+  </si>
+  <si>
+    <t>往下捲動，開始這段故事</t>
+  </si>
+  <si>
+    <t>Scroll down to start the story</t>
+  </si>
+  <si>
+    <t>landing.types.eyebrow</t>
+  </si>
+  <si>
+    <t>三種創作 · 一個舞台</t>
+  </si>
+  <si>
+    <t>Three crafts · One stage</t>
+  </si>
+  <si>
+    <t>landing.types.browse</t>
+  </si>
+  <si>
+    <t>去市集逛逛</t>
+  </si>
+  <si>
+    <t>Browse the market</t>
+  </si>
+  <si>
+    <t>landing.types.hint</t>
+  </si>
+  <si>
+    <t>繼續捲動，翻到下一頁</t>
+  </si>
+  <si>
+    <t>Keep scrolling to turn the page</t>
+  </si>
+  <si>
+    <t>landing.types.pageAria</t>
+  </si>
+  <si>
+    <t>切換到第 {n} 頁</t>
+  </si>
+  <si>
+    <t>Go to page {n}</t>
+  </si>
+  <si>
+    <t>landing.types.music.title</t>
+  </si>
+  <si>
+    <t>樂譜與音樂</t>
+  </si>
+  <si>
+    <t>Sheet music &amp; audio</t>
+  </si>
+  <si>
+    <t>landing.types.music.tagline</t>
+  </si>
+  <si>
+    <t>讓旋律離開你的房間</t>
+  </si>
+  <si>
+    <t>Let the melody leave your room</t>
+  </si>
+  <si>
+    <t>landing.types.music.desc</t>
+  </si>
+  <si>
+    <t>原創單曲、編曲樂譜、取樣素材與配樂授權——不論你寫的是鋼琴譜還是 Lo-fi 節拍，都能在這裡找到願意按下播放鍵的耳朵。</t>
+  </si>
+  <si>
+    <t>Original tracks, arrangements, sample packs and score licensing — whether you write piano sheets or lo-fi beats, ears willing to press play are waiting here.</t>
+  </si>
+  <si>
+    <t>landing.types.music.chips.0</t>
+  </si>
+  <si>
+    <t>原創單曲</t>
+  </si>
+  <si>
+    <t>Original tracks</t>
+  </si>
+  <si>
+    <t>landing.types.music.chips.1</t>
+  </si>
+  <si>
+    <t>編曲樂譜</t>
+  </si>
+  <si>
+    <t>Arrangements</t>
+  </si>
+  <si>
+    <t>landing.types.music.chips.2</t>
+  </si>
+  <si>
+    <t>取樣素材</t>
+  </si>
+  <si>
+    <t>Sample packs</t>
+  </si>
+  <si>
+    <t>landing.types.music.chips.3</t>
+  </si>
+  <si>
+    <t>配樂授權</t>
+  </si>
+  <si>
+    <t>Score licensing</t>
+  </si>
+  <si>
+    <t>landing.types.photo.title</t>
+  </si>
+  <si>
+    <t>攝影與照片集</t>
+  </si>
+  <si>
+    <t>Photography &amp; photo packs</t>
+  </si>
+  <si>
+    <t>landing.types.photo.tagline</t>
+  </si>
+  <si>
+    <t>快門之後，故事繼續</t>
+  </si>
+  <si>
+    <t>After the shutter, the story goes on</t>
+  </si>
+  <si>
+    <t>landing.types.photo.desc</t>
+  </si>
+  <si>
+    <t>風景寫真、人像企劃、街拍系列與高解析素材包。把硬碟裡沉睡的作品整理成照片集，讓每一次按下快門都有回音。</t>
+  </si>
+  <si>
+    <t>Landscape series, portrait projects, street collections and hi-res stock packs. Turn the work sleeping on your hard drive into photo packs that echo back.</t>
+  </si>
+  <si>
+    <t>landing.types.photo.chips.0</t>
+  </si>
+  <si>
+    <t>風景寫真</t>
+  </si>
+  <si>
+    <t>Landscape</t>
+  </si>
+  <si>
+    <t>landing.types.photo.chips.1</t>
+  </si>
+  <si>
+    <t>人像企劃</t>
+  </si>
+  <si>
+    <t>Portrait projects</t>
+  </si>
+  <si>
+    <t>landing.types.photo.chips.2</t>
+  </si>
+  <si>
+    <t>街拍系列</t>
+  </si>
+  <si>
+    <t>Street series</t>
+  </si>
+  <si>
+    <t>landing.types.photo.chips.3</t>
+  </si>
+  <si>
+    <t>素材圖庫</t>
+  </si>
+  <si>
+    <t>Stock packs</t>
+  </si>
+  <si>
+    <t>landing.types.ebook.title</t>
+  </si>
+  <si>
+    <t>電子書與文件</t>
+  </si>
+  <si>
+    <t>E-books &amp; documents</t>
+  </si>
+  <si>
+    <t>landing.types.ebook.tagline</t>
+  </si>
+  <si>
+    <t>文字，是最輕的行李</t>
+  </si>
+  <si>
+    <t>Words are the lightest luggage</t>
+  </si>
+  <si>
+    <t>landing.types.ebook.desc</t>
+  </si>
+  <si>
+    <t>小說、散文、教學手冊與獨立誌。從第一頁到最後一頁都由你決定——寫完、上架，讀者用一個信箱就能開始閱讀。</t>
+  </si>
+  <si>
+    <t>Novels, essays, tutorials and indie zines. From the first page to the last, it is all yours — finish it, publish it, and readers start reading with just an email.</t>
+  </si>
+  <si>
+    <t>landing.types.ebook.chips.0</t>
+  </si>
+  <si>
+    <t>小說散文</t>
+  </si>
+  <si>
+    <t>Novels &amp; essays</t>
+  </si>
+  <si>
+    <t>landing.types.ebook.chips.1</t>
+  </si>
+  <si>
+    <t>教學手冊</t>
+  </si>
+  <si>
+    <t>Tutorials</t>
+  </si>
+  <si>
+    <t>landing.types.ebook.chips.2</t>
+  </si>
+  <si>
+    <t>獨立誌</t>
+  </si>
+  <si>
+    <t>Indie zines</t>
+  </si>
+  <si>
+    <t>landing.types.ebook.chips.3</t>
+  </si>
+  <si>
+    <t>模板文件</t>
+  </si>
+  <si>
+    <t>Templates</t>
+  </si>
+  <si>
+    <t>landing.planned.badge</t>
+  </si>
+  <si>
+    <t>即將登場</t>
+  </si>
+  <si>
+    <t>Coming soon</t>
+  </si>
+  <si>
+    <t>landing.planned.title</t>
+  </si>
+  <si>
+    <t>更多故事，正在路上</t>
+  </si>
+  <si>
+    <t>More of the story is on its way</t>
+  </si>
+  <si>
+    <t>landing.planned.text</t>
+  </si>
+  <si>
+    <t>這個區塊還在企劃中，敬請期待。</t>
+  </si>
+  <si>
+    <t>This section is still in the works — stay tuned.</t>
+  </si>
+  <si>
+    <t>landing.cta.eyebrow</t>
+  </si>
+  <si>
+    <t>故事的下一頁，由你翻開</t>
+  </si>
+  <si>
+    <t>The next page of the story is yours to turn</t>
+  </si>
+  <si>
+    <t>landing.cta.creator.title</t>
+  </si>
+  <si>
+    <t>我是創作者</t>
+  </si>
+  <si>
+    <t>I'm a creator</t>
+  </si>
+  <si>
+    <t>landing.cta.creator.text</t>
+  </si>
+  <si>
+    <t>三分鐘開一間自己的店，把作品變成收入。</t>
+  </si>
+  <si>
+    <t>Open your own shop in three minutes and turn your work into income.</t>
+  </si>
+  <si>
+    <t>landing.cta.creator.button</t>
+  </si>
+  <si>
+    <t>免費開店上架</t>
+  </si>
+  <si>
+    <t>Start selling for free</t>
+  </si>
+  <si>
+    <t>landing.cta.buyer.title</t>
+  </si>
+  <si>
+    <t>我想找靈感</t>
+  </si>
+  <si>
+    <t>I'm looking for inspiration</t>
+  </si>
+  <si>
+    <t>landing.cta.buyer.text</t>
+  </si>
+  <si>
+    <t>免註冊、憑信箱購買，馬上開始探索市集。</t>
+  </si>
+  <si>
+    <t>No sign-up needed — buy with just an email and start exploring now.</t>
+  </si>
+  <si>
+    <t>landing.cta.buyer.button</t>
+  </si>
+  <si>
+    <t>瀏覽市集作品</t>
   </si>
 </sst>
 </file>
@@ -1938,7 +2307,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C182"/>
+  <dimension ref="A1:C224"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -3947,6 +4316,468 @@
         <v>513</v>
       </c>
     </row>
+    <row r="183" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A183" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="B183" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="C183" s="2" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A184" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="B184" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C184" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A185" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="B185" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="C185" s="2" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A186" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="B186" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="C186" s="2" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A187" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="B187" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="C187" s="2" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A188" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="B188" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="C188" s="2" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="B189" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="C189" s="2" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="190" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A190" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="B190" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="C190" s="2" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A191" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="B191" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="C191" s="2" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A192" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="B192" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="C192" s="2" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A193" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="B193" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="C193" s="2" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A194" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="B194" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="C194" s="2" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="195" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A195" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="B195" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="C195" s="2" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="196" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A196" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="B196" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="C196" s="2" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A197" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="B197" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="C197" s="2" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A198" s="2" t="s">
+        <v>557</v>
+      </c>
+      <c r="B198" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="C198" s="2" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="199" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A199" s="2" t="s">
+        <v>560</v>
+      </c>
+      <c r="B199" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="C199" s="2" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="200" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A200" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B200" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="C200" s="2" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A201" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="B201" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="C201" s="2" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="202" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A202" s="2" t="s">
+        <v>569</v>
+      </c>
+      <c r="B202" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="C202" s="2" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="203" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A203" s="2" t="s">
+        <v>572</v>
+      </c>
+      <c r="B203" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="C203" s="2" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="204" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A204" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="B204" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="C204" s="2" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="205" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A205" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="B205" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="C205" s="2" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="206" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A206" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="B206" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="C206" s="2" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="207" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A207" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="B207" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="C207" s="2" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="208" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A208" s="2" t="s">
+        <v>587</v>
+      </c>
+      <c r="B208" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="C208" s="2" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="209" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A209" s="2" t="s">
+        <v>590</v>
+      </c>
+      <c r="B209" s="2" t="s">
+        <v>591</v>
+      </c>
+      <c r="C209" s="2" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="210" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A210" s="2" t="s">
+        <v>593</v>
+      </c>
+      <c r="B210" s="2" t="s">
+        <v>594</v>
+      </c>
+      <c r="C210" s="2" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="211" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A211" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B211" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="C211" s="2" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="212" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A212" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="B212" s="2" t="s">
+        <v>600</v>
+      </c>
+      <c r="C212" s="2" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="213" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A213" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="B213" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="C213" s="2" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="214" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A214" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="B214" s="2" t="s">
+        <v>606</v>
+      </c>
+      <c r="C214" s="2" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A215" s="2" t="s">
+        <v>608</v>
+      </c>
+      <c r="B215" s="2" t="s">
+        <v>609</v>
+      </c>
+      <c r="C215" s="2" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="216" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A216" s="2" t="s">
+        <v>611</v>
+      </c>
+      <c r="B216" s="2" t="s">
+        <v>612</v>
+      </c>
+      <c r="C216" s="2" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A217" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="B217" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="C217" s="2" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="218" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A218" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="B218" s="2" t="s">
+        <v>618</v>
+      </c>
+      <c r="C218" s="2" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="219" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A219" s="2" t="s">
+        <v>620</v>
+      </c>
+      <c r="B219" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="C219" s="2" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="220" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A220" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="B220" s="2" t="s">
+        <v>624</v>
+      </c>
+      <c r="C220" s="2" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="221" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A221" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B221" s="2" t="s">
+        <v>627</v>
+      </c>
+      <c r="C221" s="2" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="222" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A222" s="2" t="s">
+        <v>629</v>
+      </c>
+      <c r="B222" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="C222" s="2" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="223" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A223" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="B223" s="2" t="s">
+        <v>633</v>
+      </c>
+      <c r="C223" s="2" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="224" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A224" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="B224" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="C224" s="2" t="s">
+        <v>538</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat(portal-web): landing 改版為六區塊 storytelling 架構
- Hero 品牌宣言：收藏/支持/記得三色 highlight、漂浮商品卡、波形
- Pinned Product Story：同舞台三章推進（非換頁蓋板），每章列出
  可販售項目——音樂（播放器+波形）、攝影（preset before/after
  隨捲動拉動）、電子書（翻頁書+章節卡），rail 可點擊跳章
- 新增 Creator Workflow 五步驟（漸層線 scrub 長出）、
  Consumer Experience collage、Why Open Jam 理念四卡
- 修正 snap 方向性/慣性甩章（directional+inertia: false）與
  grid auto track 被原始圖寬撐開推出視窗的問題

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/portal-web/i18n.xlsx
+++ b/apps/portal-web/i18n.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="637">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="722">
   <si>
     <t>key</t>
   </si>
@@ -1567,40 +1567,46 @@
     <t>landing.hero.eyebrow</t>
   </si>
   <si>
-    <t>landing.hero.title1</t>
-  </si>
-  <si>
-    <t>把你的創作，</t>
-  </si>
-  <si>
-    <t>Put your creations</t>
-  </si>
-  <si>
-    <t>landing.hero.title2</t>
-  </si>
-  <si>
-    <t>交到{hl}手上</t>
-  </si>
-  <si>
-    <t>into {hl} hands</t>
-  </si>
-  <si>
-    <t>landing.hero.hl</t>
-  </si>
-  <si>
-    <t>對的人</t>
-  </si>
-  <si>
-    <t>the right</t>
-  </si>
-  <si>
-    <t>landing.hero.lede</t>
-  </si>
-  <si>
-    <t>Open Jam 是台灣創作者的數位商品平台。用自己的子網域開一間小店，上架音樂、攝影與電子書；買家免註冊，一個信箱就能把作品帶回家。</t>
-  </si>
-  <si>
-    <t>Open Jam is a digital goods platform for creators in Taiwan. Open a shop on your own subdomain and sell music, photography and e-books — buyers need no account, just an email to take your work home.</t>
+    <t>landing.hero.title</t>
+  </si>
+  <si>
+    <t>把你的創作，變成有人{collect}、{support}、{remember}的存在。</t>
+  </si>
+  <si>
+    <t>Turn your creative work into something people can {collect}, {support} and {remember}.</t>
+  </si>
+  <si>
+    <t>landing.hero.collect</t>
+  </si>
+  <si>
+    <t>collect</t>
+  </si>
+  <si>
+    <t>landing.hero.support</t>
+  </si>
+  <si>
+    <t>支持</t>
+  </si>
+  <si>
+    <t>support</t>
+  </si>
+  <si>
+    <t>landing.hero.remember</t>
+  </si>
+  <si>
+    <t>記得</t>
+  </si>
+  <si>
+    <t>remember</t>
+  </si>
+  <si>
+    <t>landing.hero.slogan</t>
+  </si>
+  <si>
+    <t>獨立創作的數位市集——你的作品，找得到它的人。</t>
+  </si>
+  <si>
+    <t>A home for independent work — where what you make finds its people.</t>
   </si>
   <si>
     <t>landing.hero.scrollHint</t>
@@ -1612,7 +1618,7 @@
     <t>Scroll down to start the story</t>
   </si>
   <si>
-    <t>landing.types.eyebrow</t>
+    <t>landing.story.eyebrow</t>
   </si>
   <si>
     <t>三種創作 · 一個舞台</t>
@@ -1621,247 +1627,493 @@
     <t>Three crafts · One stage</t>
   </si>
   <si>
-    <t>landing.types.browse</t>
-  </si>
-  <si>
-    <t>去市集逛逛</t>
-  </si>
-  <si>
-    <t>Browse the market</t>
-  </si>
-  <si>
-    <t>landing.types.hint</t>
-  </si>
-  <si>
-    <t>繼續捲動，翻到下一頁</t>
-  </si>
-  <si>
-    <t>Keep scrolling to turn the page</t>
-  </si>
-  <si>
-    <t>landing.types.pageAria</t>
-  </si>
-  <si>
-    <t>切換到第 {n} 頁</t>
-  </si>
-  <si>
-    <t>Go to page {n}</t>
-  </si>
-  <si>
-    <t>landing.types.music.title</t>
-  </si>
-  <si>
-    <t>樂譜與音樂</t>
-  </si>
-  <si>
-    <t>Sheet music &amp; audio</t>
-  </si>
-  <si>
-    <t>landing.types.music.tagline</t>
-  </si>
-  <si>
-    <t>讓旋律離開你的房間</t>
-  </si>
-  <si>
-    <t>Let the melody leave your room</t>
-  </si>
-  <si>
-    <t>landing.types.music.desc</t>
-  </si>
-  <si>
-    <t>原創單曲、編曲樂譜、取樣素材與配樂授權——不論你寫的是鋼琴譜還是 Lo-fi 節拍，都能在這裡找到願意按下播放鍵的耳朵。</t>
-  </si>
-  <si>
-    <t>Original tracks, arrangements, sample packs and score licensing — whether you write piano sheets or lo-fi beats, ears willing to press play are waiting here.</t>
-  </si>
-  <si>
-    <t>landing.types.music.chips.0</t>
-  </si>
-  <si>
-    <t>原創單曲</t>
-  </si>
-  <si>
-    <t>Original tracks</t>
-  </si>
-  <si>
-    <t>landing.types.music.chips.1</t>
-  </si>
-  <si>
-    <t>編曲樂譜</t>
-  </si>
-  <si>
-    <t>Arrangements</t>
-  </si>
-  <si>
-    <t>landing.types.music.chips.2</t>
-  </si>
-  <si>
-    <t>取樣素材</t>
+    <t>landing.story.title</t>
+  </si>
+  <si>
+    <t>創作者能在這裡賣什麼？</t>
+  </si>
+  <si>
+    <t>What can creators sell here?</t>
+  </si>
+  <si>
+    <t>landing.story.hint</t>
+  </si>
+  <si>
+    <t>繼續捲動，故事往下走</t>
+  </si>
+  <si>
+    <t>Keep scrolling — the story goes on</t>
+  </si>
+  <si>
+    <t>landing.story.pageAria</t>
+  </si>
+  <si>
+    <t>切換到第 {n} 章</t>
+  </si>
+  <si>
+    <t>Go to chapter {n}</t>
+  </si>
+  <si>
+    <t>landing.story.music.label</t>
+  </si>
+  <si>
+    <t>音樂</t>
+  </si>
+  <si>
+    <t>Music</t>
+  </si>
+  <si>
+    <t>landing.story.music.title</t>
+  </si>
+  <si>
+    <t>從 demo 到完整作品</t>
+  </si>
+  <si>
+    <t>From rough demos to finished records</t>
+  </si>
+  <si>
+    <t>landing.story.music.desc</t>
+  </si>
+  <si>
+    <t>一段 demo、一包取樣素材、一份六線譜——把練團室裡的聲音，變成別人創作與練習的起點。</t>
+  </si>
+  <si>
+    <t>A demo, a sample pack, a set of tabs — turn the sound in your practice room into the starting point of someone else's craft.</t>
+  </si>
+  <si>
+    <t>landing.story.music.chips.0</t>
+  </si>
+  <si>
+    <t>Demo</t>
+  </si>
+  <si>
+    <t>Demos</t>
+  </si>
+  <si>
+    <t>landing.story.music.chips.1</t>
+  </si>
+  <si>
+    <t>Sample Pack</t>
   </si>
   <si>
     <t>Sample packs</t>
   </si>
   <si>
-    <t>landing.types.music.chips.3</t>
-  </si>
-  <si>
-    <t>配樂授權</t>
-  </si>
-  <si>
-    <t>Score licensing</t>
-  </si>
-  <si>
-    <t>landing.types.photo.title</t>
-  </si>
-  <si>
-    <t>攝影與照片集</t>
-  </si>
-  <si>
-    <t>Photography &amp; photo packs</t>
-  </si>
-  <si>
-    <t>landing.types.photo.tagline</t>
-  </si>
-  <si>
-    <t>快門之後，故事繼續</t>
-  </si>
-  <si>
-    <t>After the shutter, the story goes on</t>
-  </si>
-  <si>
-    <t>landing.types.photo.desc</t>
-  </si>
-  <si>
-    <t>風景寫真、人像企劃、街拍系列與高解析素材包。把硬碟裡沉睡的作品整理成照片集，讓每一次按下快門都有回音。</t>
-  </si>
-  <si>
-    <t>Landscape series, portrait projects, street collections and hi-res stock packs. Turn the work sleeping on your hard drive into photo packs that echo back.</t>
-  </si>
-  <si>
-    <t>landing.types.photo.chips.0</t>
-  </si>
-  <si>
-    <t>風景寫真</t>
-  </si>
-  <si>
-    <t>Landscape</t>
-  </si>
-  <si>
-    <t>landing.types.photo.chips.1</t>
-  </si>
-  <si>
-    <t>人像企劃</t>
-  </si>
-  <si>
-    <t>Portrait projects</t>
-  </si>
-  <si>
-    <t>landing.types.photo.chips.2</t>
-  </si>
-  <si>
-    <t>街拍系列</t>
-  </si>
-  <si>
-    <t>Street series</t>
-  </si>
-  <si>
-    <t>landing.types.photo.chips.3</t>
-  </si>
-  <si>
-    <t>素材圖庫</t>
-  </si>
-  <si>
-    <t>Stock packs</t>
-  </si>
-  <si>
-    <t>landing.types.ebook.title</t>
-  </si>
-  <si>
-    <t>電子書與文件</t>
-  </si>
-  <si>
-    <t>E-books &amp; documents</t>
-  </si>
-  <si>
-    <t>landing.types.ebook.tagline</t>
-  </si>
-  <si>
-    <t>文字，是最輕的行李</t>
-  </si>
-  <si>
-    <t>Words are the lightest luggage</t>
-  </si>
-  <si>
-    <t>landing.types.ebook.desc</t>
-  </si>
-  <si>
-    <t>小說、散文、教學手冊與獨立誌。從第一頁到最後一頁都由你決定——寫完、上架，讀者用一個信箱就能開始閱讀。</t>
-  </si>
-  <si>
-    <t>Novels, essays, tutorials and indie zines. From the first page to the last, it is all yours — finish it, publish it, and readers start reading with just an email.</t>
-  </si>
-  <si>
-    <t>landing.types.ebook.chips.0</t>
-  </si>
-  <si>
-    <t>小說散文</t>
-  </si>
-  <si>
-    <t>Novels &amp; essays</t>
-  </si>
-  <si>
-    <t>landing.types.ebook.chips.1</t>
-  </si>
-  <si>
-    <t>教學手冊</t>
+    <t>landing.story.music.chips.2</t>
+  </si>
+  <si>
+    <t>Tabs 六線譜</t>
+  </si>
+  <si>
+    <t>Tabs</t>
+  </si>
+  <si>
+    <t>landing.story.music.chips.3</t>
+  </si>
+  <si>
+    <t>Backing Track</t>
+  </si>
+  <si>
+    <t>Backing tracks</t>
+  </si>
+  <si>
+    <t>landing.story.music.chips.4</t>
+  </si>
+  <si>
+    <t>線上課程</t>
+  </si>
+  <si>
+    <t>Lessons</t>
+  </si>
+  <si>
+    <t>landing.story.photo.label</t>
+  </si>
+  <si>
+    <t>攝影</t>
+  </si>
+  <si>
+    <t>landing.story.photo.title</t>
+  </si>
+  <si>
+    <t>快門之後，作品的第二人生</t>
+  </si>
+  <si>
+    <t>After the shutter, a second life</t>
+  </si>
+  <si>
+    <t>landing.story.photo.desc</t>
+  </si>
+  <si>
+    <t>調色預設、照片包、可掛上牆的輸出與桌布——硬碟裡沉睡的作品，都有人願意帶回家。</t>
+  </si>
+  <si>
+    <t>Presets, photo packs, prints for the wall and wallpapers — the work sleeping on your drive is something people will take home.</t>
+  </si>
+  <si>
+    <t>landing.story.photo.chips.0</t>
+  </si>
+  <si>
+    <t>Lightroom Presets</t>
+  </si>
+  <si>
+    <t>Presets</t>
+  </si>
+  <si>
+    <t>landing.story.photo.chips.1</t>
+  </si>
+  <si>
+    <t>Prints 輸出</t>
+  </si>
+  <si>
+    <t>Prints</t>
+  </si>
+  <si>
+    <t>landing.story.photo.chips.2</t>
+  </si>
+  <si>
+    <t>Photo Pack</t>
+  </si>
+  <si>
+    <t>Photo packs</t>
+  </si>
+  <si>
+    <t>landing.story.photo.chips.3</t>
+  </si>
+  <si>
+    <t>Wallpaper</t>
+  </si>
+  <si>
+    <t>Wallpapers</t>
+  </si>
+  <si>
+    <t>landing.story.ebook.label</t>
+  </si>
+  <si>
+    <t>E-book</t>
+  </si>
+  <si>
+    <t>landing.story.ebook.title</t>
+  </si>
+  <si>
+    <t>文字，直接送到讀者手上</t>
+  </si>
+  <si>
+    <t>Words, delivered straight to readers</t>
+  </si>
+  <si>
+    <t>landing.story.ebook.desc</t>
+  </si>
+  <si>
+    <t>一本獨立誌、一份教學指南、一章一章寫下去的長篇——不用等出版社點頭，寫完就能上架。</t>
+  </si>
+  <si>
+    <t>A zine, a guide, a long-form story written chapter by chapter — no publisher's nod needed, publish the day you finish.</t>
+  </si>
+  <si>
+    <t>landing.story.ebook.chips.0</t>
+  </si>
+  <si>
+    <t>Guide 教學</t>
+  </si>
+  <si>
+    <t>Guides</t>
+  </si>
+  <si>
+    <t>landing.story.ebook.chips.1</t>
+  </si>
+  <si>
+    <t>Zine 獨立誌</t>
+  </si>
+  <si>
+    <t>Zines</t>
+  </si>
+  <si>
+    <t>landing.story.ebook.chips.2</t>
+  </si>
+  <si>
+    <t>PDF</t>
+  </si>
+  <si>
+    <t>PDFs</t>
+  </si>
+  <si>
+    <t>landing.story.ebook.chips.3</t>
+  </si>
+  <si>
+    <t>Tutorial</t>
   </si>
   <si>
     <t>Tutorials</t>
   </si>
   <si>
-    <t>landing.types.ebook.chips.2</t>
-  </si>
-  <si>
-    <t>獨立誌</t>
-  </si>
-  <si>
-    <t>Indie zines</t>
-  </si>
-  <si>
-    <t>landing.types.ebook.chips.3</t>
-  </si>
-  <si>
-    <t>模板文件</t>
-  </si>
-  <si>
-    <t>Templates</t>
-  </si>
-  <si>
-    <t>landing.planned.badge</t>
-  </si>
-  <si>
-    <t>即將登場</t>
-  </si>
-  <si>
-    <t>Coming soon</t>
-  </si>
-  <si>
-    <t>landing.planned.title</t>
-  </si>
-  <si>
-    <t>更多故事，正在路上</t>
-  </si>
-  <si>
-    <t>More of the story is on its way</t>
-  </si>
-  <si>
-    <t>landing.planned.text</t>
-  </si>
-  <si>
-    <t>這個區塊還在企劃中，敬請期待。</t>
-  </si>
-  <si>
-    <t>This section is still in the works — stay tuned.</t>
+    <t>landing.flow.eyebrow</t>
+  </si>
+  <si>
+    <t>創作者旅程</t>
+  </si>
+  <si>
+    <t>The creator journey</t>
+  </si>
+  <si>
+    <t>landing.flow.title</t>
+  </si>
+  <si>
+    <t>從上傳到開店，只要幾分鐘。</t>
+  </si>
+  <si>
+    <t>From upload to storefront in minutes.</t>
+  </si>
+  <si>
+    <t>landing.flow.sub</t>
+  </si>
+  <si>
+    <t>不是只有展示——這裡是真的能收到支持的地方。</t>
+  </si>
+  <si>
+    <t>Not just a showcase — this is where support actually reaches you.</t>
+  </si>
+  <si>
+    <t>landing.flow.steps.0.title</t>
+  </si>
+  <si>
+    <t>上傳作品</t>
+  </si>
+  <si>
+    <t>Upload your work</t>
+  </si>
+  <si>
+    <t>landing.flow.steps.0.text</t>
+  </si>
+  <si>
+    <t>音檔、照片、PDF，拖進來就好。</t>
+  </si>
+  <si>
+    <t>Audio, photos, PDFs — just drag them in.</t>
+  </si>
+  <si>
+    <t>landing.flow.steps.1.title</t>
+  </si>
+  <si>
+    <t>設定價格</t>
+  </si>
+  <si>
+    <t>Set your price</t>
+  </si>
+  <si>
+    <t>landing.flow.steps.1.text</t>
+  </si>
+  <si>
+    <t>定價或自由贊助，由你決定。</t>
+  </si>
+  <si>
+    <t>Fixed price or pay-what-you-want — your call.</t>
+  </si>
+  <si>
+    <t>landing.flow.steps.2.title</t>
+  </si>
+  <si>
+    <t>建立創作者頁</t>
+  </si>
+  <si>
+    <t>Build your storefront</t>
+  </si>
+  <si>
+    <t>landing.flow.steps.2.text</t>
+  </si>
+  <si>
+    <t>你的子網域小店，一分鐘開張。</t>
+  </si>
+  <si>
+    <t>Your own subdomain shop, open in a minute.</t>
+  </si>
+  <si>
+    <t>landing.flow.steps.3.title</t>
+  </si>
+  <si>
+    <t>分享連結</t>
+  </si>
+  <si>
+    <t>Share the link</t>
+  </si>
+  <si>
+    <t>landing.flow.steps.3.text</t>
+  </si>
+  <si>
+    <t>貼在 IG bio、影片說明欄、任何地方。</t>
+  </si>
+  <si>
+    <t>Drop it in your bio, video descriptions, anywhere.</t>
+  </si>
+  <si>
+    <t>landing.flow.steps.4.title</t>
+  </si>
+  <si>
+    <t>收到支持</t>
+  </si>
+  <si>
+    <t>Get supported</t>
+  </si>
+  <si>
+    <t>landing.flow.steps.4.text</t>
+  </si>
+  <si>
+    <t>買家免註冊，一封信箱就能付款下載。</t>
+  </si>
+  <si>
+    <t>Buyers pay and download with just an email.</t>
+  </si>
+  <si>
+    <t>landing.discover.eyebrow</t>
+  </si>
+  <si>
+    <t>給探索者</t>
+  </si>
+  <si>
+    <t>For explorers</t>
+  </si>
+  <si>
+    <t>landing.discover.title</t>
+  </si>
+  <si>
+    <t>在它們成為主流之前，先發現它們。</t>
+  </si>
+  <si>
+    <t>Discover independent works before they become mainstream.</t>
+  </si>
+  <si>
+    <t>landing.discover.text</t>
+  </si>
+  <si>
+    <t>每一次購買，都是直接支持一位創作者。逛市集、追蹤喜歡的店、把作品收進自己的收藏庫——隨時回來下載。</t>
+  </si>
+  <si>
+    <t>Every purchase directly supports a creator. Browse the market, follow the shops you love, and keep every find in your library — ready to download anytime.</t>
+  </si>
+  <si>
+    <t>landing.discover.gridLabel</t>
+  </si>
+  <si>
+    <t>市集精選</t>
+  </si>
+  <si>
+    <t>Marketplace picks</t>
+  </si>
+  <si>
+    <t>landing.discover.profileLabel</t>
+  </si>
+  <si>
+    <t>創作者主頁</t>
+  </si>
+  <si>
+    <t>Creator profile</t>
+  </si>
+  <si>
+    <t>landing.discover.favLabel</t>
+  </si>
+  <si>
+    <t>我的收藏</t>
+  </si>
+  <si>
+    <t>My library</t>
+  </si>
+  <si>
+    <t>landing.discover.follow</t>
+  </si>
+  <si>
+    <t>追蹤</t>
+  </si>
+  <si>
+    <t>Follow</t>
+  </si>
+  <si>
+    <t>landing.why.eyebrow</t>
+  </si>
+  <si>
+    <t>為什麼是 Open Jam</t>
+  </si>
+  <si>
+    <t>Why Open Jam</t>
+  </si>
+  <si>
+    <t>landing.why.title</t>
+  </si>
+  <si>
+    <t>我們相信的事</t>
+  </si>
+  <si>
+    <t>What we believe in</t>
+  </si>
+  <si>
+    <t>landing.why.items.0.title</t>
+  </si>
+  <si>
+    <t>沒有演算法綁架</t>
+  </si>
+  <si>
+    <t>No algorithm hostage</t>
+  </si>
+  <si>
+    <t>landing.why.items.0.text</t>
+  </si>
+  <si>
+    <t>作品不必討好推薦系統，追蹤你的人，就是真心想看你的人。</t>
+  </si>
+  <si>
+    <t>Your work doesn't have to please a feed. The people following you actually want to see you.</t>
+  </si>
+  <si>
+    <t>landing.why.items.1.title</t>
+  </si>
+  <si>
+    <t>專注創作者與作品</t>
+  </si>
+  <si>
+    <t>Creators and works first</t>
+  </si>
+  <si>
+    <t>landing.why.items.1.text</t>
+  </si>
+  <si>
+    <t>乾淨的店面、直接的支持，沒有廣告與雜訊。</t>
+  </si>
+  <si>
+    <t>Clean storefronts and direct support — no ads, no noise.</t>
+  </si>
+  <si>
+    <t>landing.why.items.2.title</t>
+  </si>
+  <si>
+    <t>小型創作者快速上架</t>
+  </si>
+  <si>
+    <t>Built for small creators</t>
+  </si>
+  <si>
+    <t>landing.why.items.2.text</t>
+  </si>
+  <si>
+    <t>不用談合約、不用等審核，今天上架、今天開賣。</t>
+  </si>
+  <si>
+    <t>No contracts, no gatekeeping — publish today, sell today.</t>
+  </si>
+  <si>
+    <t>landing.why.items.3.title</t>
+  </si>
+  <si>
+    <t>音樂人友善，不只音樂</t>
+  </si>
+  <si>
+    <t>Musician-friendly, not music-only</t>
+  </si>
+  <si>
+    <t>landing.why.items.3.text</t>
+  </si>
+  <si>
+    <t>從波形、照片到文字，每種創作都是第一等公民。</t>
+  </si>
+  <si>
+    <t>From waveforms to photos to words, every craft is a first-class citizen.</t>
   </si>
   <si>
     <t>landing.cta.eyebrow</t>
@@ -1894,10 +2146,10 @@
     <t>landing.cta.creator.button</t>
   </si>
   <si>
-    <t>免費開店上架</t>
-  </si>
-  <si>
-    <t>Start selling for free</t>
+    <t>開始販售你的作品</t>
+  </si>
+  <si>
+    <t>Start selling your work</t>
   </si>
   <si>
     <t>landing.cta.buyer.title</t>
@@ -1921,7 +2173,10 @@
     <t>landing.cta.buyer.button</t>
   </si>
   <si>
-    <t>瀏覽市集作品</t>
+    <t>探索創作者</t>
+  </si>
+  <si>
+    <t>Explore creators</t>
   </si>
 </sst>
 </file>
@@ -2307,7 +2562,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C224"/>
+  <dimension ref="A1:C253"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -4354,428 +4609,747 @@
         <v>521</v>
       </c>
       <c r="B186" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C186" s="2" t="s">
         <v>522</v>
-      </c>
-      <c r="C186" s="2" t="s">
-        <v>523</v>
       </c>
     </row>
     <row r="187" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="B187" s="2" t="s">
         <v>524</v>
       </c>
-      <c r="B187" s="2" t="s">
+      <c r="C187" s="2" t="s">
         <v>525</v>
-      </c>
-      <c r="C187" s="2" t="s">
-        <v>526</v>
       </c>
     </row>
     <row r="188" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="B188" s="2" t="s">
         <v>527</v>
       </c>
-      <c r="B188" s="2" t="s">
+      <c r="C188" s="2" t="s">
         <v>528</v>
-      </c>
-      <c r="C188" s="2" t="s">
-        <v>529</v>
       </c>
     </row>
     <row r="189" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="B189" s="2" t="s">
         <v>530</v>
       </c>
-      <c r="B189" s="2" t="s">
+      <c r="C189" s="2" t="s">
         <v>531</v>
-      </c>
-      <c r="C189" s="2" t="s">
-        <v>532</v>
       </c>
     </row>
     <row r="190" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="B190" s="2" t="s">
         <v>533</v>
       </c>
-      <c r="B190" s="2" t="s">
+      <c r="C190" s="2" t="s">
         <v>534</v>
-      </c>
-      <c r="C190" s="2" t="s">
-        <v>535</v>
       </c>
     </row>
     <row r="191" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="B191" s="2" t="s">
         <v>536</v>
       </c>
-      <c r="B191" s="2" t="s">
+      <c r="C191" s="2" t="s">
         <v>537</v>
-      </c>
-      <c r="C191" s="2" t="s">
-        <v>538</v>
       </c>
     </row>
     <row r="192" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="B192" s="2" t="s">
         <v>539</v>
       </c>
-      <c r="B192" s="2" t="s">
+      <c r="C192" s="2" t="s">
         <v>540</v>
-      </c>
-      <c r="C192" s="2" t="s">
-        <v>541</v>
       </c>
     </row>
     <row r="193" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="B193" s="2" t="s">
         <v>542</v>
       </c>
-      <c r="B193" s="2" t="s">
+      <c r="C193" s="2" t="s">
         <v>543</v>
-      </c>
-      <c r="C193" s="2" t="s">
-        <v>544</v>
       </c>
     </row>
     <row r="194" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="B194" s="2" t="s">
         <v>545</v>
       </c>
-      <c r="B194" s="2" t="s">
+      <c r="C194" s="2" t="s">
         <v>546</v>
-      </c>
-      <c r="C194" s="2" t="s">
-        <v>547</v>
       </c>
     </row>
     <row r="195" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="B195" s="2" t="s">
         <v>548</v>
       </c>
-      <c r="B195" s="2" t="s">
+      <c r="C195" s="2" t="s">
         <v>549</v>
-      </c>
-      <c r="C195" s="2" t="s">
-        <v>550</v>
       </c>
     </row>
     <row r="196" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="B196" s="2" t="s">
         <v>551</v>
       </c>
-      <c r="B196" s="2" t="s">
+      <c r="C196" s="2" t="s">
         <v>552</v>
-      </c>
-      <c r="C196" s="2" t="s">
-        <v>553</v>
       </c>
     </row>
     <row r="197" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="B197" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="B197" s="2" t="s">
+      <c r="C197" s="2" t="s">
         <v>555</v>
-      </c>
-      <c r="C197" s="2" t="s">
-        <v>556</v>
       </c>
     </row>
     <row r="198" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
+        <v>556</v>
+      </c>
+      <c r="B198" s="2" t="s">
         <v>557</v>
       </c>
-      <c r="B198" s="2" t="s">
+      <c r="C198" s="2" t="s">
         <v>558</v>
-      </c>
-      <c r="C198" s="2" t="s">
-        <v>559</v>
       </c>
     </row>
     <row r="199" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
+        <v>559</v>
+      </c>
+      <c r="B199" s="2" t="s">
         <v>560</v>
       </c>
-      <c r="B199" s="2" t="s">
+      <c r="C199" s="2" t="s">
         <v>561</v>
-      </c>
-      <c r="C199" s="2" t="s">
-        <v>562</v>
       </c>
     </row>
     <row r="200" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="B200" s="2" t="s">
         <v>563</v>
       </c>
-      <c r="B200" s="2" t="s">
+      <c r="C200" s="2" t="s">
         <v>564</v>
-      </c>
-      <c r="C200" s="2" t="s">
-        <v>565</v>
       </c>
     </row>
     <row r="201" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B201" s="2" t="s">
         <v>566</v>
       </c>
-      <c r="B201" s="2" t="s">
+      <c r="C201" s="2" t="s">
         <v>567</v>
-      </c>
-      <c r="C201" s="2" t="s">
-        <v>568</v>
       </c>
     </row>
     <row r="202" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="B202" s="2" t="s">
         <v>569</v>
       </c>
-      <c r="B202" s="2" t="s">
+      <c r="C202" s="2" t="s">
         <v>570</v>
-      </c>
-      <c r="C202" s="2" t="s">
-        <v>571</v>
       </c>
     </row>
     <row r="203" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="B203" s="2" t="s">
         <v>572</v>
       </c>
-      <c r="B203" s="2" t="s">
-        <v>573</v>
-      </c>
       <c r="C203" s="2" t="s">
-        <v>574</v>
+        <v>60</v>
       </c>
     </row>
     <row r="204" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="B204" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="C204" s="2" t="s">
         <v>575</v>
-      </c>
-      <c r="B204" s="2" t="s">
-        <v>576</v>
-      </c>
-      <c r="C204" s="2" t="s">
-        <v>577</v>
       </c>
     </row>
     <row r="205" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="B205" s="2" t="s">
+        <v>577</v>
+      </c>
+      <c r="C205" s="2" t="s">
         <v>578</v>
-      </c>
-      <c r="B205" s="2" t="s">
-        <v>579</v>
-      </c>
-      <c r="C205" s="2" t="s">
-        <v>580</v>
       </c>
     </row>
     <row r="206" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="B206" s="2" t="s">
+        <v>580</v>
+      </c>
+      <c r="C206" s="2" t="s">
         <v>581</v>
-      </c>
-      <c r="B206" s="2" t="s">
-        <v>582</v>
-      </c>
-      <c r="C206" s="2" t="s">
-        <v>583</v>
       </c>
     </row>
     <row r="207" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="B207" s="2" t="s">
+        <v>583</v>
+      </c>
+      <c r="C207" s="2" t="s">
         <v>584</v>
-      </c>
-      <c r="B207" s="2" t="s">
-        <v>585</v>
-      </c>
-      <c r="C207" s="2" t="s">
-        <v>586</v>
       </c>
     </row>
     <row r="208" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="B208" s="2" t="s">
+        <v>586</v>
+      </c>
+      <c r="C208" s="2" t="s">
         <v>587</v>
-      </c>
-      <c r="B208" s="2" t="s">
-        <v>588</v>
-      </c>
-      <c r="C208" s="2" t="s">
-        <v>589</v>
       </c>
     </row>
     <row r="209" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="B209" s="2" t="s">
+        <v>589</v>
+      </c>
+      <c r="C209" s="2" t="s">
         <v>590</v>
-      </c>
-      <c r="B209" s="2" t="s">
-        <v>591</v>
-      </c>
-      <c r="C209" s="2" t="s">
-        <v>592</v>
       </c>
     </row>
     <row r="210" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>594</v>
+        <v>92</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
     </row>
     <row r="211" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
     </row>
     <row r="212" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
     </row>
     <row r="213" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="C213" s="2" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
     </row>
     <row r="214" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="C214" s="2" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
     </row>
     <row r="215" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A215" s="2" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="C215" s="2" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
     </row>
     <row r="216" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A216" s="2" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="C216" s="2" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
     </row>
     <row r="217" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A217" s="2" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="C217" s="2" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
     </row>
     <row r="218" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A218" s="2" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="C218" s="2" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
     </row>
     <row r="219" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="C219" s="2" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
     </row>
     <row r="220" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A220" s="2" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="C220" s="2" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
     </row>
     <row r="221" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A221" s="2" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="C221" s="2" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
     </row>
     <row r="222" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A222" s="2" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
       <c r="C222" s="2" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
     </row>
     <row r="223" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A223" s="2" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="C223" s="2" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
     </row>
     <row r="224" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A224" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="B224" s="2" t="s">
+        <v>633</v>
+      </c>
+      <c r="C224" s="2" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="225" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A225" s="2" t="s">
         <v>635</v>
       </c>
-      <c r="B224" s="2" t="s">
+      <c r="B225" s="2" t="s">
         <v>636</v>
       </c>
-      <c r="C224" s="2" t="s">
-        <v>538</v>
+      <c r="C225" s="2" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="226" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A226" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="B226" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="C226" s="2" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="227" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A227" s="2" t="s">
+        <v>641</v>
+      </c>
+      <c r="B227" s="2" t="s">
+        <v>642</v>
+      </c>
+      <c r="C227" s="2" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="228" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A228" s="2" t="s">
+        <v>644</v>
+      </c>
+      <c r="B228" s="2" t="s">
+        <v>645</v>
+      </c>
+      <c r="C228" s="2" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="229" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A229" s="2" t="s">
+        <v>647</v>
+      </c>
+      <c r="B229" s="2" t="s">
+        <v>648</v>
+      </c>
+      <c r="C229" s="2" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="230" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A230" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="B230" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="C230" s="2" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="231" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A231" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="B231" s="2" t="s">
+        <v>654</v>
+      </c>
+      <c r="C231" s="2" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="232" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A232" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="B232" s="2" t="s">
+        <v>657</v>
+      </c>
+      <c r="C232" s="2" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="233" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A233" s="2" t="s">
+        <v>659</v>
+      </c>
+      <c r="B233" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="C233" s="2" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="234" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A234" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="B234" s="2" t="s">
+        <v>663</v>
+      </c>
+      <c r="C234" s="2" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="235" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A235" s="2" t="s">
+        <v>665</v>
+      </c>
+      <c r="B235" s="2" t="s">
+        <v>666</v>
+      </c>
+      <c r="C235" s="2" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="236" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A236" s="2" t="s">
+        <v>668</v>
+      </c>
+      <c r="B236" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="C236" s="2" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="237" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A237" s="2" t="s">
+        <v>671</v>
+      </c>
+      <c r="B237" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="C237" s="2" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="238" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A238" s="2" t="s">
+        <v>674</v>
+      </c>
+      <c r="B238" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="C238" s="2" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="239" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A239" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="B239" s="2" t="s">
+        <v>678</v>
+      </c>
+      <c r="C239" s="2" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="240" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A240" s="2" t="s">
+        <v>680</v>
+      </c>
+      <c r="B240" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="C240" s="2" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="241" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A241" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="B241" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="C241" s="2" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="242" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A242" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="B242" s="2" t="s">
+        <v>687</v>
+      </c>
+      <c r="C242" s="2" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="243" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A243" s="2" t="s">
+        <v>689</v>
+      </c>
+      <c r="B243" s="2" t="s">
+        <v>690</v>
+      </c>
+      <c r="C243" s="2" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="244" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A244" s="2" t="s">
+        <v>692</v>
+      </c>
+      <c r="B244" s="2" t="s">
+        <v>693</v>
+      </c>
+      <c r="C244" s="2" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="245" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A245" s="2" t="s">
+        <v>695</v>
+      </c>
+      <c r="B245" s="2" t="s">
+        <v>696</v>
+      </c>
+      <c r="C245" s="2" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="246" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A246" s="2" t="s">
+        <v>698</v>
+      </c>
+      <c r="B246" s="2" t="s">
+        <v>699</v>
+      </c>
+      <c r="C246" s="2" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="247" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A247" s="2" t="s">
+        <v>701</v>
+      </c>
+      <c r="B247" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="C247" s="2" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="248" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A248" s="2" t="s">
+        <v>704</v>
+      </c>
+      <c r="B248" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="C248" s="2" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="249" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A249" s="2" t="s">
+        <v>707</v>
+      </c>
+      <c r="B249" s="2" t="s">
+        <v>708</v>
+      </c>
+      <c r="C249" s="2" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="250" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A250" s="2" t="s">
+        <v>710</v>
+      </c>
+      <c r="B250" s="2" t="s">
+        <v>711</v>
+      </c>
+      <c r="C250" s="2" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="251" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A251" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B251" s="2" t="s">
+        <v>714</v>
+      </c>
+      <c r="C251" s="2" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="252" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A252" s="2" t="s">
+        <v>716</v>
+      </c>
+      <c r="B252" s="2" t="s">
+        <v>717</v>
+      </c>
+      <c r="C252" s="2" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="253" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A253" s="2" t="s">
+        <v>719</v>
+      </c>
+      <c r="B253" s="2" t="s">
+        <v>720</v>
+      </c>
+      <c r="C253" s="2" t="s">
+        <v>721</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(portal-web): landing 視覺強化——參考 Begonia Design 的張力手法
- 全頁紙質顆粒（SVG feTurbulence）+ 五欄貫穿細格線
- 各區巨型 outline 出血字（OPEN JAM / MUSIC / PHOTO / E-BOOK /
  WORKFLOW / DISCOVER / BELIEVE / JAM ON!）隨捲動水平飄移
- story 三章改整屏飽和色反白（深紫 / 桃紅 / 深青）
- workflow 改深色滿版 band、why 改滿版黃 band
- story 與 workflow 間新增斜角品牌跑馬燈帶（landing.marquee i18n）
- hero / CTA 標題字級加大

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/portal-web/i18n.xlsx
+++ b/apps/portal-web/i18n.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="722">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="734">
   <si>
     <t>key</t>
   </si>
@@ -2177,6 +2177,42 @@
   </si>
   <si>
     <t>Explore creators</t>
+  </si>
+  <si>
+    <t>landing.marquee.0</t>
+  </si>
+  <si>
+    <t>Collect</t>
+  </si>
+  <si>
+    <t>landing.marquee.1</t>
+  </si>
+  <si>
+    <t>Support</t>
+  </si>
+  <si>
+    <t>landing.marquee.2</t>
+  </si>
+  <si>
+    <t>Remember</t>
+  </si>
+  <si>
+    <t>landing.marquee.3</t>
+  </si>
+  <si>
+    <t>把作品交到對的人手上</t>
+  </si>
+  <si>
+    <t>Work finds its people</t>
+  </si>
+  <si>
+    <t>landing.marquee.4</t>
+  </si>
+  <si>
+    <t>你的小店，開在自己的網址上</t>
+  </si>
+  <si>
+    <t>A shop at your own address</t>
   </si>
 </sst>
 </file>
@@ -2562,7 +2598,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C253"/>
+  <dimension ref="A1:C258"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -5352,6 +5388,61 @@
         <v>721</v>
       </c>
     </row>
+    <row r="254" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A254" s="2" t="s">
+        <v>722</v>
+      </c>
+      <c r="B254" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C254" s="2" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="255" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A255" s="2" t="s">
+        <v>724</v>
+      </c>
+      <c r="B255" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="C255" s="2" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="256" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A256" s="2" t="s">
+        <v>726</v>
+      </c>
+      <c r="B256" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="C256" s="2" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="257" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A257" s="2" t="s">
+        <v>728</v>
+      </c>
+      <c r="B257" s="2" t="s">
+        <v>729</v>
+      </c>
+      <c r="C257" s="2" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="258" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A258" s="2" t="s">
+        <v>731</v>
+      </c>
+      <c r="B258" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="C258" s="2" t="s">
+        <v>733</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
refactor(portal-web): 法律頁改版為 hero 色帶 + 重點速覽 + sticky 目錄
版面結構重排：Hero 漸層色帶（版本 meta pill 取 ContentService
啟用版本）、資料夾式頁籤 + 內容卡（重點速覽摘要卡片格、sticky
章節目錄、編號章節與色塊列點）、聯絡 CTA（前往常見問題）。
樣式沿用既有視覺 token；移除 GSAP 大字視差與顆粒/格線氛圍層。
i18n 新增 legal.heroTitleMark / tldrLabel / tocLabel / cta 與
兩份文件各三張 tldr 摘要卡。
FAQ 頁一併調整：列表區塊加寬至 1080 與 CTA 對齊、CTA 按鈕統一
白色款。

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/portal-web/i18n.xlsx
+++ b/apps/portal-web/i18n.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="994">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1131" uniqueCount="1049">
   <si>
     <t>key</t>
   </si>
@@ -982,10 +982,10 @@
     <t>legal.heroTitle</t>
   </si>
   <si>
-    <t>Open Jam 背後的規範與承諾。</t>
-  </si>
-  <si>
-    <t>The rules and promises behind Open Jam.</t>
+    <t>Open Jam 背後的{mark}與承諾</t>
+  </si>
+  <si>
+    <t>The {mark} and promises behind Open Jam</t>
   </si>
   <si>
     <t>legal.lede</t>
@@ -1000,6 +1000,60 @@
     <t>legal.terms.title</t>
   </si>
   <si>
+    <t>legal.terms.tldr.0.t</t>
+  </si>
+  <si>
+    <t>作品永遠是你的</t>
+  </si>
+  <si>
+    <t>Your work stays yours</t>
+  </si>
+  <si>
+    <t>legal.terms.tldr.0.d</t>
+  </si>
+  <si>
+    <t>上架不轉移著作權，你只授權平台展示與銷售你的作品。</t>
+  </si>
+  <si>
+    <t>Listing never transfers copyright — you only license us to display and sell it.</t>
+  </si>
+  <si>
+    <t>legal.terms.tldr.1.t</t>
+  </si>
+  <si>
+    <t>免月費、只抽 3%</t>
+  </si>
+  <si>
+    <t>No monthly fee, 3% cut</t>
+  </si>
+  <si>
+    <t>legal.terms.tldr.1.d</t>
+  </si>
+  <si>
+    <t>開店與上架不收費，作品售出時平台收取 3% 手續費。</t>
+  </si>
+  <si>
+    <t>Opening a shop and listing are free; we take a 3% fee only when a work sells.</t>
+  </si>
+  <si>
+    <t>legal.terms.tldr.2.t</t>
+  </si>
+  <si>
+    <t>內容須原創或已授權</t>
+  </si>
+  <si>
+    <t>Original or licensed only</t>
+  </si>
+  <si>
+    <t>legal.terms.tldr.2.d</t>
+  </si>
+  <si>
+    <t>嚴禁上架侵權內容，違反條款可能被暫停或終止帳號。</t>
+  </si>
+  <si>
+    <t>Infringing content is strictly prohibited; violations can suspend or end your account.</t>
+  </si>
+  <si>
     <t>legal.terms.sections.0.h</t>
   </si>
   <si>
@@ -1141,6 +1195,60 @@
     <t>隱私政策</t>
   </si>
   <si>
+    <t>legal.privacy.tldr.0.t</t>
+  </si>
+  <si>
+    <t>只蒐集必要資料</t>
+  </si>
+  <si>
+    <t>Only what's needed</t>
+  </si>
+  <si>
+    <t>legal.privacy.tldr.0.d</t>
+  </si>
+  <si>
+    <t>Email、訂單與使用紀錄，用於營運平台、處理交易與客戶支援。</t>
+  </si>
+  <si>
+    <t>Email, orders, and usage records — used to run the platform, process transactions, and support you.</t>
+  </si>
+  <si>
+    <t>legal.privacy.tldr.1.t</t>
+  </si>
+  <si>
+    <t>不碰你的卡號</t>
+  </si>
+  <si>
+    <t>We never see your card</t>
+  </si>
+  <si>
+    <t>legal.privacy.tldr.1.d</t>
+  </si>
+  <si>
+    <t>金流全程由 Stripe 處理，我們不接觸也不儲存信用卡資料。</t>
+  </si>
+  <si>
+    <t>Payments are handled entirely by Stripe; we never touch or store card data.</t>
+  </si>
+  <si>
+    <t>legal.privacy.tldr.2.t</t>
+  </si>
+  <si>
+    <t>資料由你作主</t>
+  </si>
+  <si>
+    <t>Your data, your call</t>
+  </si>
+  <si>
+    <t>legal.privacy.tldr.2.d</t>
+  </si>
+  <si>
+    <t>你可以隨時查詢、更正或刪除個人資料，也能取消行銷通知。</t>
+  </si>
+  <si>
+    <t>Access, correct, or delete your personal data any time, and opt out of marketing.</t>
+  </si>
+  <si>
     <t>legal.privacy.sections.0.h</t>
   </si>
   <si>
@@ -1276,6 +1384,69 @@
     <t>You have the right to access, correct, or delete your personal data, and you may unsubscribe from marketing notices at any time. You can handle these requests via the settings page or by contacting support.</t>
   </si>
   <si>
+    <t>legal.heroTitleMark</t>
+  </si>
+  <si>
+    <t>規範</t>
+  </si>
+  <si>
+    <t>rules</t>
+  </si>
+  <si>
+    <t>legal.tldrLabel</t>
+  </si>
+  <si>
+    <t>重點速覽 — 30 秒看完</t>
+  </si>
+  <si>
+    <t>The gist — a 30-second read</t>
+  </si>
+  <si>
+    <t>legal.tocLabel</t>
+  </si>
+  <si>
+    <t>目錄</t>
+  </si>
+  <si>
+    <t>Contents</t>
+  </si>
+  <si>
+    <t>legal.cta.title</t>
+  </si>
+  <si>
+    <t>對條款或隱私有疑問？</t>
+  </si>
+  <si>
+    <t>Questions about our terms or privacy?</t>
+  </si>
+  <si>
+    <t>legal.cta.text</t>
+  </si>
+  <si>
+    <t>寫信給我們，或先到常見問題找找，多數疑問都有現成答案。</t>
+  </si>
+  <si>
+    <t>Email us, or check the FAQ first — most questions already have answers there.</t>
+  </si>
+  <si>
+    <t>legal.cta.contact</t>
+  </si>
+  <si>
+    <t>聯絡我們</t>
+  </si>
+  <si>
+    <t>Contact us</t>
+  </si>
+  <si>
+    <t>legal.cta.faq</t>
+  </si>
+  <si>
+    <t>前往常見問題</t>
+  </si>
+  <si>
+    <t>Browse the FAQ</t>
+  </si>
+  <si>
     <t>onboarding.modalAria</t>
   </si>
   <si>
@@ -2483,12 +2654,6 @@
   </si>
   <si>
     <t>faq.cta.contact</t>
-  </si>
-  <si>
-    <t>聯絡我們</t>
-  </si>
-  <si>
-    <t>Contact us</t>
   </si>
   <si>
     <t>faq.cta.github</t>
@@ -3378,7 +3543,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C358"/>
+  <dimension ref="A1:C377"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -4834,73 +4999,73 @@
         <v>375</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>42</v>
+        <v>376</v>
       </c>
     </row>
     <row r="133" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="134" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="135" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="136" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="137" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="138" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>393</v>
+        <v>42</v>
       </c>
     </row>
     <row r="139" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5032,359 +5197,359 @@
         <v>428</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
     <row r="151" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>277</v>
+        <v>431</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>278</v>
+        <v>432</v>
       </c>
     </row>
     <row r="152" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
     </row>
     <row r="153" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
     </row>
     <row r="154" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="155" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
     </row>
     <row r="156" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
     </row>
     <row r="157" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
     </row>
     <row r="158" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
     </row>
     <row r="159" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
     </row>
     <row r="160" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
     </row>
     <row r="161" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>17</v>
+        <v>461</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>18</v>
+        <v>462</v>
       </c>
     </row>
     <row r="162" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>457</v>
+        <v>463</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>458</v>
+        <v>464</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
     </row>
     <row r="163" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>20</v>
+        <v>467</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>21</v>
+        <v>468</v>
       </c>
     </row>
     <row r="164" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
-        <v>461</v>
+        <v>469</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>462</v>
+        <v>470</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>463</v>
+        <v>471</v>
       </c>
     </row>
     <row r="165" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
-        <v>464</v>
+        <v>472</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>465</v>
+        <v>473</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>466</v>
+        <v>474</v>
       </c>
     </row>
     <row r="166" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
-        <v>467</v>
+        <v>475</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>468</v>
+        <v>476</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>469</v>
+        <v>477</v>
       </c>
     </row>
     <row r="167" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>470</v>
+        <v>478</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>471</v>
+        <v>479</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>472</v>
+        <v>480</v>
       </c>
     </row>
     <row r="168" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>473</v>
+        <v>481</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>474</v>
+        <v>482</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>475</v>
+        <v>483</v>
       </c>
     </row>
     <row r="169" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>476</v>
+        <v>484</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>478</v>
+        <v>485</v>
       </c>
     </row>
     <row r="170" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
-        <v>479</v>
+        <v>486</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>480</v>
+        <v>277</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>481</v>
+        <v>278</v>
       </c>
     </row>
     <row r="171" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
-        <v>482</v>
+        <v>487</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>484</v>
+        <v>489</v>
       </c>
     </row>
     <row r="172" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>486</v>
+        <v>491</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
     </row>
     <row r="173" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
     </row>
     <row r="174" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
-        <v>491</v>
+        <v>496</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>493</v>
+        <v>498</v>
       </c>
     </row>
     <row r="175" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
     </row>
     <row r="176" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
     </row>
     <row r="177" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
     </row>
     <row r="178" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
     </row>
     <row r="179" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
     </row>
     <row r="180" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>510</v>
+        <v>17</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>511</v>
+        <v>18</v>
       </c>
     </row>
     <row r="181" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="182" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>516</v>
+        <v>20</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>517</v>
+        <v>21</v>
       </c>
     </row>
     <row r="183" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5425,502 +5590,502 @@
         <v>527</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>71</v>
+        <v>528</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>72</v>
+        <v>529</v>
       </c>
     </row>
     <row r="187" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row r="188" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>77</v>
+        <v>534</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
     </row>
     <row r="189" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
     </row>
     <row r="190" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
     </row>
     <row r="191" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
     </row>
     <row r="192" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
     </row>
     <row r="193" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="194" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
     </row>
     <row r="195" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
     </row>
     <row r="196" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
     </row>
     <row r="197" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
     </row>
     <row r="198" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
     </row>
     <row r="199" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
     </row>
     <row r="200" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
     </row>
     <row r="201" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
     </row>
     <row r="202" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
     </row>
     <row r="203" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
     </row>
     <row r="204" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
     </row>
     <row r="205" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>582</v>
+        <v>71</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
     </row>
     <row r="206" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="C206" s="2" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="207" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>587</v>
+        <v>77</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
     </row>
     <row r="208" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="C208" s="2" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
     </row>
     <row r="209" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="C209" s="2" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
     </row>
     <row r="210" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
     </row>
     <row r="211" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
     </row>
     <row r="212" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>89</v>
+        <v>603</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
     </row>
     <row r="213" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="C213" s="2" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
     </row>
     <row r="214" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="C214" s="2" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
     </row>
     <row r="215" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A215" s="2" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="C215" s="2" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
     </row>
     <row r="216" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A216" s="2" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="C216" s="2" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
     </row>
     <row r="217" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A217" s="2" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="C217" s="2" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
     </row>
     <row r="218" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A218" s="2" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="C218" s="2" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
     </row>
     <row r="219" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="C219" s="2" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
     </row>
     <row r="220" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A220" s="2" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="C220" s="2" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
     </row>
     <row r="221" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A221" s="2" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="C221" s="2" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
     </row>
     <row r="222" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A222" s="2" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="C222" s="2" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
     </row>
     <row r="223" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A223" s="2" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="C223" s="2" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
     </row>
     <row r="224" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A224" s="2" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="C224" s="2" t="s">
-        <v>638</v>
+        <v>57</v>
       </c>
     </row>
     <row r="225" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A225" s="2" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="C225" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
     </row>
     <row r="226" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A226" s="2" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="C226" s="2" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
     </row>
     <row r="227" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A227" s="2" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="C227" s="2" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
     </row>
     <row r="228" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A228" s="2" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="C228" s="2" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
     </row>
     <row r="229" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A229" s="2" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="B229" s="2" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="C229" s="2" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
     </row>
     <row r="230" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A230" s="2" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="B230" s="2" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C230" s="2" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
     </row>
     <row r="231" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A231" s="2" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B231" s="2" t="s">
-        <v>658</v>
+        <v>89</v>
       </c>
       <c r="C231" s="2" t="s">
         <v>659</v>
@@ -6195,274 +6360,274 @@
         <v>732</v>
       </c>
       <c r="B256" s="2" t="s">
-        <v>77</v>
+        <v>733</v>
       </c>
       <c r="C256" s="2" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
     </row>
     <row r="257" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A257" s="2" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>534</v>
+        <v>736</v>
       </c>
       <c r="C257" s="2" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
     </row>
     <row r="258" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A258" s="2" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>537</v>
+        <v>739</v>
       </c>
       <c r="C258" s="2" t="s">
-        <v>737</v>
+        <v>740</v>
       </c>
     </row>
     <row r="259" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A259" s="2" t="s">
-        <v>738</v>
+        <v>741</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>739</v>
+        <v>742</v>
       </c>
       <c r="C259" s="2" t="s">
-        <v>740</v>
+        <v>743</v>
       </c>
     </row>
     <row r="260" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A260" s="2" t="s">
-        <v>741</v>
+        <v>744</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>742</v>
+        <v>745</v>
       </c>
       <c r="C260" s="2" t="s">
-        <v>743</v>
+        <v>746</v>
       </c>
     </row>
     <row r="261" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A261" s="2" t="s">
-        <v>744</v>
+        <v>747</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>50</v>
+        <v>748</v>
       </c>
       <c r="C261" s="2" t="s">
-        <v>51</v>
+        <v>749</v>
       </c>
     </row>
     <row r="262" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A262" s="2" t="s">
-        <v>745</v>
+        <v>750</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>746</v>
+        <v>751</v>
       </c>
       <c r="C262" s="2" t="s">
-        <v>747</v>
+        <v>752</v>
       </c>
     </row>
     <row r="263" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A263" s="2" t="s">
-        <v>748</v>
+        <v>753</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>749</v>
+        <v>754</v>
       </c>
       <c r="C263" s="2" t="s">
-        <v>750</v>
+        <v>755</v>
       </c>
     </row>
     <row r="264" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A264" s="2" t="s">
-        <v>751</v>
+        <v>756</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>752</v>
+        <v>757</v>
       </c>
       <c r="C264" s="2" t="s">
-        <v>753</v>
+        <v>758</v>
       </c>
     </row>
     <row r="265" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A265" s="2" t="s">
-        <v>754</v>
+        <v>759</v>
       </c>
       <c r="B265" s="2" t="s">
-        <v>755</v>
+        <v>760</v>
       </c>
       <c r="C265" s="2" t="s">
-        <v>756</v>
+        <v>761</v>
       </c>
     </row>
     <row r="266" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A266" s="2" t="s">
-        <v>757</v>
+        <v>762</v>
       </c>
       <c r="B266" s="2" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="C266" s="2" t="s">
-        <v>759</v>
+        <v>764</v>
       </c>
     </row>
     <row r="267" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A267" s="2" t="s">
-        <v>760</v>
+        <v>765</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>761</v>
+        <v>766</v>
       </c>
       <c r="C267" s="2" t="s">
-        <v>762</v>
+        <v>767</v>
       </c>
     </row>
     <row r="268" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A268" s="2" t="s">
-        <v>763</v>
+        <v>768</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="C268" s="2" t="s">
-        <v>765</v>
+        <v>770</v>
       </c>
     </row>
     <row r="269" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A269" s="2" t="s">
-        <v>766</v>
+        <v>771</v>
       </c>
       <c r="B269" s="2" t="s">
-        <v>767</v>
+        <v>772</v>
       </c>
       <c r="C269" s="2" t="s">
-        <v>768</v>
+        <v>773</v>
       </c>
     </row>
     <row r="270" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A270" s="2" t="s">
-        <v>769</v>
+        <v>774</v>
       </c>
       <c r="B270" s="2" t="s">
-        <v>770</v>
+        <v>775</v>
       </c>
       <c r="C270" s="2" t="s">
-        <v>771</v>
+        <v>776</v>
       </c>
     </row>
     <row r="271" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A271" s="2" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>773</v>
+        <v>778</v>
       </c>
       <c r="C271" s="2" t="s">
-        <v>774</v>
+        <v>779</v>
       </c>
     </row>
     <row r="272" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A272" s="2" t="s">
-        <v>775</v>
+        <v>780</v>
       </c>
       <c r="B272" s="2" t="s">
-        <v>776</v>
+        <v>781</v>
       </c>
       <c r="C272" s="2" t="s">
-        <v>777</v>
+        <v>782</v>
       </c>
     </row>
     <row r="273" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A273" s="2" t="s">
-        <v>778</v>
+        <v>783</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>779</v>
+        <v>784</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>780</v>
+        <v>785</v>
       </c>
     </row>
     <row r="274" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A274" s="2" t="s">
-        <v>781</v>
+        <v>786</v>
       </c>
       <c r="B274" s="2" t="s">
-        <v>782</v>
+        <v>787</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>783</v>
+        <v>788</v>
       </c>
     </row>
     <row r="275" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A275" s="2" t="s">
-        <v>784</v>
+        <v>789</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>785</v>
+        <v>77</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
     </row>
     <row r="276" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A276" s="2" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
       <c r="B276" s="2" t="s">
-        <v>788</v>
+        <v>591</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>789</v>
+        <v>792</v>
       </c>
     </row>
     <row r="277" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A277" s="2" t="s">
-        <v>790</v>
+        <v>793</v>
       </c>
       <c r="B277" s="2" t="s">
-        <v>791</v>
+        <v>594</v>
       </c>
       <c r="C277" s="2" t="s">
-        <v>792</v>
+        <v>794</v>
       </c>
     </row>
     <row r="278" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A278" s="2" t="s">
-        <v>793</v>
+        <v>795</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>794</v>
+        <v>796</v>
       </c>
       <c r="C278" s="2" t="s">
-        <v>795</v>
+        <v>797</v>
       </c>
     </row>
     <row r="279" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A279" s="2" t="s">
-        <v>796</v>
+        <v>798</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>797</v>
+        <v>799</v>
       </c>
       <c r="C279" s="2" t="s">
-        <v>798</v>
+        <v>800</v>
       </c>
     </row>
     <row r="280" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A280" s="2" t="s">
-        <v>799</v>
+        <v>801</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>800</v>
+        <v>50</v>
       </c>
       <c r="C280" s="2" t="s">
-        <v>801</v>
+        <v>51</v>
       </c>
     </row>
     <row r="281" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6572,755 +6737,964 @@
         <v>830</v>
       </c>
       <c r="C290" s="2" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
     </row>
     <row r="291" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A291" s="2" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="B291" s="2" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="C291" s="2" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
     </row>
     <row r="292" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A292" s="2" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="B292" s="2" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
     </row>
     <row r="293" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A293" s="2" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="B293" s="2" t="s">
-        <v>830</v>
+        <v>839</v>
       </c>
       <c r="C293" s="2" t="s">
-        <v>830</v>
+        <v>840</v>
       </c>
     </row>
     <row r="294" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A294" s="2" t="s">
-        <v>838</v>
+        <v>841</v>
       </c>
       <c r="B294" s="2" t="s">
-        <v>839</v>
+        <v>842</v>
       </c>
       <c r="C294" s="2" t="s">
-        <v>840</v>
+        <v>843</v>
       </c>
     </row>
     <row r="295" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A295" s="2" t="s">
-        <v>841</v>
+        <v>844</v>
       </c>
       <c r="B295" s="2" t="s">
-        <v>842</v>
+        <v>845</v>
       </c>
       <c r="C295" s="2" t="s">
-        <v>843</v>
+        <v>846</v>
       </c>
     </row>
     <row r="296" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A296" s="2" t="s">
-        <v>844</v>
+        <v>847</v>
       </c>
       <c r="B296" s="2" t="s">
-        <v>830</v>
+        <v>848</v>
       </c>
       <c r="C296" s="2" t="s">
-        <v>830</v>
+        <v>849</v>
       </c>
     </row>
     <row r="297" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A297" s="2" t="s">
-        <v>845</v>
+        <v>850</v>
       </c>
       <c r="B297" s="2" t="s">
-        <v>846</v>
+        <v>851</v>
       </c>
       <c r="C297" s="2" t="s">
-        <v>847</v>
+        <v>852</v>
       </c>
     </row>
     <row r="298" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A298" s="2" t="s">
-        <v>848</v>
+        <v>853</v>
       </c>
       <c r="B298" s="2" t="s">
-        <v>849</v>
+        <v>854</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>850</v>
+        <v>855</v>
       </c>
     </row>
     <row r="299" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A299" s="2" t="s">
-        <v>851</v>
+        <v>856</v>
       </c>
       <c r="B299" s="2" t="s">
-        <v>830</v>
+        <v>857</v>
       </c>
       <c r="C299" s="2" t="s">
-        <v>830</v>
+        <v>858</v>
       </c>
     </row>
     <row r="300" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A300" s="2" t="s">
-        <v>852</v>
+        <v>859</v>
       </c>
       <c r="B300" s="2" t="s">
-        <v>853</v>
+        <v>860</v>
       </c>
       <c r="C300" s="2" t="s">
-        <v>854</v>
+        <v>861</v>
       </c>
     </row>
     <row r="301" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A301" s="2" t="s">
-        <v>855</v>
+        <v>862</v>
       </c>
       <c r="B301" s="2" t="s">
-        <v>856</v>
+        <v>863</v>
       </c>
       <c r="C301" s="2" t="s">
-        <v>857</v>
+        <v>864</v>
       </c>
     </row>
     <row r="302" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A302" s="2" t="s">
-        <v>858</v>
+        <v>865</v>
       </c>
       <c r="B302" s="2" t="s">
-        <v>830</v>
+        <v>866</v>
       </c>
       <c r="C302" s="2" t="s">
-        <v>830</v>
+        <v>867</v>
       </c>
     </row>
     <row r="303" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A303" s="2" t="s">
-        <v>859</v>
+        <v>868</v>
       </c>
       <c r="B303" s="2" t="s">
-        <v>860</v>
+        <v>869</v>
       </c>
       <c r="C303" s="2" t="s">
-        <v>861</v>
+        <v>870</v>
       </c>
     </row>
     <row r="304" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A304" s="2" t="s">
-        <v>862</v>
+        <v>871</v>
       </c>
       <c r="B304" s="2" t="s">
-        <v>863</v>
+        <v>872</v>
       </c>
       <c r="C304" s="2" t="s">
-        <v>864</v>
+        <v>873</v>
       </c>
     </row>
     <row r="305" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A305" s="2" t="s">
-        <v>865</v>
+        <v>874</v>
       </c>
       <c r="B305" s="2" t="s">
-        <v>866</v>
+        <v>875</v>
       </c>
       <c r="C305" s="2" t="s">
-        <v>866</v>
+        <v>876</v>
       </c>
     </row>
     <row r="306" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A306" s="2" t="s">
-        <v>867</v>
+        <v>877</v>
       </c>
       <c r="B306" s="2" t="s">
-        <v>868</v>
+        <v>878</v>
       </c>
       <c r="C306" s="2" t="s">
-        <v>869</v>
+        <v>879</v>
       </c>
     </row>
     <row r="307" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A307" s="2" t="s">
-        <v>870</v>
+        <v>880</v>
       </c>
       <c r="B307" s="2" t="s">
-        <v>871</v>
+        <v>473</v>
       </c>
       <c r="C307" s="2" t="s">
-        <v>872</v>
+        <v>474</v>
       </c>
     </row>
     <row r="308" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A308" s="2" t="s">
-        <v>873</v>
+        <v>881</v>
       </c>
       <c r="B308" s="2" t="s">
-        <v>866</v>
+        <v>882</v>
       </c>
       <c r="C308" s="2" t="s">
-        <v>866</v>
+        <v>883</v>
       </c>
     </row>
     <row r="309" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A309" s="2" t="s">
-        <v>874</v>
+        <v>884</v>
       </c>
       <c r="B309" s="2" t="s">
-        <v>875</v>
+        <v>885</v>
       </c>
       <c r="C309" s="2" t="s">
-        <v>876</v>
+        <v>885</v>
       </c>
     </row>
     <row r="310" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A310" s="2" t="s">
-        <v>877</v>
+        <v>886</v>
       </c>
       <c r="B310" s="2" t="s">
-        <v>878</v>
+        <v>887</v>
       </c>
       <c r="C310" s="2" t="s">
-        <v>879</v>
+        <v>888</v>
       </c>
     </row>
     <row r="311" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A311" s="2" t="s">
-        <v>880</v>
+        <v>889</v>
       </c>
       <c r="B311" s="2" t="s">
-        <v>866</v>
+        <v>890</v>
       </c>
       <c r="C311" s="2" t="s">
-        <v>866</v>
+        <v>891</v>
       </c>
     </row>
     <row r="312" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A312" s="2" t="s">
-        <v>881</v>
+        <v>892</v>
       </c>
       <c r="B312" s="2" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="C312" s="2" t="s">
-        <v>883</v>
+        <v>885</v>
       </c>
     </row>
     <row r="313" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A313" s="2" t="s">
-        <v>884</v>
+        <v>893</v>
       </c>
       <c r="B313" s="2" t="s">
-        <v>885</v>
+        <v>894</v>
       </c>
       <c r="C313" s="2" t="s">
-        <v>886</v>
+        <v>895</v>
       </c>
     </row>
     <row r="314" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A314" s="2" t="s">
-        <v>887</v>
+        <v>896</v>
       </c>
       <c r="B314" s="2" t="s">
-        <v>866</v>
+        <v>897</v>
       </c>
       <c r="C314" s="2" t="s">
-        <v>866</v>
+        <v>898</v>
       </c>
     </row>
     <row r="315" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A315" s="2" t="s">
-        <v>888</v>
+        <v>899</v>
       </c>
       <c r="B315" s="2" t="s">
-        <v>889</v>
+        <v>885</v>
       </c>
       <c r="C315" s="2" t="s">
-        <v>890</v>
+        <v>885</v>
       </c>
     </row>
     <row r="316" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A316" s="2" t="s">
-        <v>891</v>
+        <v>900</v>
       </c>
       <c r="B316" s="2" t="s">
-        <v>892</v>
+        <v>901</v>
       </c>
       <c r="C316" s="2" t="s">
-        <v>893</v>
+        <v>902</v>
       </c>
     </row>
     <row r="317" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A317" s="2" t="s">
-        <v>894</v>
+        <v>903</v>
       </c>
       <c r="B317" s="2" t="s">
-        <v>866</v>
+        <v>904</v>
       </c>
       <c r="C317" s="2" t="s">
-        <v>866</v>
+        <v>905</v>
       </c>
     </row>
     <row r="318" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A318" s="2" t="s">
-        <v>895</v>
+        <v>906</v>
       </c>
       <c r="B318" s="2" t="s">
-        <v>896</v>
+        <v>885</v>
       </c>
       <c r="C318" s="2" t="s">
-        <v>897</v>
+        <v>885</v>
       </c>
     </row>
     <row r="319" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A319" s="2" t="s">
-        <v>898</v>
+        <v>907</v>
       </c>
       <c r="B319" s="2" t="s">
-        <v>899</v>
+        <v>908</v>
       </c>
       <c r="C319" s="2" t="s">
-        <v>900</v>
+        <v>909</v>
       </c>
     </row>
     <row r="320" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A320" s="2" t="s">
-        <v>901</v>
+        <v>910</v>
       </c>
       <c r="B320" s="2" t="s">
-        <v>866</v>
+        <v>911</v>
       </c>
       <c r="C320" s="2" t="s">
-        <v>866</v>
+        <v>912</v>
       </c>
     </row>
     <row r="321" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A321" s="2" t="s">
-        <v>902</v>
+        <v>913</v>
       </c>
       <c r="B321" s="2" t="s">
-        <v>903</v>
+        <v>885</v>
       </c>
       <c r="C321" s="2" t="s">
-        <v>904</v>
+        <v>885</v>
       </c>
     </row>
     <row r="322" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A322" s="2" t="s">
-        <v>905</v>
+        <v>914</v>
       </c>
       <c r="B322" s="2" t="s">
-        <v>906</v>
+        <v>915</v>
       </c>
       <c r="C322" s="2" t="s">
-        <v>907</v>
+        <v>916</v>
       </c>
     </row>
     <row r="323" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A323" s="2" t="s">
-        <v>908</v>
+        <v>917</v>
       </c>
       <c r="B323" s="2" t="s">
-        <v>866</v>
+        <v>918</v>
       </c>
       <c r="C323" s="2" t="s">
-        <v>866</v>
+        <v>919</v>
       </c>
     </row>
     <row r="324" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A324" s="2" t="s">
-        <v>909</v>
+        <v>920</v>
       </c>
       <c r="B324" s="2" t="s">
-        <v>910</v>
+        <v>921</v>
       </c>
       <c r="C324" s="2" t="s">
-        <v>911</v>
+        <v>921</v>
       </c>
     </row>
     <row r="325" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A325" s="2" t="s">
-        <v>912</v>
+        <v>922</v>
       </c>
       <c r="B325" s="2" t="s">
-        <v>913</v>
+        <v>923</v>
       </c>
       <c r="C325" s="2" t="s">
-        <v>914</v>
+        <v>924</v>
       </c>
     </row>
     <row r="326" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A326" s="2" t="s">
-        <v>915</v>
+        <v>925</v>
       </c>
       <c r="B326" s="2" t="s">
-        <v>916</v>
+        <v>926</v>
       </c>
       <c r="C326" s="2" t="s">
-        <v>916</v>
+        <v>927</v>
       </c>
     </row>
     <row r="327" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A327" s="2" t="s">
-        <v>917</v>
+        <v>928</v>
       </c>
       <c r="B327" s="2" t="s">
-        <v>918</v>
+        <v>921</v>
       </c>
       <c r="C327" s="2" t="s">
-        <v>919</v>
+        <v>921</v>
       </c>
     </row>
     <row r="328" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A328" s="2" t="s">
-        <v>920</v>
+        <v>929</v>
       </c>
       <c r="B328" s="2" t="s">
-        <v>921</v>
+        <v>930</v>
       </c>
       <c r="C328" s="2" t="s">
-        <v>922</v>
+        <v>931</v>
       </c>
     </row>
     <row r="329" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A329" s="2" t="s">
-        <v>923</v>
+        <v>932</v>
       </c>
       <c r="B329" s="2" t="s">
-        <v>916</v>
+        <v>933</v>
       </c>
       <c r="C329" s="2" t="s">
-        <v>916</v>
+        <v>934</v>
       </c>
     </row>
     <row r="330" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A330" s="2" t="s">
-        <v>924</v>
+        <v>935</v>
       </c>
       <c r="B330" s="2" t="s">
-        <v>925</v>
+        <v>921</v>
       </c>
       <c r="C330" s="2" t="s">
-        <v>926</v>
+        <v>921</v>
       </c>
     </row>
     <row r="331" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A331" s="2" t="s">
-        <v>927</v>
+        <v>936</v>
       </c>
       <c r="B331" s="2" t="s">
-        <v>928</v>
+        <v>937</v>
       </c>
       <c r="C331" s="2" t="s">
-        <v>929</v>
+        <v>938</v>
       </c>
     </row>
     <row r="332" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A332" s="2" t="s">
-        <v>930</v>
+        <v>939</v>
       </c>
       <c r="B332" s="2" t="s">
-        <v>916</v>
+        <v>940</v>
       </c>
       <c r="C332" s="2" t="s">
-        <v>916</v>
+        <v>941</v>
       </c>
     </row>
     <row r="333" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A333" s="2" t="s">
-        <v>931</v>
+        <v>942</v>
       </c>
       <c r="B333" s="2" t="s">
-        <v>932</v>
+        <v>921</v>
       </c>
       <c r="C333" s="2" t="s">
-        <v>933</v>
+        <v>921</v>
       </c>
     </row>
     <row r="334" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A334" s="2" t="s">
-        <v>934</v>
+        <v>943</v>
       </c>
       <c r="B334" s="2" t="s">
-        <v>935</v>
+        <v>944</v>
       </c>
       <c r="C334" s="2" t="s">
-        <v>936</v>
+        <v>945</v>
       </c>
     </row>
     <row r="335" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A335" s="2" t="s">
-        <v>937</v>
+        <v>946</v>
       </c>
       <c r="B335" s="2" t="s">
-        <v>916</v>
+        <v>947</v>
       </c>
       <c r="C335" s="2" t="s">
-        <v>916</v>
+        <v>948</v>
       </c>
     </row>
     <row r="336" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A336" s="2" t="s">
-        <v>938</v>
+        <v>949</v>
       </c>
       <c r="B336" s="2" t="s">
-        <v>939</v>
+        <v>921</v>
       </c>
       <c r="C336" s="2" t="s">
-        <v>940</v>
+        <v>921</v>
       </c>
     </row>
     <row r="337" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A337" s="2" t="s">
-        <v>941</v>
+        <v>950</v>
       </c>
       <c r="B337" s="2" t="s">
-        <v>942</v>
+        <v>951</v>
       </c>
       <c r="C337" s="2" t="s">
-        <v>943</v>
+        <v>952</v>
       </c>
     </row>
     <row r="338" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A338" s="2" t="s">
-        <v>944</v>
+        <v>953</v>
       </c>
       <c r="B338" s="2" t="s">
-        <v>916</v>
+        <v>954</v>
       </c>
       <c r="C338" s="2" t="s">
-        <v>916</v>
+        <v>955</v>
       </c>
     </row>
     <row r="339" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A339" s="2" t="s">
-        <v>945</v>
+        <v>956</v>
       </c>
       <c r="B339" s="2" t="s">
-        <v>946</v>
+        <v>921</v>
       </c>
       <c r="C339" s="2" t="s">
-        <v>947</v>
+        <v>921</v>
       </c>
     </row>
     <row r="340" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A340" s="2" t="s">
-        <v>948</v>
+        <v>957</v>
       </c>
       <c r="B340" s="2" t="s">
-        <v>949</v>
+        <v>958</v>
       </c>
       <c r="C340" s="2" t="s">
-        <v>950</v>
+        <v>959</v>
       </c>
     </row>
     <row r="341" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A341" s="2" t="s">
-        <v>951</v>
+        <v>960</v>
       </c>
       <c r="B341" s="2" t="s">
-        <v>916</v>
+        <v>961</v>
       </c>
       <c r="C341" s="2" t="s">
-        <v>916</v>
+        <v>962</v>
       </c>
     </row>
     <row r="342" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A342" s="2" t="s">
-        <v>952</v>
+        <v>963</v>
       </c>
       <c r="B342" s="2" t="s">
-        <v>953</v>
+        <v>921</v>
       </c>
       <c r="C342" s="2" t="s">
-        <v>954</v>
+        <v>921</v>
       </c>
     </row>
     <row r="343" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A343" s="2" t="s">
-        <v>955</v>
+        <v>964</v>
       </c>
       <c r="B343" s="2" t="s">
-        <v>956</v>
+        <v>965</v>
       </c>
       <c r="C343" s="2" t="s">
-        <v>957</v>
+        <v>966</v>
       </c>
     </row>
     <row r="344" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A344" s="2" t="s">
-        <v>958</v>
+        <v>967</v>
       </c>
       <c r="B344" s="2" t="s">
-        <v>959</v>
+        <v>968</v>
       </c>
       <c r="C344" s="2" t="s">
-        <v>959</v>
+        <v>969</v>
       </c>
     </row>
     <row r="345" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A345" s="2" t="s">
-        <v>960</v>
+        <v>970</v>
       </c>
       <c r="B345" s="2" t="s">
-        <v>961</v>
+        <v>971</v>
       </c>
       <c r="C345" s="2" t="s">
-        <v>962</v>
+        <v>971</v>
       </c>
     </row>
     <row r="346" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A346" s="2" t="s">
-        <v>963</v>
+        <v>972</v>
       </c>
       <c r="B346" s="2" t="s">
-        <v>964</v>
+        <v>973</v>
       </c>
       <c r="C346" s="2" t="s">
-        <v>965</v>
+        <v>974</v>
       </c>
     </row>
     <row r="347" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A347" s="2" t="s">
-        <v>966</v>
+        <v>975</v>
       </c>
       <c r="B347" s="2" t="s">
-        <v>959</v>
+        <v>976</v>
       </c>
       <c r="C347" s="2" t="s">
-        <v>959</v>
+        <v>977</v>
       </c>
     </row>
     <row r="348" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A348" s="2" t="s">
-        <v>967</v>
+        <v>978</v>
       </c>
       <c r="B348" s="2" t="s">
-        <v>968</v>
+        <v>971</v>
       </c>
       <c r="C348" s="2" t="s">
-        <v>969</v>
+        <v>971</v>
       </c>
     </row>
     <row r="349" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A349" s="2" t="s">
-        <v>970</v>
+        <v>979</v>
       </c>
       <c r="B349" s="2" t="s">
-        <v>971</v>
+        <v>980</v>
       </c>
       <c r="C349" s="2" t="s">
-        <v>972</v>
+        <v>981</v>
       </c>
     </row>
     <row r="350" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A350" s="2" t="s">
-        <v>973</v>
+        <v>982</v>
       </c>
       <c r="B350" s="2" t="s">
-        <v>959</v>
+        <v>983</v>
       </c>
       <c r="C350" s="2" t="s">
-        <v>959</v>
+        <v>984</v>
       </c>
     </row>
     <row r="351" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A351" s="2" t="s">
-        <v>974</v>
+        <v>985</v>
       </c>
       <c r="B351" s="2" t="s">
-        <v>975</v>
+        <v>971</v>
       </c>
       <c r="C351" s="2" t="s">
-        <v>976</v>
+        <v>971</v>
       </c>
     </row>
     <row r="352" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A352" s="2" t="s">
-        <v>977</v>
+        <v>986</v>
       </c>
       <c r="B352" s="2" t="s">
-        <v>978</v>
+        <v>987</v>
       </c>
       <c r="C352" s="2" t="s">
-        <v>979</v>
+        <v>988</v>
       </c>
     </row>
     <row r="353" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A353" s="2" t="s">
-        <v>980</v>
+        <v>989</v>
       </c>
       <c r="B353" s="2" t="s">
-        <v>959</v>
+        <v>990</v>
       </c>
       <c r="C353" s="2" t="s">
-        <v>959</v>
+        <v>991</v>
       </c>
     </row>
     <row r="354" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A354" s="2" t="s">
-        <v>981</v>
+        <v>992</v>
       </c>
       <c r="B354" s="2" t="s">
-        <v>982</v>
+        <v>971</v>
       </c>
       <c r="C354" s="2" t="s">
-        <v>983</v>
+        <v>971</v>
       </c>
     </row>
     <row r="355" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A355" s="2" t="s">
-        <v>984</v>
+        <v>993</v>
       </c>
       <c r="B355" s="2" t="s">
-        <v>985</v>
+        <v>994</v>
       </c>
       <c r="C355" s="2" t="s">
-        <v>986</v>
+        <v>995</v>
       </c>
     </row>
     <row r="356" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A356" s="2" t="s">
-        <v>987</v>
+        <v>996</v>
       </c>
       <c r="B356" s="2" t="s">
-        <v>959</v>
+        <v>997</v>
       </c>
       <c r="C356" s="2" t="s">
-        <v>959</v>
+        <v>998</v>
       </c>
     </row>
     <row r="357" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A357" s="2" t="s">
-        <v>988</v>
+        <v>999</v>
       </c>
       <c r="B357" s="2" t="s">
-        <v>989</v>
+        <v>971</v>
       </c>
       <c r="C357" s="2" t="s">
-        <v>990</v>
+        <v>971</v>
       </c>
     </row>
     <row r="358" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A358" s="2" t="s">
-        <v>991</v>
+        <v>1000</v>
       </c>
       <c r="B358" s="2" t="s">
-        <v>992</v>
+        <v>1001</v>
       </c>
       <c r="C358" s="2" t="s">
-        <v>993</v>
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="359" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A359" s="2" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B359" s="2" t="s">
+        <v>1004</v>
+      </c>
+      <c r="C359" s="2" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="360" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A360" s="2" t="s">
+        <v>1006</v>
+      </c>
+      <c r="B360" s="2" t="s">
+        <v>971</v>
+      </c>
+      <c r="C360" s="2" t="s">
+        <v>971</v>
+      </c>
+    </row>
+    <row r="361" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A361" s="2" t="s">
+        <v>1007</v>
+      </c>
+      <c r="B361" s="2" t="s">
+        <v>1008</v>
+      </c>
+      <c r="C361" s="2" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="362" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A362" s="2" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B362" s="2" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C362" s="2" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="363" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A363" s="2" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B363" s="2" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C363" s="2" t="s">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="364" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A364" s="2" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B364" s="2" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C364" s="2" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="365" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A365" s="2" t="s">
+        <v>1018</v>
+      </c>
+      <c r="B365" s="2" t="s">
+        <v>1019</v>
+      </c>
+      <c r="C365" s="2" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="366" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A366" s="2" t="s">
+        <v>1021</v>
+      </c>
+      <c r="B366" s="2" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C366" s="2" t="s">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="367" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A367" s="2" t="s">
+        <v>1022</v>
+      </c>
+      <c r="B367" s="2" t="s">
+        <v>1023</v>
+      </c>
+      <c r="C367" s="2" t="s">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="368" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A368" s="2" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B368" s="2" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C368" s="2" t="s">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="369" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A369" s="2" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B369" s="2" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C369" s="2" t="s">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="370" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A370" s="2" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B370" s="2" t="s">
+        <v>1030</v>
+      </c>
+      <c r="C370" s="2" t="s">
+        <v>1031</v>
+      </c>
+    </row>
+    <row r="371" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A371" s="2" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B371" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="C371" s="2" t="s">
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="372" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A372" s="2" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B372" s="2" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C372" s="2" t="s">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="373" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A373" s="2" t="s">
+        <v>1036</v>
+      </c>
+      <c r="B373" s="2" t="s">
+        <v>1037</v>
+      </c>
+      <c r="C373" s="2" t="s">
+        <v>1038</v>
+      </c>
+    </row>
+    <row r="374" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A374" s="2" t="s">
+        <v>1039</v>
+      </c>
+      <c r="B374" s="2" t="s">
+        <v>1040</v>
+      </c>
+      <c r="C374" s="2" t="s">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="375" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A375" s="2" t="s">
+        <v>1042</v>
+      </c>
+      <c r="B375" s="2" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C375" s="2" t="s">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="376" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A376" s="2" t="s">
+        <v>1043</v>
+      </c>
+      <c r="B376" s="2" t="s">
+        <v>1044</v>
+      </c>
+      <c r="C376" s="2" t="s">
+        <v>1045</v>
+      </c>
+    </row>
+    <row r="377" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A377" s="2" t="s">
+        <v>1046</v>
+      </c>
+      <c r="B377" s="2" t="s">
+        <v>1047</v>
+      </c>
+      <c r="C377" s="2" t="s">
+        <v>1048</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(portal-web): 手機版 header 改為右側 burger 展開選單
原本 ≤860px 時 actions 換行成兩行；改為固定單行，actions 收進
burger 下拉卡片，icon 鈕攤平為 icon + 文字列。語系鈕比照登入膠囊
外型並顯示完整語言名稱；鈴鐺收進選單後 burger 以小圓點提示未讀。

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/portal-web/i18n.xlsx
+++ b/apps/portal-web/i18n.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1479" uniqueCount="1322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1515" uniqueCount="1352">
   <si>
     <t>key</t>
   </si>
@@ -106,6 +106,15 @@
     <t>Sign out</t>
   </si>
   <si>
+    <t>nav.menu</t>
+  </si>
+  <si>
+    <t>選單</t>
+  </si>
+  <si>
+    <t>Menu</t>
+  </si>
+  <si>
     <t>nav.menuAria</t>
   </si>
   <si>
@@ -2251,10 +2260,19 @@
     <t>landing.discover.title</t>
   </si>
   <si>
-    <t>在它們成為主流之前，先發現它們。</t>
-  </si>
-  <si>
-    <t>Discover independent works before they become mainstream.</t>
+    <t>在它們成為主流之前，先{mark}它們。</t>
+  </si>
+  <si>
+    <t>Discover independent works before they become {mark}.</t>
+  </si>
+  <si>
+    <t>landing.discover.titleMark</t>
+  </si>
+  <si>
+    <t>發現</t>
+  </si>
+  <si>
+    <t>mainstream</t>
   </si>
   <si>
     <t>landing.discover.text</t>
@@ -2293,6 +2311,15 @@
     <t>My library</t>
   </si>
   <si>
+    <t>landing.discover.trackLabel</t>
+  </si>
+  <si>
+    <t>曲目試聽</t>
+  </si>
+  <si>
+    <t>Track preview</t>
+  </si>
+  <si>
     <t>landing.discover.follow</t>
   </si>
   <si>
@@ -2302,6 +2329,60 @@
     <t>Follow</t>
   </si>
   <si>
+    <t>landing.publish.eyebrow</t>
+  </si>
+  <si>
+    <t>想發表，就發表</t>
+  </si>
+  <si>
+    <t>Want to publish? Just publish.</t>
+  </si>
+  <si>
+    <t>landing.publish.title</t>
+  </si>
+  <si>
+    <t>一本獨立誌、一份教學指南、一張一張寫下去的樂譜。</t>
+  </si>
+  <si>
+    <t>An indie zine, a how-to guide, a score written one line at a time.</t>
+  </si>
+  <si>
+    <t>landing.publish.text</t>
+  </si>
+  <si>
+    <t>不用等出版社點頭、不用經紀約、不用演算法賞臉——寫完就上架，價格自己定，粉絲直接跟你買。</t>
+  </si>
+  <si>
+    <t>No publisher's nod, no agent contract, no algorithm to please — finish it, list it, set your own price, and let fans buy straight from you.</t>
+  </si>
+  <si>
+    <t>landing.publish.tags.0</t>
+  </si>
+  <si>
+    <t>Guide</t>
+  </si>
+  <si>
+    <t>landing.publish.tags.1</t>
+  </si>
+  <si>
+    <t>Zine</t>
+  </si>
+  <si>
+    <t>landing.publish.tags.2</t>
+  </si>
+  <si>
+    <t>landing.publish.tags.3</t>
+  </si>
+  <si>
+    <t>landing.publish.badge</t>
+  </si>
+  <si>
+    <t>寫完 → 上架 → 開賣</t>
+  </si>
+  <si>
+    <t>Write → List → Sell</t>
+  </si>
+  <si>
     <t>landing.why.eyebrow</t>
   </si>
   <si>
@@ -2395,10 +2476,19 @@
     <t>landing.cta.eyebrow</t>
   </si>
   <si>
-    <t>故事的下一頁，由你翻開</t>
-  </si>
-  <si>
-    <t>The next page of the story is yours to turn</t>
+    <t>・故事的下一頁，由{mark}翻開・</t>
+  </si>
+  <si>
+    <t>The next page of the story is {mark} to turn</t>
+  </si>
+  <si>
+    <t>landing.cta.eyebrowMark</t>
+  </si>
+  <si>
+    <t>你</t>
+  </si>
+  <si>
+    <t>yours</t>
   </si>
   <si>
     <t>landing.cta.creator.title</t>
@@ -4366,7 +4456,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C493"/>
+  <dimension ref="A1:C505"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -4554,21 +4644,21 @@
         <v>46</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4763,18 +4853,18 @@
         <v>101</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>69</v>
+        <v>102</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="37" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>105</v>
@@ -4898,15 +4988,15 @@
         <v>137</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="49" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>140</v>
@@ -4931,15 +5021,15 @@
         <v>145</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="52" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>148</v>
@@ -5016,32 +5106,32 @@
         <v>167</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>131</v>
+        <v>168</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>132</v>
+        <v>169</v>
       </c>
     </row>
     <row r="60" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>169</v>
+        <v>134</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>157</v>
+        <v>135</v>
       </c>
     </row>
     <row r="61" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
     </row>
     <row r="62" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5060,21 +5150,21 @@
         <v>176</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>44</v>
+        <v>177</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>45</v>
+        <v>178</v>
       </c>
     </row>
     <row r="64" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>178</v>
+        <v>47</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>179</v>
+        <v>48</v>
       </c>
     </row>
     <row r="65" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5085,15 +5175,15 @@
         <v>181</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="66" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C66" s="2" t="s">
         <v>184</v>
@@ -5140,15 +5230,15 @@
         <v>195</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="71" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C71" s="2" t="s">
         <v>198</v>
@@ -5390,21 +5480,21 @@
         <v>262</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>159</v>
+        <v>263</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>160</v>
+        <v>264</v>
       </c>
     </row>
     <row r="94" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>264</v>
+        <v>162</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>265</v>
+        <v>163</v>
       </c>
     </row>
     <row r="95" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5434,51 +5524,51 @@
         <v>272</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>7</v>
+        <v>273</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>8</v>
+        <v>274</v>
       </c>
     </row>
     <row r="98" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>274</v>
+        <v>7</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>274</v>
+        <v>8</v>
       </c>
     </row>
     <row r="99" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="100" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="101" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C101" s="2" t="s">
         <v>281</v>
@@ -5555,21 +5645,21 @@
         <v>300</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>156</v>
+        <v>301</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>157</v>
+        <v>302</v>
       </c>
     </row>
     <row r="109" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>302</v>
+        <v>159</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>303</v>
+        <v>160</v>
       </c>
     </row>
     <row r="110" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5731,21 +5821,21 @@
         <v>346</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>51</v>
+        <v>347</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>52</v>
+        <v>348</v>
       </c>
     </row>
     <row r="125" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>348</v>
+        <v>54</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>349</v>
+        <v>55</v>
       </c>
     </row>
     <row r="126" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5973,21 +6063,21 @@
         <v>410</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>48</v>
+        <v>411</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>49</v>
+        <v>412</v>
       </c>
     </row>
     <row r="147" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>412</v>
+        <v>51</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>413</v>
+        <v>52</v>
       </c>
     </row>
     <row r="148" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6306,15 +6396,15 @@
         <v>499</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="177" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="C177" s="2" t="s">
         <v>502</v>
@@ -6339,29 +6429,29 @@
         <v>507</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
     </row>
     <row r="180" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>295</v>
+        <v>510</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>296</v>
+        <v>510</v>
       </c>
     </row>
     <row r="181" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>510</v>
+        <v>298</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>511</v>
+        <v>299</v>
       </c>
     </row>
     <row r="182" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6405,15 +6495,15 @@
         <v>522</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
     </row>
     <row r="186" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="C186" s="2" t="s">
         <v>525</v>
@@ -6457,21 +6547,21 @@
         <v>535</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>17</v>
+        <v>536</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>18</v>
+        <v>537</v>
       </c>
     </row>
     <row r="191" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>537</v>
+        <v>17</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>538</v>
+        <v>18</v>
       </c>
     </row>
     <row r="192" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6479,21 +6569,21 @@
         <v>539</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>20</v>
+        <v>540</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>21</v>
+        <v>541</v>
       </c>
     </row>
     <row r="193" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>541</v>
+        <v>20</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>542</v>
+        <v>21</v>
       </c>
     </row>
     <row r="194" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6743,21 +6833,21 @@
         <v>609</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>78</v>
+        <v>610</v>
       </c>
       <c r="C216" s="2" t="s">
-        <v>79</v>
+        <v>611</v>
       </c>
     </row>
     <row r="217" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A217" s="2" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>611</v>
+        <v>81</v>
       </c>
       <c r="C217" s="2" t="s">
-        <v>612</v>
+        <v>82</v>
       </c>
     </row>
     <row r="218" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6765,18 +6855,18 @@
         <v>613</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>84</v>
+        <v>614</v>
       </c>
       <c r="C218" s="2" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
     </row>
     <row r="219" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>616</v>
+        <v>87</v>
       </c>
       <c r="C219" s="2" t="s">
         <v>617</v>
@@ -6955,18 +7045,18 @@
         <v>664</v>
       </c>
       <c r="C235" s="2" t="s">
-        <v>64</v>
+        <v>665</v>
       </c>
     </row>
     <row r="236" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A236" s="2" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B236" s="2" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="C236" s="2" t="s">
-        <v>667</v>
+        <v>67</v>
       </c>
     </row>
     <row r="237" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7029,18 +7119,18 @@
         <v>683</v>
       </c>
       <c r="B242" s="2" t="s">
-        <v>96</v>
+        <v>684</v>
       </c>
       <c r="C242" s="2" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
     </row>
     <row r="243" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A243" s="2" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="B243" s="2" t="s">
-        <v>686</v>
+        <v>99</v>
       </c>
       <c r="C243" s="2" t="s">
         <v>687</v>
@@ -7392,197 +7482,197 @@
         <v>781</v>
       </c>
       <c r="B275" s="2" t="s">
+        <v>695</v>
+      </c>
+      <c r="C275" s="2" t="s">
         <v>782</v>
-      </c>
-      <c r="C275" s="2" t="s">
-        <v>783</v>
       </c>
     </row>
     <row r="276" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A276" s="2" t="s">
+        <v>783</v>
+      </c>
+      <c r="B276" s="2" t="s">
+        <v>698</v>
+      </c>
+      <c r="C276" s="2" t="s">
         <v>784</v>
-      </c>
-      <c r="B276" s="2" t="s">
-        <v>785</v>
-      </c>
-      <c r="C276" s="2" t="s">
-        <v>786</v>
       </c>
     </row>
     <row r="277" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A277" s="2" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
       <c r="B277" s="2" t="s">
-        <v>788</v>
+        <v>701</v>
       </c>
       <c r="C277" s="2" t="s">
-        <v>789</v>
+        <v>701</v>
       </c>
     </row>
     <row r="278" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A278" s="2" t="s">
-        <v>790</v>
+        <v>786</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>791</v>
+        <v>704</v>
       </c>
       <c r="C278" s="2" t="s">
-        <v>792</v>
+        <v>704</v>
       </c>
     </row>
     <row r="279" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A279" s="2" t="s">
-        <v>793</v>
+        <v>787</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>794</v>
+        <v>788</v>
       </c>
       <c r="C279" s="2" t="s">
-        <v>795</v>
+        <v>789</v>
       </c>
     </row>
     <row r="280" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A280" s="2" t="s">
-        <v>796</v>
+        <v>790</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>797</v>
+        <v>791</v>
       </c>
       <c r="C280" s="2" t="s">
-        <v>798</v>
+        <v>792</v>
       </c>
     </row>
     <row r="281" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A281" s="2" t="s">
-        <v>799</v>
+        <v>793</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>800</v>
+        <v>794</v>
       </c>
       <c r="C281" s="2" t="s">
-        <v>801</v>
+        <v>795</v>
       </c>
     </row>
     <row r="282" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A282" s="2" t="s">
-        <v>802</v>
+        <v>796</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>803</v>
+        <v>797</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>804</v>
+        <v>798</v>
       </c>
     </row>
     <row r="283" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A283" s="2" t="s">
-        <v>805</v>
+        <v>799</v>
       </c>
       <c r="B283" s="2" t="s">
-        <v>806</v>
+        <v>800</v>
       </c>
       <c r="C283" s="2" t="s">
-        <v>807</v>
+        <v>801</v>
       </c>
     </row>
     <row r="284" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A284" s="2" t="s">
-        <v>808</v>
+        <v>802</v>
       </c>
       <c r="B284" s="2" t="s">
-        <v>809</v>
+        <v>803</v>
       </c>
       <c r="C284" s="2" t="s">
-        <v>810</v>
+        <v>804</v>
       </c>
     </row>
     <row r="285" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A285" s="2" t="s">
-        <v>811</v>
+        <v>805</v>
       </c>
       <c r="B285" s="2" t="s">
-        <v>812</v>
+        <v>806</v>
       </c>
       <c r="C285" s="2" t="s">
-        <v>813</v>
+        <v>807</v>
       </c>
     </row>
     <row r="286" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A286" s="2" t="s">
-        <v>814</v>
+        <v>808</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>815</v>
+        <v>809</v>
       </c>
       <c r="C286" s="2" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
     </row>
     <row r="287" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A287" s="2" t="s">
-        <v>816</v>
+        <v>811</v>
       </c>
       <c r="B287" s="2" t="s">
-        <v>84</v>
+        <v>812</v>
       </c>
       <c r="C287" s="2" t="s">
-        <v>817</v>
+        <v>813</v>
       </c>
     </row>
     <row r="288" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A288" s="2" t="s">
-        <v>818</v>
+        <v>814</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>616</v>
+        <v>815</v>
       </c>
       <c r="C288" s="2" t="s">
-        <v>819</v>
+        <v>816</v>
       </c>
     </row>
     <row r="289" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A289" s="2" t="s">
-        <v>820</v>
+        <v>817</v>
       </c>
       <c r="B289" s="2" t="s">
-        <v>619</v>
+        <v>818</v>
       </c>
       <c r="C289" s="2" t="s">
-        <v>821</v>
+        <v>819</v>
       </c>
     </row>
     <row r="290" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A290" s="2" t="s">
+        <v>820</v>
+      </c>
+      <c r="B290" s="2" t="s">
+        <v>821</v>
+      </c>
+      <c r="C290" s="2" t="s">
         <v>822</v>
-      </c>
-      <c r="B290" s="2" t="s">
-        <v>823</v>
-      </c>
-      <c r="C290" s="2" t="s">
-        <v>824</v>
       </c>
     </row>
     <row r="291" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A291" s="2" t="s">
+        <v>823</v>
+      </c>
+      <c r="B291" s="2" t="s">
+        <v>824</v>
+      </c>
+      <c r="C291" s="2" t="s">
         <v>825</v>
-      </c>
-      <c r="B291" s="2" t="s">
-        <v>826</v>
-      </c>
-      <c r="C291" s="2" t="s">
-        <v>827</v>
       </c>
     </row>
     <row r="292" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A292" s="2" t="s">
+        <v>826</v>
+      </c>
+      <c r="B292" s="2" t="s">
+        <v>827</v>
+      </c>
+      <c r="C292" s="2" t="s">
         <v>828</v>
-      </c>
-      <c r="B292" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C292" s="2" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="293" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7648,315 +7738,315 @@
         <v>845</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="299" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A299" s="2" t="s">
+        <v>846</v>
+      </c>
+      <c r="B299" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C299" s="2" t="s">
         <v>847</v>
-      </c>
-      <c r="B299" s="2" t="s">
-        <v>848</v>
-      </c>
-      <c r="C299" s="2" t="s">
-        <v>849</v>
       </c>
     </row>
     <row r="300" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A300" s="2" t="s">
-        <v>850</v>
+        <v>848</v>
       </c>
       <c r="B300" s="2" t="s">
-        <v>851</v>
+        <v>619</v>
       </c>
       <c r="C300" s="2" t="s">
-        <v>852</v>
+        <v>849</v>
       </c>
     </row>
     <row r="301" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A301" s="2" t="s">
-        <v>853</v>
+        <v>850</v>
       </c>
       <c r="B301" s="2" t="s">
-        <v>854</v>
+        <v>622</v>
       </c>
       <c r="C301" s="2" t="s">
-        <v>855</v>
+        <v>851</v>
       </c>
     </row>
     <row r="302" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A302" s="2" t="s">
-        <v>856</v>
+        <v>852</v>
       </c>
       <c r="B302" s="2" t="s">
-        <v>857</v>
+        <v>853</v>
       </c>
       <c r="C302" s="2" t="s">
-        <v>858</v>
+        <v>854</v>
       </c>
     </row>
     <row r="303" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A303" s="2" t="s">
-        <v>859</v>
+        <v>855</v>
       </c>
       <c r="B303" s="2" t="s">
-        <v>860</v>
+        <v>856</v>
       </c>
       <c r="C303" s="2" t="s">
-        <v>861</v>
+        <v>857</v>
       </c>
     </row>
     <row r="304" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A304" s="2" t="s">
-        <v>862</v>
+        <v>858</v>
       </c>
       <c r="B304" s="2" t="s">
-        <v>863</v>
+        <v>60</v>
       </c>
       <c r="C304" s="2" t="s">
-        <v>864</v>
+        <v>61</v>
       </c>
     </row>
     <row r="305" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A305" s="2" t="s">
-        <v>865</v>
+        <v>859</v>
       </c>
       <c r="B305" s="2" t="s">
-        <v>866</v>
+        <v>860</v>
       </c>
       <c r="C305" s="2" t="s">
-        <v>867</v>
+        <v>861</v>
       </c>
     </row>
     <row r="306" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A306" s="2" t="s">
-        <v>868</v>
+        <v>862</v>
       </c>
       <c r="B306" s="2" t="s">
-        <v>869</v>
+        <v>863</v>
       </c>
       <c r="C306" s="2" t="s">
-        <v>870</v>
+        <v>864</v>
       </c>
     </row>
     <row r="307" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A307" s="2" t="s">
-        <v>871</v>
+        <v>865</v>
       </c>
       <c r="B307" s="2" t="s">
-        <v>872</v>
+        <v>866</v>
       </c>
       <c r="C307" s="2" t="s">
-        <v>873</v>
+        <v>867</v>
       </c>
     </row>
     <row r="308" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A308" s="2" t="s">
-        <v>874</v>
+        <v>868</v>
       </c>
       <c r="B308" s="2" t="s">
-        <v>875</v>
+        <v>869</v>
       </c>
       <c r="C308" s="2" t="s">
-        <v>876</v>
+        <v>870</v>
       </c>
     </row>
     <row r="309" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A309" s="2" t="s">
-        <v>877</v>
+        <v>871</v>
       </c>
       <c r="B309" s="2" t="s">
-        <v>878</v>
+        <v>872</v>
       </c>
       <c r="C309" s="2" t="s">
-        <v>879</v>
+        <v>873</v>
       </c>
     </row>
     <row r="310" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A310" s="2" t="s">
-        <v>880</v>
+        <v>874</v>
       </c>
       <c r="B310" s="2" t="s">
-        <v>881</v>
+        <v>875</v>
       </c>
       <c r="C310" s="2" t="s">
-        <v>882</v>
+        <v>876</v>
       </c>
     </row>
     <row r="311" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A311" s="2" t="s">
-        <v>883</v>
+        <v>877</v>
       </c>
       <c r="B311" s="2" t="s">
-        <v>884</v>
+        <v>878</v>
       </c>
       <c r="C311" s="2" t="s">
-        <v>885</v>
+        <v>879</v>
       </c>
     </row>
     <row r="312" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A312" s="2" t="s">
-        <v>886</v>
+        <v>880</v>
       </c>
       <c r="B312" s="2" t="s">
-        <v>887</v>
+        <v>881</v>
       </c>
       <c r="C312" s="2" t="s">
-        <v>888</v>
+        <v>882</v>
       </c>
     </row>
     <row r="313" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A313" s="2" t="s">
-        <v>889</v>
+        <v>883</v>
       </c>
       <c r="B313" s="2" t="s">
-        <v>890</v>
+        <v>884</v>
       </c>
       <c r="C313" s="2" t="s">
-        <v>891</v>
+        <v>885</v>
       </c>
     </row>
     <row r="314" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A314" s="2" t="s">
-        <v>892</v>
+        <v>886</v>
       </c>
       <c r="B314" s="2" t="s">
-        <v>893</v>
+        <v>887</v>
       </c>
       <c r="C314" s="2" t="s">
-        <v>894</v>
+        <v>888</v>
       </c>
     </row>
     <row r="315" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A315" s="2" t="s">
-        <v>895</v>
+        <v>889</v>
       </c>
       <c r="B315" s="2" t="s">
-        <v>896</v>
+        <v>890</v>
       </c>
       <c r="C315" s="2" t="s">
-        <v>897</v>
+        <v>891</v>
       </c>
     </row>
     <row r="316" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A316" s="2" t="s">
-        <v>898</v>
+        <v>892</v>
       </c>
       <c r="B316" s="2" t="s">
-        <v>899</v>
+        <v>893</v>
       </c>
       <c r="C316" s="2" t="s">
-        <v>900</v>
+        <v>894</v>
       </c>
     </row>
     <row r="317" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A317" s="2" t="s">
-        <v>901</v>
+        <v>895</v>
       </c>
       <c r="B317" s="2" t="s">
-        <v>902</v>
+        <v>896</v>
       </c>
       <c r="C317" s="2" t="s">
-        <v>903</v>
+        <v>897</v>
       </c>
     </row>
     <row r="318" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A318" s="2" t="s">
-        <v>904</v>
+        <v>898</v>
       </c>
       <c r="B318" s="2" t="s">
-        <v>905</v>
+        <v>899</v>
       </c>
       <c r="C318" s="2" t="s">
-        <v>906</v>
+        <v>900</v>
       </c>
     </row>
     <row r="319" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A319" s="2" t="s">
-        <v>907</v>
+        <v>901</v>
       </c>
       <c r="B319" s="2" t="s">
-        <v>490</v>
+        <v>902</v>
       </c>
       <c r="C319" s="2" t="s">
-        <v>491</v>
+        <v>903</v>
       </c>
     </row>
     <row r="320" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A320" s="2" t="s">
-        <v>908</v>
+        <v>904</v>
       </c>
       <c r="B320" s="2" t="s">
-        <v>909</v>
+        <v>905</v>
       </c>
       <c r="C320" s="2" t="s">
-        <v>910</v>
+        <v>906</v>
       </c>
     </row>
     <row r="321" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A321" s="2" t="s">
-        <v>911</v>
+        <v>907</v>
       </c>
       <c r="B321" s="2" t="s">
-        <v>912</v>
+        <v>908</v>
       </c>
       <c r="C321" s="2" t="s">
-        <v>913</v>
+        <v>909</v>
       </c>
     </row>
     <row r="322" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A322" s="2" t="s">
-        <v>914</v>
+        <v>910</v>
       </c>
       <c r="B322" s="2" t="s">
-        <v>915</v>
+        <v>911</v>
       </c>
       <c r="C322" s="2" t="s">
-        <v>915</v>
+        <v>912</v>
       </c>
     </row>
     <row r="323" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A323" s="2" t="s">
-        <v>916</v>
+        <v>913</v>
       </c>
       <c r="B323" s="2" t="s">
-        <v>917</v>
+        <v>914</v>
       </c>
       <c r="C323" s="2" t="s">
-        <v>917</v>
+        <v>915</v>
       </c>
     </row>
     <row r="324" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A324" s="2" t="s">
+        <v>916</v>
+      </c>
+      <c r="B324" s="2" t="s">
+        <v>917</v>
+      </c>
+      <c r="C324" s="2" t="s">
         <v>918</v>
-      </c>
-      <c r="B324" s="2" t="s">
-        <v>919</v>
-      </c>
-      <c r="C324" s="2" t="s">
-        <v>920</v>
       </c>
     </row>
     <row r="325" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A325" s="2" t="s">
+        <v>919</v>
+      </c>
+      <c r="B325" s="2" t="s">
+        <v>920</v>
+      </c>
+      <c r="C325" s="2" t="s">
         <v>921</v>
-      </c>
-      <c r="B325" s="2" t="s">
-        <v>922</v>
-      </c>
-      <c r="C325" s="2" t="s">
-        <v>923</v>
       </c>
     </row>
     <row r="326" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A326" s="2" t="s">
+        <v>922</v>
+      </c>
+      <c r="B326" s="2" t="s">
+        <v>923</v>
+      </c>
+      <c r="C326" s="2" t="s">
         <v>924</v>
-      </c>
-      <c r="B326" s="2" t="s">
-        <v>917</v>
-      </c>
-      <c r="C326" s="2" t="s">
-        <v>917</v>
       </c>
     </row>
     <row r="327" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7986,32 +8076,32 @@
         <v>931</v>
       </c>
       <c r="B329" s="2" t="s">
-        <v>917</v>
+        <v>932</v>
       </c>
       <c r="C329" s="2" t="s">
-        <v>917</v>
+        <v>933</v>
       </c>
     </row>
     <row r="330" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A330" s="2" t="s">
-        <v>932</v>
+        <v>934</v>
       </c>
       <c r="B330" s="2" t="s">
-        <v>933</v>
+        <v>935</v>
       </c>
       <c r="C330" s="2" t="s">
-        <v>934</v>
+        <v>936</v>
       </c>
     </row>
     <row r="331" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A331" s="2" t="s">
-        <v>935</v>
+        <v>937</v>
       </c>
       <c r="B331" s="2" t="s">
-        <v>936</v>
+        <v>493</v>
       </c>
       <c r="C331" s="2" t="s">
-        <v>937</v>
+        <v>494</v>
       </c>
     </row>
     <row r="332" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8019,670 +8109,670 @@
         <v>938</v>
       </c>
       <c r="B332" s="2" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="C332" s="2" t="s">
-        <v>917</v>
+        <v>940</v>
       </c>
     </row>
     <row r="333" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A333" s="2" t="s">
-        <v>939</v>
+        <v>941</v>
       </c>
       <c r="B333" s="2" t="s">
-        <v>940</v>
+        <v>942</v>
       </c>
       <c r="C333" s="2" t="s">
-        <v>941</v>
+        <v>943</v>
       </c>
     </row>
     <row r="334" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A334" s="2" t="s">
-        <v>942</v>
+        <v>944</v>
       </c>
       <c r="B334" s="2" t="s">
-        <v>943</v>
+        <v>945</v>
       </c>
       <c r="C334" s="2" t="s">
-        <v>944</v>
+        <v>945</v>
       </c>
     </row>
     <row r="335" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A335" s="2" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
       <c r="B335" s="2" t="s">
-        <v>917</v>
+        <v>947</v>
       </c>
       <c r="C335" s="2" t="s">
-        <v>917</v>
+        <v>947</v>
       </c>
     </row>
     <row r="336" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A336" s="2" t="s">
-        <v>946</v>
+        <v>948</v>
       </c>
       <c r="B336" s="2" t="s">
-        <v>947</v>
+        <v>949</v>
       </c>
       <c r="C336" s="2" t="s">
-        <v>948</v>
+        <v>950</v>
       </c>
     </row>
     <row r="337" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A337" s="2" t="s">
-        <v>949</v>
+        <v>951</v>
       </c>
       <c r="B337" s="2" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="C337" s="2" t="s">
-        <v>951</v>
+        <v>953</v>
       </c>
     </row>
     <row r="338" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A338" s="2" t="s">
-        <v>952</v>
+        <v>954</v>
       </c>
       <c r="B338" s="2" t="s">
-        <v>953</v>
+        <v>947</v>
       </c>
       <c r="C338" s="2" t="s">
-        <v>953</v>
+        <v>947</v>
       </c>
     </row>
     <row r="339" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A339" s="2" t="s">
-        <v>954</v>
+        <v>955</v>
       </c>
       <c r="B339" s="2" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="C339" s="2" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
     </row>
     <row r="340" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A340" s="2" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="B340" s="2" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="C340" s="2" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
     </row>
     <row r="341" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A341" s="2" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="B341" s="2" t="s">
-        <v>953</v>
+        <v>947</v>
       </c>
       <c r="C341" s="2" t="s">
-        <v>953</v>
+        <v>947</v>
       </c>
     </row>
     <row r="342" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A342" s="2" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="B342" s="2" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="C342" s="2" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
     </row>
     <row r="343" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A343" s="2" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="B343" s="2" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="C343" s="2" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
     </row>
     <row r="344" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A344" s="2" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="B344" s="2" t="s">
-        <v>953</v>
+        <v>947</v>
       </c>
       <c r="C344" s="2" t="s">
-        <v>953</v>
+        <v>947</v>
       </c>
     </row>
     <row r="345" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A345" s="2" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="B345" s="2" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="C345" s="2" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
     </row>
     <row r="346" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A346" s="2" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="B346" s="2" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="C346" s="2" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
     </row>
     <row r="347" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A347" s="2" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="B347" s="2" t="s">
-        <v>953</v>
+        <v>947</v>
       </c>
       <c r="C347" s="2" t="s">
-        <v>953</v>
+        <v>947</v>
       </c>
     </row>
     <row r="348" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A348" s="2" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="B348" s="2" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="C348" s="2" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
     </row>
     <row r="349" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A349" s="2" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="B349" s="2" t="s">
-        <v>979</v>
+        <v>980</v>
       </c>
       <c r="C349" s="2" t="s">
-        <v>980</v>
+        <v>981</v>
       </c>
     </row>
     <row r="350" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A350" s="2" t="s">
-        <v>981</v>
+        <v>982</v>
       </c>
       <c r="B350" s="2" t="s">
-        <v>953</v>
+        <v>983</v>
       </c>
       <c r="C350" s="2" t="s">
-        <v>953</v>
+        <v>983</v>
       </c>
     </row>
     <row r="351" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A351" s="2" t="s">
-        <v>982</v>
+        <v>984</v>
       </c>
       <c r="B351" s="2" t="s">
-        <v>983</v>
+        <v>985</v>
       </c>
       <c r="C351" s="2" t="s">
-        <v>984</v>
+        <v>986</v>
       </c>
     </row>
     <row r="352" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A352" s="2" t="s">
-        <v>985</v>
+        <v>987</v>
       </c>
       <c r="B352" s="2" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
       <c r="C352" s="2" t="s">
-        <v>987</v>
+        <v>989</v>
       </c>
     </row>
     <row r="353" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A353" s="2" t="s">
-        <v>988</v>
+        <v>990</v>
       </c>
       <c r="B353" s="2" t="s">
-        <v>953</v>
+        <v>983</v>
       </c>
       <c r="C353" s="2" t="s">
-        <v>953</v>
+        <v>983</v>
       </c>
     </row>
     <row r="354" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A354" s="2" t="s">
-        <v>989</v>
+        <v>991</v>
       </c>
       <c r="B354" s="2" t="s">
-        <v>990</v>
+        <v>992</v>
       </c>
       <c r="C354" s="2" t="s">
-        <v>991</v>
+        <v>993</v>
       </c>
     </row>
     <row r="355" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A355" s="2" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="B355" s="2" t="s">
-        <v>993</v>
+        <v>995</v>
       </c>
       <c r="C355" s="2" t="s">
-        <v>994</v>
+        <v>996</v>
       </c>
     </row>
     <row r="356" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A356" s="2" t="s">
-        <v>995</v>
+        <v>997</v>
       </c>
       <c r="B356" s="2" t="s">
-        <v>953</v>
+        <v>983</v>
       </c>
       <c r="C356" s="2" t="s">
-        <v>953</v>
+        <v>983</v>
       </c>
     </row>
     <row r="357" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A357" s="2" t="s">
-        <v>996</v>
+        <v>998</v>
       </c>
       <c r="B357" s="2" t="s">
-        <v>997</v>
+        <v>999</v>
       </c>
       <c r="C357" s="2" t="s">
-        <v>998</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="358" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A358" s="2" t="s">
-        <v>999</v>
+        <v>1001</v>
       </c>
       <c r="B358" s="2" t="s">
-        <v>1000</v>
+        <v>1002</v>
       </c>
       <c r="C358" s="2" t="s">
-        <v>1001</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="359" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A359" s="2" t="s">
-        <v>1002</v>
+        <v>1004</v>
       </c>
       <c r="B359" s="2" t="s">
-        <v>1003</v>
+        <v>983</v>
       </c>
       <c r="C359" s="2" t="s">
-        <v>1003</v>
+        <v>983</v>
       </c>
     </row>
     <row r="360" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A360" s="2" t="s">
-        <v>1004</v>
+        <v>1005</v>
       </c>
       <c r="B360" s="2" t="s">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="C360" s="2" t="s">
-        <v>1006</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="361" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A361" s="2" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="B361" s="2" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="C361" s="2" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="362" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A362" s="2" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="B362" s="2" t="s">
-        <v>1003</v>
+        <v>983</v>
       </c>
       <c r="C362" s="2" t="s">
-        <v>1003</v>
+        <v>983</v>
       </c>
     </row>
     <row r="363" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A363" s="2" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="B363" s="2" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="C363" s="2" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="364" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A364" s="2" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="B364" s="2" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="C364" s="2" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="365" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A365" s="2" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="B365" s="2" t="s">
-        <v>1003</v>
+        <v>983</v>
       </c>
       <c r="C365" s="2" t="s">
-        <v>1003</v>
+        <v>983</v>
       </c>
     </row>
     <row r="366" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A366" s="2" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="B366" s="2" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="C366" s="2" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="367" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A367" s="2" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="B367" s="2" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="C367" s="2" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="368" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A368" s="2" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="B368" s="2" t="s">
-        <v>1003</v>
+        <v>983</v>
       </c>
       <c r="C368" s="2" t="s">
-        <v>1003</v>
+        <v>983</v>
       </c>
     </row>
     <row r="369" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A369" s="2" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="B369" s="2" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="C369" s="2" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="370" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A370" s="2" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="B370" s="2" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="C370" s="2" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="371" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A371" s="2" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="B371" s="2" t="s">
-        <v>1003</v>
+        <v>1033</v>
       </c>
       <c r="C371" s="2" t="s">
-        <v>1003</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="372" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A372" s="2" t="s">
-        <v>1032</v>
+        <v>1034</v>
       </c>
       <c r="B372" s="2" t="s">
-        <v>1033</v>
+        <v>1035</v>
       </c>
       <c r="C372" s="2" t="s">
-        <v>1034</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="373" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A373" s="2" t="s">
-        <v>1035</v>
+        <v>1037</v>
       </c>
       <c r="B373" s="2" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
       <c r="C373" s="2" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="374" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A374" s="2" t="s">
-        <v>1038</v>
+        <v>1040</v>
       </c>
       <c r="B374" s="2" t="s">
-        <v>1003</v>
+        <v>1033</v>
       </c>
       <c r="C374" s="2" t="s">
-        <v>1003</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="375" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A375" s="2" t="s">
-        <v>1039</v>
+        <v>1041</v>
       </c>
       <c r="B375" s="2" t="s">
-        <v>1040</v>
+        <v>1042</v>
       </c>
       <c r="C375" s="2" t="s">
-        <v>1041</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="376" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A376" s="2" t="s">
-        <v>1042</v>
+        <v>1044</v>
       </c>
       <c r="B376" s="2" t="s">
-        <v>1043</v>
+        <v>1045</v>
       </c>
       <c r="C376" s="2" t="s">
-        <v>1044</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="377" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A377" s="2" t="s">
-        <v>1045</v>
+        <v>1047</v>
       </c>
       <c r="B377" s="2" t="s">
-        <v>1046</v>
+        <v>1033</v>
       </c>
       <c r="C377" s="2" t="s">
-        <v>1046</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="378" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A378" s="2" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="B378" s="2" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="C378" s="2" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="379" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A379" s="2" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="B379" s="2" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="C379" s="2" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="380" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A380" s="2" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="B380" s="2" t="s">
-        <v>1046</v>
+        <v>1033</v>
       </c>
       <c r="C380" s="2" t="s">
-        <v>1046</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="381" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A381" s="2" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="B381" s="2" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
       <c r="C381" s="2" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="382" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A382" s="2" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="B382" s="2" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="C382" s="2" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="383" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A383" s="2" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
       <c r="B383" s="2" t="s">
-        <v>1046</v>
+        <v>1033</v>
       </c>
       <c r="C383" s="2" t="s">
-        <v>1046</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="384" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A384" s="2" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="B384" s="2" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="C384" s="2" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="385" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A385" s="2" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="B385" s="2" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="C385" s="2" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="386" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A386" s="2" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="B386" s="2" t="s">
-        <v>1046</v>
+        <v>1033</v>
       </c>
       <c r="C386" s="2" t="s">
-        <v>1046</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="387" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A387" s="2" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="B387" s="2" t="s">
-        <v>1069</v>
+        <v>1070</v>
       </c>
       <c r="C387" s="2" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
     </row>
     <row r="388" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A388" s="2" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="B388" s="2" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="C388" s="2" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="389" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A389" s="2" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
       <c r="B389" s="2" t="s">
-        <v>1046</v>
+        <v>1076</v>
       </c>
       <c r="C389" s="2" t="s">
-        <v>1046</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="390" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A390" s="2" t="s">
-        <v>1075</v>
+        <v>1077</v>
       </c>
       <c r="B390" s="2" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="C390" s="2" t="s">
-        <v>1077</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="391" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A391" s="2" t="s">
-        <v>1078</v>
+        <v>1080</v>
       </c>
       <c r="B391" s="2" t="s">
-        <v>1079</v>
+        <v>1081</v>
       </c>
       <c r="C391" s="2" t="s">
-        <v>1080</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="392" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A392" s="2" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="B392" s="2" t="s">
-        <v>1082</v>
+        <v>1076</v>
       </c>
       <c r="C392" s="2" t="s">
-        <v>1083</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="393" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8712,87 +8802,87 @@
         <v>1090</v>
       </c>
       <c r="B395" s="2" t="s">
-        <v>1091</v>
+        <v>1076</v>
       </c>
       <c r="C395" s="2" t="s">
-        <v>1092</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="396" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A396" s="2" t="s">
+        <v>1091</v>
+      </c>
+      <c r="B396" s="2" t="s">
+        <v>1092</v>
+      </c>
+      <c r="C396" s="2" t="s">
         <v>1093</v>
-      </c>
-      <c r="B396" s="2" t="s">
-        <v>1094</v>
-      </c>
-      <c r="C396" s="2" t="s">
-        <v>1095</v>
       </c>
     </row>
     <row r="397" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A397" s="2" t="s">
+        <v>1094</v>
+      </c>
+      <c r="B397" s="2" t="s">
+        <v>1095</v>
+      </c>
+      <c r="C397" s="2" t="s">
         <v>1096</v>
-      </c>
-      <c r="B397" s="2" t="s">
-        <v>1097</v>
-      </c>
-      <c r="C397" s="2" t="s">
-        <v>494</v>
       </c>
     </row>
     <row r="398" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A398" s="2" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="B398" s="2" t="s">
-        <v>1099</v>
+        <v>1076</v>
       </c>
       <c r="C398" s="2" t="s">
-        <v>1099</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="399" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A399" s="2" t="s">
+        <v>1098</v>
+      </c>
+      <c r="B399" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="C399" s="2" t="s">
         <v>1100</v>
-      </c>
-      <c r="B399" s="2" t="s">
-        <v>1101</v>
-      </c>
-      <c r="C399" s="2" t="s">
-        <v>1102</v>
       </c>
     </row>
     <row r="400" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A400" s="2" t="s">
+        <v>1101</v>
+      </c>
+      <c r="B400" s="2" t="s">
+        <v>1102</v>
+      </c>
+      <c r="C400" s="2" t="s">
         <v>1103</v>
-      </c>
-      <c r="B400" s="2" t="s">
-        <v>1104</v>
-      </c>
-      <c r="C400" s="2" t="s">
-        <v>1105</v>
       </c>
     </row>
     <row r="401" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A401" s="2" t="s">
-        <v>1106</v>
+        <v>1104</v>
       </c>
       <c r="B401" s="2" t="s">
-        <v>640</v>
+        <v>1076</v>
       </c>
       <c r="C401" s="2" t="s">
-        <v>641</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="402" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A402" s="2" t="s">
+        <v>1105</v>
+      </c>
+      <c r="B402" s="2" t="s">
+        <v>1106</v>
+      </c>
+      <c r="C402" s="2" t="s">
         <v>1107</v>
-      </c>
-      <c r="B402" s="2" t="s">
-        <v>664</v>
-      </c>
-      <c r="C402" s="2" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="403" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8800,84 +8890,84 @@
         <v>1108</v>
       </c>
       <c r="B403" s="2" t="s">
-        <v>96</v>
+        <v>1109</v>
       </c>
       <c r="C403" s="2" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="404" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A404" s="2" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B404" s="2" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="C404" s="2" t="s">
-        <v>1112</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="405" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A405" s="2" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
       <c r="B405" s="2" t="s">
-        <v>1114</v>
+        <v>1115</v>
       </c>
       <c r="C405" s="2" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="406" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A406" s="2" t="s">
-        <v>1116</v>
+        <v>1117</v>
       </c>
       <c r="B406" s="2" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="C406" s="2" t="s">
-        <v>79</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="407" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A407" s="2" t="s">
-        <v>1118</v>
+        <v>1120</v>
       </c>
       <c r="B407" s="2" t="s">
-        <v>1119</v>
+        <v>1121</v>
       </c>
       <c r="C407" s="2" t="s">
-        <v>1120</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="408" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A408" s="2" t="s">
-        <v>1121</v>
+        <v>1123</v>
       </c>
       <c r="B408" s="2" t="s">
-        <v>1122</v>
+        <v>1124</v>
       </c>
       <c r="C408" s="2" t="s">
-        <v>1123</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="409" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A409" s="2" t="s">
-        <v>1124</v>
+        <v>1126</v>
       </c>
       <c r="B409" s="2" t="s">
-        <v>1125</v>
+        <v>1127</v>
       </c>
       <c r="C409" s="2" t="s">
-        <v>1126</v>
+        <v>497</v>
       </c>
     </row>
     <row r="410" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A410" s="2" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="B410" s="2" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="C410" s="2" t="s">
         <v>1129</v>
@@ -8891,29 +8981,29 @@
         <v>1131</v>
       </c>
       <c r="C411" s="2" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="412" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A412" s="2" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="B412" s="2" t="s">
-        <v>1133</v>
+        <v>1134</v>
       </c>
       <c r="C412" s="2" t="s">
-        <v>1134</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="413" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A413" s="2" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="B413" s="2" t="s">
-        <v>1136</v>
+        <v>643</v>
       </c>
       <c r="C413" s="2" t="s">
-        <v>1136</v>
+        <v>644</v>
       </c>
     </row>
     <row r="414" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8921,10 +9011,10 @@
         <v>1137</v>
       </c>
       <c r="B414" s="2" t="s">
-        <v>317</v>
+        <v>667</v>
       </c>
       <c r="C414" s="2" t="s">
-        <v>318</v>
+        <v>67</v>
       </c>
     </row>
     <row r="415" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8932,7 +9022,7 @@
         <v>1138</v>
       </c>
       <c r="B415" s="2" t="s">
-        <v>1139</v>
+        <v>99</v>
       </c>
       <c r="C415" s="2" t="s">
         <v>1139</v>
@@ -8946,224 +9036,224 @@
         <v>1141</v>
       </c>
       <c r="C416" s="2" t="s">
-        <v>1141</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="417" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A417" s="2" t="s">
-        <v>1142</v>
+        <v>1143</v>
       </c>
       <c r="B417" s="2" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
       <c r="C417" s="2" t="s">
-        <v>1143</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="418" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A418" s="2" t="s">
-        <v>1144</v>
+        <v>1146</v>
       </c>
       <c r="B418" s="2" t="s">
-        <v>323</v>
+        <v>1147</v>
       </c>
       <c r="C418" s="2" t="s">
-        <v>324</v>
+        <v>82</v>
       </c>
     </row>
     <row r="419" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A419" s="2" t="s">
-        <v>1145</v>
+        <v>1148</v>
       </c>
       <c r="B419" s="2" t="s">
-        <v>1146</v>
+        <v>1149</v>
       </c>
       <c r="C419" s="2" t="s">
-        <v>1146</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="420" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A420" s="2" t="s">
-        <v>1147</v>
+        <v>1151</v>
       </c>
       <c r="B420" s="2" t="s">
-        <v>1148</v>
+        <v>1152</v>
       </c>
       <c r="C420" s="2" t="s">
-        <v>1148</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="421" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A421" s="2" t="s">
-        <v>1149</v>
+        <v>1154</v>
       </c>
       <c r="B421" s="2" t="s">
-        <v>1150</v>
+        <v>1155</v>
       </c>
       <c r="C421" s="2" t="s">
-        <v>1150</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="422" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A422" s="2" t="s">
-        <v>1151</v>
+        <v>1157</v>
       </c>
       <c r="B422" s="2" t="s">
-        <v>1152</v>
+        <v>1158</v>
       </c>
       <c r="C422" s="2" t="s">
-        <v>1153</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="423" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A423" s="2" t="s">
-        <v>1154</v>
+        <v>1160</v>
       </c>
       <c r="B423" s="2" t="s">
-        <v>7</v>
+        <v>1161</v>
       </c>
       <c r="C423" s="2" t="s">
-        <v>8</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="424" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A424" s="2" t="s">
-        <v>1155</v>
+        <v>1162</v>
       </c>
       <c r="B424" s="2" t="s">
-        <v>1156</v>
+        <v>1163</v>
       </c>
       <c r="C424" s="2" t="s">
-        <v>1156</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="425" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A425" s="2" t="s">
-        <v>1157</v>
+        <v>1165</v>
       </c>
       <c r="B425" s="2" t="s">
-        <v>1158</v>
+        <v>1166</v>
       </c>
       <c r="C425" s="2" t="s">
-        <v>1158</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="426" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A426" s="2" t="s">
-        <v>1159</v>
+        <v>1167</v>
       </c>
       <c r="B426" s="2" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="C426" s="2" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
     </row>
     <row r="427" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A427" s="2" t="s">
-        <v>1160</v>
+        <v>1168</v>
       </c>
       <c r="B427" s="2" t="s">
-        <v>1161</v>
+        <v>1169</v>
       </c>
       <c r="C427" s="2" t="s">
-        <v>1161</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="428" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A428" s="2" t="s">
-        <v>1162</v>
+        <v>1170</v>
       </c>
       <c r="B428" s="2" t="s">
-        <v>1148</v>
+        <v>1171</v>
       </c>
       <c r="C428" s="2" t="s">
-        <v>1148</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="429" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A429" s="2" t="s">
-        <v>1163</v>
+        <v>1172</v>
       </c>
       <c r="B429" s="2" t="s">
-        <v>1164</v>
+        <v>1173</v>
       </c>
       <c r="C429" s="2" t="s">
-        <v>1165</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="430" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A430" s="2" t="s">
-        <v>1166</v>
+        <v>1174</v>
       </c>
       <c r="B430" s="2" t="s">
-        <v>1167</v>
+        <v>326</v>
       </c>
       <c r="C430" s="2" t="s">
-        <v>1168</v>
+        <v>327</v>
       </c>
     </row>
     <row r="431" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A431" s="2" t="s">
-        <v>1169</v>
+        <v>1175</v>
       </c>
       <c r="B431" s="2" t="s">
-        <v>1170</v>
+        <v>1176</v>
       </c>
       <c r="C431" s="2" t="s">
-        <v>1171</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="432" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A432" s="2" t="s">
-        <v>1172</v>
+        <v>1177</v>
       </c>
       <c r="B432" s="2" t="s">
-        <v>1173</v>
+        <v>1178</v>
       </c>
       <c r="C432" s="2" t="s">
-        <v>1174</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="433" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A433" s="2" t="s">
-        <v>1175</v>
+        <v>1179</v>
       </c>
       <c r="B433" s="2" t="s">
-        <v>1176</v>
+        <v>1180</v>
       </c>
       <c r="C433" s="2" t="s">
-        <v>1177</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="434" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A434" s="2" t="s">
-        <v>1178</v>
+        <v>1181</v>
       </c>
       <c r="B434" s="2" t="s">
-        <v>1179</v>
+        <v>1182</v>
       </c>
       <c r="C434" s="2" t="s">
-        <v>1180</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="435" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A435" s="2" t="s">
-        <v>1181</v>
+        <v>1184</v>
       </c>
       <c r="B435" s="2" t="s">
-        <v>1182</v>
+        <v>7</v>
       </c>
       <c r="C435" s="2" t="s">
-        <v>1183</v>
+        <v>8</v>
       </c>
     </row>
     <row r="436" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A436" s="2" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="B436" s="2" t="s">
-        <v>1185</v>
+        <v>1186</v>
       </c>
       <c r="C436" s="2" t="s">
         <v>1186</v>
@@ -9177,117 +9267,117 @@
         <v>1188</v>
       </c>
       <c r="C437" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="438" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A438" s="2" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="B438" s="2" t="s">
-        <v>1139</v>
+        <v>329</v>
       </c>
       <c r="C438" s="2" t="s">
-        <v>1139</v>
+        <v>330</v>
       </c>
     </row>
     <row r="439" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A439" s="2" t="s">
+        <v>1190</v>
+      </c>
+      <c r="B439" s="2" t="s">
         <v>1191</v>
       </c>
-      <c r="B439" s="2" t="s">
-        <v>1192</v>
-      </c>
       <c r="C439" s="2" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="440" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A440" s="2" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="B440" s="2" t="s">
-        <v>1194</v>
+        <v>1178</v>
       </c>
       <c r="C440" s="2" t="s">
-        <v>1195</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="441" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A441" s="2" t="s">
-        <v>1196</v>
+        <v>1193</v>
       </c>
       <c r="B441" s="2" t="s">
-        <v>1197</v>
+        <v>1194</v>
       </c>
       <c r="C441" s="2" t="s">
-        <v>1198</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="442" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A442" s="2" t="s">
-        <v>1199</v>
+        <v>1196</v>
       </c>
       <c r="B442" s="2" t="s">
-        <v>1200</v>
+        <v>1197</v>
       </c>
       <c r="C442" s="2" t="s">
-        <v>1201</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="443" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A443" s="2" t="s">
-        <v>1202</v>
+        <v>1199</v>
       </c>
       <c r="B443" s="2" t="s">
-        <v>1203</v>
+        <v>1200</v>
       </c>
       <c r="C443" s="2" t="s">
-        <v>1204</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="444" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A444" s="2" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="B444" s="2" t="s">
-        <v>1206</v>
+        <v>1203</v>
       </c>
       <c r="C444" s="2" t="s">
-        <v>1207</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="445" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A445" s="2" t="s">
-        <v>1208</v>
+        <v>1205</v>
       </c>
       <c r="B445" s="2" t="s">
-        <v>1209</v>
+        <v>1206</v>
       </c>
       <c r="C445" s="2" t="s">
-        <v>1210</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="446" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A446" s="2" t="s">
-        <v>1211</v>
+        <v>1208</v>
       </c>
       <c r="B446" s="2" t="s">
-        <v>1212</v>
+        <v>1209</v>
       </c>
       <c r="C446" s="2" t="s">
-        <v>1212</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="447" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A447" s="2" t="s">
+        <v>1211</v>
+      </c>
+      <c r="B447" s="2" t="s">
+        <v>1212</v>
+      </c>
+      <c r="C447" s="2" t="s">
         <v>1213</v>
-      </c>
-      <c r="B447" s="2" t="s">
-        <v>1146</v>
-      </c>
-      <c r="C447" s="2" t="s">
-        <v>1146</v>
       </c>
     </row>
     <row r="448" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9295,150 +9385,150 @@
         <v>1214</v>
       </c>
       <c r="B448" s="2" t="s">
-        <v>323</v>
+        <v>1215</v>
       </c>
       <c r="C448" s="2" t="s">
-        <v>324</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="449" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A449" s="2" t="s">
-        <v>1215</v>
+        <v>1217</v>
       </c>
       <c r="B449" s="2" t="s">
-        <v>1216</v>
+        <v>1218</v>
       </c>
       <c r="C449" s="2" t="s">
-        <v>1216</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="450" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A450" s="2" t="s">
-        <v>1217</v>
+        <v>1220</v>
       </c>
       <c r="B450" s="2" t="s">
-        <v>1146</v>
+        <v>1169</v>
       </c>
       <c r="C450" s="2" t="s">
-        <v>1146</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="451" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A451" s="2" t="s">
-        <v>1218</v>
+        <v>1221</v>
       </c>
       <c r="B451" s="2" t="s">
-        <v>1219</v>
+        <v>1222</v>
       </c>
       <c r="C451" s="2" t="s">
-        <v>1220</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="452" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A452" s="2" t="s">
-        <v>1221</v>
+        <v>1223</v>
       </c>
       <c r="B452" s="2" t="s">
-        <v>1212</v>
+        <v>1224</v>
       </c>
       <c r="C452" s="2" t="s">
-        <v>1212</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="453" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A453" s="2" t="s">
-        <v>1222</v>
+        <v>1226</v>
       </c>
       <c r="B453" s="2" t="s">
-        <v>7</v>
+        <v>1227</v>
       </c>
       <c r="C453" s="2" t="s">
-        <v>8</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="454" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A454" s="2" t="s">
-        <v>1223</v>
+        <v>1229</v>
       </c>
       <c r="B454" s="2" t="s">
-        <v>1224</v>
+        <v>1230</v>
       </c>
       <c r="C454" s="2" t="s">
-        <v>1225</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="455" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A455" s="2" t="s">
-        <v>1226</v>
+        <v>1232</v>
       </c>
       <c r="B455" s="2" t="s">
-        <v>1227</v>
+        <v>1233</v>
       </c>
       <c r="C455" s="2" t="s">
-        <v>1228</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="456" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A456" s="2" t="s">
-        <v>1229</v>
+        <v>1235</v>
       </c>
       <c r="B456" s="2" t="s">
-        <v>1230</v>
+        <v>1236</v>
       </c>
       <c r="C456" s="2" t="s">
-        <v>1231</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="457" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A457" s="2" t="s">
-        <v>1232</v>
+        <v>1238</v>
       </c>
       <c r="B457" s="2" t="s">
-        <v>1233</v>
+        <v>1239</v>
       </c>
       <c r="C457" s="2" t="s">
-        <v>1234</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="458" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A458" s="2" t="s">
-        <v>1235</v>
+        <v>1241</v>
       </c>
       <c r="B458" s="2" t="s">
-        <v>1236</v>
+        <v>1242</v>
       </c>
       <c r="C458" s="2" t="s">
-        <v>1237</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="459" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A459" s="2" t="s">
-        <v>1238</v>
+        <v>1243</v>
       </c>
       <c r="B459" s="2" t="s">
-        <v>1239</v>
+        <v>1176</v>
       </c>
       <c r="C459" s="2" t="s">
-        <v>1240</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="460" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A460" s="2" t="s">
-        <v>1241</v>
+        <v>1244</v>
       </c>
       <c r="B460" s="2" t="s">
-        <v>1242</v>
+        <v>326</v>
       </c>
       <c r="C460" s="2" t="s">
-        <v>1243</v>
+        <v>327</v>
       </c>
     </row>
     <row r="461" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A461" s="2" t="s">
-        <v>1244</v>
+        <v>1245</v>
       </c>
       <c r="B461" s="2" t="s">
-        <v>1245</v>
+        <v>1246</v>
       </c>
       <c r="C461" s="2" t="s">
         <v>1246</v>
@@ -9449,274 +9539,274 @@
         <v>1247</v>
       </c>
       <c r="B462" s="2" t="s">
-        <v>1248</v>
+        <v>1176</v>
       </c>
       <c r="C462" s="2" t="s">
-        <v>1248</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="463" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A463" s="2" t="s">
+        <v>1248</v>
+      </c>
+      <c r="B463" s="2" t="s">
         <v>1249</v>
       </c>
-      <c r="B463" s="2" t="s">
+      <c r="C463" s="2" t="s">
         <v>1250</v>
-      </c>
-      <c r="C463" s="2" t="s">
-        <v>1251</v>
       </c>
     </row>
     <row r="464" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A464" s="2" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
       <c r="B464" s="2" t="s">
-        <v>1253</v>
+        <v>1242</v>
       </c>
       <c r="C464" s="2" t="s">
-        <v>1254</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="465" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A465" s="2" t="s">
-        <v>1255</v>
+        <v>1252</v>
       </c>
       <c r="B465" s="2" t="s">
-        <v>1256</v>
+        <v>7</v>
       </c>
       <c r="C465" s="2" t="s">
-        <v>1257</v>
+        <v>8</v>
       </c>
     </row>
     <row r="466" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A466" s="2" t="s">
-        <v>1258</v>
+        <v>1253</v>
       </c>
       <c r="B466" s="2" t="s">
-        <v>1259</v>
+        <v>1254</v>
       </c>
       <c r="C466" s="2" t="s">
-        <v>1260</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="467" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A467" s="2" t="s">
-        <v>1261</v>
+        <v>1256</v>
       </c>
       <c r="B467" s="2" t="s">
-        <v>1262</v>
+        <v>1257</v>
       </c>
       <c r="C467" s="2" t="s">
-        <v>1263</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="468" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A468" s="2" t="s">
-        <v>1264</v>
+        <v>1259</v>
       </c>
       <c r="B468" s="2" t="s">
-        <v>1265</v>
+        <v>1260</v>
       </c>
       <c r="C468" s="2" t="s">
-        <v>1266</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="469" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A469" s="2" t="s">
-        <v>1267</v>
+        <v>1262</v>
       </c>
       <c r="B469" s="2" t="s">
-        <v>1268</v>
+        <v>1263</v>
       </c>
       <c r="C469" s="2" t="s">
-        <v>1269</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="470" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A470" s="2" t="s">
-        <v>1270</v>
+        <v>1265</v>
       </c>
       <c r="B470" s="2" t="s">
-        <v>1271</v>
+        <v>1266</v>
       </c>
       <c r="C470" s="2" t="s">
-        <v>1272</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="471" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A471" s="2" t="s">
-        <v>1273</v>
+        <v>1268</v>
       </c>
       <c r="B471" s="2" t="s">
-        <v>1274</v>
+        <v>1269</v>
       </c>
       <c r="C471" s="2" t="s">
-        <v>1275</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="472" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A472" s="2" t="s">
-        <v>1276</v>
+        <v>1271</v>
       </c>
       <c r="B472" s="2" t="s">
-        <v>1277</v>
+        <v>1272</v>
       </c>
       <c r="C472" s="2" t="s">
-        <v>1278</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="473" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A473" s="2" t="s">
-        <v>1279</v>
+        <v>1274</v>
       </c>
       <c r="B473" s="2" t="s">
-        <v>1280</v>
+        <v>1275</v>
       </c>
       <c r="C473" s="2" t="s">
-        <v>1281</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="474" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A474" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="B474" s="2" t="s">
-        <v>1283</v>
+        <v>1278</v>
       </c>
       <c r="C474" s="2" t="s">
-        <v>1284</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="475" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A475" s="2" t="s">
-        <v>1285</v>
+        <v>1279</v>
       </c>
       <c r="B475" s="2" t="s">
-        <v>1286</v>
+        <v>1280</v>
       </c>
       <c r="C475" s="2" t="s">
-        <v>1287</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="476" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A476" s="2" t="s">
-        <v>1288</v>
+        <v>1282</v>
       </c>
       <c r="B476" s="2" t="s">
-        <v>1289</v>
+        <v>1283</v>
       </c>
       <c r="C476" s="2" t="s">
-        <v>1290</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="477" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A477" s="2" t="s">
-        <v>1291</v>
+        <v>1285</v>
       </c>
       <c r="B477" s="2" t="s">
-        <v>1292</v>
+        <v>1286</v>
       </c>
       <c r="C477" s="2" t="s">
-        <v>1293</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="478" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A478" s="2" t="s">
-        <v>1294</v>
+        <v>1288</v>
       </c>
       <c r="B478" s="2" t="s">
-        <v>1295</v>
+        <v>1289</v>
       </c>
       <c r="C478" s="2" t="s">
-        <v>1296</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="479" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A479" s="2" t="s">
-        <v>1297</v>
+        <v>1291</v>
       </c>
       <c r="B479" s="2" t="s">
-        <v>1298</v>
+        <v>1292</v>
       </c>
       <c r="C479" s="2" t="s">
-        <v>1299</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="480" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A480" s="2" t="s">
-        <v>1300</v>
+        <v>1294</v>
       </c>
       <c r="B480" s="2" t="s">
-        <v>1301</v>
+        <v>1295</v>
       </c>
       <c r="C480" s="2" t="s">
-        <v>1302</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="481" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A481" s="2" t="s">
-        <v>1303</v>
+        <v>1297</v>
       </c>
       <c r="B481" s="2" t="s">
-        <v>1304</v>
+        <v>1298</v>
       </c>
       <c r="C481" s="2" t="s">
-        <v>1305</v>
+        <v>1299</v>
       </c>
     </row>
     <row r="482" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A482" s="2" t="s">
-        <v>1306</v>
+        <v>1300</v>
       </c>
       <c r="B482" s="2" t="s">
-        <v>1307</v>
+        <v>1301</v>
       </c>
       <c r="C482" s="2" t="s">
-        <v>1308</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="483" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A483" s="2" t="s">
-        <v>1309</v>
+        <v>1303</v>
       </c>
       <c r="B483" s="2" t="s">
-        <v>1310</v>
+        <v>1304</v>
       </c>
       <c r="C483" s="2" t="s">
-        <v>1115</v>
+        <v>1305</v>
       </c>
     </row>
     <row r="484" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A484" s="2" t="s">
-        <v>1311</v>
+        <v>1306</v>
       </c>
       <c r="B484" s="2" t="s">
-        <v>1312</v>
+        <v>1307</v>
       </c>
       <c r="C484" s="2" t="s">
-        <v>1312</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="485" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A485" s="2" t="s">
-        <v>1313</v>
+        <v>1309</v>
       </c>
       <c r="B485" s="2" t="s">
-        <v>1136</v>
+        <v>1310</v>
       </c>
       <c r="C485" s="2" t="s">
-        <v>1136</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="486" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A486" s="2" t="s">
+        <v>1312</v>
+      </c>
+      <c r="B486" s="2" t="s">
+        <v>1313</v>
+      </c>
+      <c r="C486" s="2" t="s">
         <v>1314</v>
-      </c>
-      <c r="B486" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="C486" s="2" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="487" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9724,75 +9814,207 @@
         <v>1315</v>
       </c>
       <c r="B487" s="2" t="s">
-        <v>1139</v>
+        <v>1316</v>
       </c>
       <c r="C487" s="2" t="s">
-        <v>1139</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="488" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A488" s="2" t="s">
-        <v>1316</v>
+        <v>1318</v>
       </c>
       <c r="B488" s="2" t="s">
-        <v>1143</v>
+        <v>1319</v>
       </c>
       <c r="C488" s="2" t="s">
-        <v>1143</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="489" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A489" s="2" t="s">
-        <v>1317</v>
+        <v>1321</v>
       </c>
       <c r="B489" s="2" t="s">
-        <v>323</v>
+        <v>1322</v>
       </c>
       <c r="C489" s="2" t="s">
-        <v>324</v>
+        <v>1323</v>
       </c>
     </row>
     <row r="490" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A490" s="2" t="s">
-        <v>1318</v>
+        <v>1324</v>
       </c>
       <c r="B490" s="2" t="s">
-        <v>1146</v>
+        <v>1325</v>
       </c>
       <c r="C490" s="2" t="s">
-        <v>1146</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="491" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A491" s="2" t="s">
-        <v>1319</v>
+        <v>1327</v>
       </c>
       <c r="B491" s="2" t="s">
-        <v>1150</v>
+        <v>1328</v>
       </c>
       <c r="C491" s="2" t="s">
-        <v>1150</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="492" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A492" s="2" t="s">
-        <v>1320</v>
+        <v>1330</v>
       </c>
       <c r="B492" s="2" t="s">
-        <v>1152</v>
+        <v>1331</v>
       </c>
       <c r="C492" s="2" t="s">
-        <v>1153</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="493" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A493" s="2" t="s">
-        <v>1321</v>
+        <v>1333</v>
       </c>
       <c r="B493" s="2" t="s">
+        <v>1334</v>
+      </c>
+      <c r="C493" s="2" t="s">
+        <v>1335</v>
+      </c>
+    </row>
+    <row r="494" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A494" s="2" t="s">
+        <v>1336</v>
+      </c>
+      <c r="B494" s="2" t="s">
+        <v>1337</v>
+      </c>
+      <c r="C494" s="2" t="s">
+        <v>1338</v>
+      </c>
+    </row>
+    <row r="495" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A495" s="2" t="s">
+        <v>1339</v>
+      </c>
+      <c r="B495" s="2" t="s">
+        <v>1340</v>
+      </c>
+      <c r="C495" s="2" t="s">
+        <v>1145</v>
+      </c>
+    </row>
+    <row r="496" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A496" s="2" t="s">
+        <v>1341</v>
+      </c>
+      <c r="B496" s="2" t="s">
+        <v>1342</v>
+      </c>
+      <c r="C496" s="2" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="497" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A497" s="2" t="s">
+        <v>1343</v>
+      </c>
+      <c r="B497" s="2" t="s">
+        <v>1166</v>
+      </c>
+      <c r="C497" s="2" t="s">
+        <v>1166</v>
+      </c>
+    </row>
+    <row r="498" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A498" s="2" t="s">
+        <v>1344</v>
+      </c>
+      <c r="B498" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C498" s="2" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="499" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A499" s="2" t="s">
+        <v>1345</v>
+      </c>
+      <c r="B499" s="2" t="s">
+        <v>1169</v>
+      </c>
+      <c r="C499" s="2" t="s">
+        <v>1169</v>
+      </c>
+    </row>
+    <row r="500" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A500" s="2" t="s">
+        <v>1346</v>
+      </c>
+      <c r="B500" s="2" t="s">
+        <v>1173</v>
+      </c>
+      <c r="C500" s="2" t="s">
+        <v>1173</v>
+      </c>
+    </row>
+    <row r="501" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A501" s="2" t="s">
+        <v>1347</v>
+      </c>
+      <c r="B501" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C501" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="502" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A502" s="2" t="s">
+        <v>1348</v>
+      </c>
+      <c r="B502" s="2" t="s">
+        <v>1176</v>
+      </c>
+      <c r="C502" s="2" t="s">
+        <v>1176</v>
+      </c>
+    </row>
+    <row r="503" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A503" s="2" t="s">
+        <v>1349</v>
+      </c>
+      <c r="B503" s="2" t="s">
+        <v>1180</v>
+      </c>
+      <c r="C503" s="2" t="s">
+        <v>1180</v>
+      </c>
+    </row>
+    <row r="504" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A504" s="2" t="s">
+        <v>1350</v>
+      </c>
+      <c r="B504" s="2" t="s">
+        <v>1182</v>
+      </c>
+      <c r="C504" s="2" t="s">
+        <v>1183</v>
+      </c>
+    </row>
+    <row r="505" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A505" s="2" t="s">
+        <v>1351</v>
+      </c>
+      <c r="B505" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C493" s="2" t="s">
+      <c r="C505" s="2" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(portal-web): 移除首訪專案說明 dialog 與 coach 指引
刪除 OnboardingGuide（intro modal + 右上角 GitHub / 文件 coach-marks）、
App.vue 掛載與 onboarding i18n 區塊，i18n.xlsx 同步重產。

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/portal-web/i18n.xlsx
+++ b/apps/portal-web/i18n.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1518" uniqueCount="1355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="1309">
   <si>
     <t>key</t>
   </si>
@@ -553,10 +553,10 @@
     <t>market.ctaBand.sub</t>
   </si>
   <si>
-    <t>把樂譜、攝影集與電子書帶到 Open Jam——免月費開店，成功售出才收 3% 手續費。</t>
-  </si>
-  <si>
-    <t>Bring your sheet music, photography, and e-books to Open Jam — no monthly fee, just a 3% cut when a work sells.</t>
+    <t>把樂譜、攝影集與電子書帶到 Open Jam——免月費開店，成功售出才收 10% + 每筆 NT$12 手續費。</t>
+  </si>
+  <si>
+    <t>Bring your sheet music, photography, and e-books to Open Jam — no monthly fee, just 10% + NT$12 per sale when a work sells.</t>
   </si>
   <si>
     <t>market.ctaBand.button</t>
@@ -1093,19 +1093,19 @@
     <t>legal.terms.tldr.1.t</t>
   </si>
   <si>
-    <t>免月費、只抽 3%</t>
-  </si>
-  <si>
-    <t>No monthly fee, 3% cut</t>
+    <t>免月費，售出才收費</t>
+  </si>
+  <si>
+    <t>No monthly fee, pay only when you sell</t>
   </si>
   <si>
     <t>legal.terms.tldr.1.d</t>
   </si>
   <si>
-    <t>開店與上架不收費，作品售出時平台收取 3% 手續費。</t>
-  </si>
-  <si>
-    <t>Opening a shop and listing are free; we take a 3% fee only when a work sells.</t>
+    <t>開店與上架不收費，作品售出時平台收取 10% + 每筆 NT$12 手續費。</t>
+  </si>
+  <si>
+    <t>Opening a shop and listing are free; we take 10% + NT$12 per sale only when a work sells.</t>
   </si>
   <si>
     <t>legal.terms.tldr.2.t</t>
@@ -1219,10 +1219,10 @@
     <t>legal.terms.sections.3.p</t>
   </si>
   <si>
-    <t>Open Jam 採免月費制，作品成功售出後平台收取 3% 手續費。款項將依結算週期撥付至你綁定的收款帳戶。</t>
-  </si>
-  <si>
-    <t>Open Jam charges no monthly fee; once a work sells, the platform takes a 3% transaction fee. Funds are paid out to your linked payout account according to the settlement cycle.</t>
+    <t>Open Jam 採免月費制，作品成功售出後平台收取售價 10% 加每筆 NT$12 的交易手續費。款項將依結算週期撥付至你綁定的收款帳戶。</t>
+  </si>
+  <si>
+    <t>Open Jam charges no monthly fee; once a work sells, the platform takes a transaction fee of 10% of the sale price plus NT$12 per transaction. Funds are paid out to your linked payout account according to the settlement cycle.</t>
   </si>
   <si>
     <t>legal.terms.sections.4.h</t>
@@ -1531,144 +1531,6 @@
     <t>the boring pages, made friendly ♡</t>
   </si>
   <si>
-    <t>onboarding.modalAria</t>
-  </si>
-  <si>
-    <t>平台說明</t>
-  </si>
-  <si>
-    <t>Platform notice</t>
-  </si>
-  <si>
-    <t>onboarding.title</t>
-  </si>
-  <si>
-    <t>關於這個平台</t>
-  </si>
-  <si>
-    <t>About this platform</t>
-  </si>
-  <si>
-    <t>onboarding.meta</t>
-  </si>
-  <si>
-    <t>OPEN JAM · SIDE PROJECT</t>
-  </si>
-  <si>
-    <t>onboarding.closeAria</t>
-  </si>
-  <si>
-    <t>onboarding.s1.title</t>
-  </si>
-  <si>
-    <t>這是一個 Side Project</t>
-  </si>
-  <si>
-    <t>This is a side project</t>
-  </si>
-  <si>
-    <t>onboarding.s1.body</t>
-  </si>
-  <si>
-    <t>Open Jam 是個人開發的 side project，純粹作為技術測試與作品集展示之用，並非正式營運的商業平台。</t>
-  </si>
-  <si>
-    <t>Open Jam is a personal side project, built purely for technical experimentation and as a portfolio showcase — it is not a commercially operated platform.</t>
-  </si>
-  <si>
-    <t>onboarding.s2.title</t>
-  </si>
-  <si>
-    <t>金流為測試模式</t>
-  </si>
-  <si>
-    <t>Payments are in test mode</t>
-  </si>
-  <si>
-    <t>onboarding.s2.body</t>
-  </si>
-  <si>
-    <t>結帳僅串接 Stripe 金流的 {testMode}，不會產生任何真實扣款。請勿輸入真實信用卡資訊，可使用 Stripe 提供的測試卡號（例如 {card}）。</t>
-  </si>
-  <si>
-    <t>Checkout only connects to Stripe’s {testMode}, so no real charges are ever made. Please do not enter real credit card details; you can use a Stripe test card number (for example {card}).</t>
-  </si>
-  <si>
-    <t>onboarding.s2.testMode</t>
-  </si>
-  <si>
-    <t>Test Mode</t>
-  </si>
-  <si>
-    <t>onboarding.s3.title</t>
-  </si>
-  <si>
-    <t>資料僅供展示</t>
-  </si>
-  <si>
-    <t>Data is for demonstration only</t>
-  </si>
-  <si>
-    <t>onboarding.s3.body</t>
-  </si>
-  <si>
-    <t>站上的作品與資料皆為示範內容，可能隨時調整或重置，請勿用於正式交易。</t>
-  </si>
-  <si>
-    <t>The works and data on the site are sample content and may be changed or reset at any time. Please do not use it for real transactions.</t>
-  </si>
-  <si>
-    <t>onboarding.start</t>
-  </si>
-  <si>
-    <t>我知道了，開始逛逛</t>
-  </si>
-  <si>
-    <t>Got it, start browsing</t>
-  </si>
-  <si>
-    <t>onboarding.coachEyebrow</t>
-  </si>
-  <si>
-    <t>右上角工具列</t>
-  </si>
-  <si>
-    <t>Top-right toolbar</t>
-  </si>
-  <si>
-    <t>onboarding.coachGithubTitle</t>
-  </si>
-  <si>
-    <t>onboarding.coachGithubDesc</t>
-  </si>
-  <si>
-    <t>本平台完整原始碼 repository</t>
-  </si>
-  <si>
-    <t>The platform’s full source code repository</t>
-  </si>
-  <si>
-    <t>onboarding.coachDocsTitle</t>
-  </si>
-  <si>
-    <t>onboarding.coachDocsDesc</t>
-  </si>
-  <si>
-    <t>系統設計與規格說明文件</t>
-  </si>
-  <si>
-    <t>System design and specification docs</t>
-  </si>
-  <si>
-    <t>onboarding.coachDone</t>
-  </si>
-  <si>
-    <t>知道了</t>
-  </si>
-  <si>
-    <t>Got it</t>
-  </si>
-  <si>
     <t>notifications.title</t>
   </si>
   <si>
@@ -3157,10 +3019,10 @@
     <t>faq.items.13.a</t>
   </si>
   <si>
-    <t>開店與上架不收月費。只有在作品實際售出時，平台才收取少額交易手續費（3%）。</t>
-  </si>
-  <si>
-    <t>There's no monthly fee to open a shop or list works. The platform only takes a small transaction fee (3%) when a work actually sells.</t>
+    <t>開店與上架不收月費。只有在作品實際售出時，平台才收取交易手續費（售價 10% + 每筆 NT$12）。</t>
+  </si>
+  <si>
+    <t>There's no monthly fee to open a shop or list works. The platform only takes a transaction fee (10% of the sale price + NT$12 per transaction) when a work actually sells.</t>
   </si>
   <si>
     <t>faq.items.14.cat</t>
@@ -3286,10 +3148,10 @@
     <t>faq.items.19.a</t>
   </si>
   <si>
-    <t>平台不收月費，只在作品售出時收取 3% 的交易手續費。</t>
-  </si>
-  <si>
-    <t>No monthly fee — the platform only takes a 3% transaction fee when a work sells.</t>
+    <t>平台不收月費，只在作品售出時收取售價 10% 加每筆 NT$12 的交易手續費。</t>
+  </si>
+  <si>
+    <t>No monthly fee — the platform only takes 10% of the sale price plus NT$12 per transaction when a work sells.</t>
   </si>
   <si>
     <t>faq.items.20.cat</t>
@@ -4001,10 +3863,10 @@
     <t>landingPage.rules.items.2.text</t>
   </si>
   <si>
-    <t>每筆成交 97% 歸創作者，平台只收 3%，開店免月費。</t>
-  </si>
-  <si>
-    <t>97% of every sale goes to the creator. The platform takes 3%, and shops are free to open.</t>
+    <t>作品售出時平台只收 10% + 每筆 NT$12，其餘全數歸創作者，開店免月費。</t>
+  </si>
+  <si>
+    <t>When a work sells, the platform takes just 10% + NT$12 — the rest goes to the creator, and shops are free to open.</t>
   </si>
   <si>
     <t>landingPage.final.title</t>
@@ -4465,7 +4327,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C506"/>
+  <dimension ref="A1:C488"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -6460,1580 +6322,1580 @@
         <v>513</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
     </row>
     <row r="182" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>301</v>
+        <v>516</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>302</v>
+        <v>517</v>
       </c>
     </row>
     <row r="183" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
     </row>
     <row r="184" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
     </row>
     <row r="185" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
     </row>
     <row r="186" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
     </row>
     <row r="187" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
     </row>
     <row r="188" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
     </row>
     <row r="189" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
     </row>
     <row r="190" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
     </row>
     <row r="191" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
     </row>
     <row r="192" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>17</v>
+        <v>546</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>18</v>
+        <v>547</v>
       </c>
     </row>
     <row r="193" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
     </row>
     <row r="194" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>20</v>
+        <v>552</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>21</v>
+        <v>553</v>
       </c>
     </row>
     <row r="195" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
-        <v>546</v>
+        <v>554</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>547</v>
+        <v>555</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>548</v>
+        <v>556</v>
       </c>
     </row>
     <row r="196" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
-        <v>549</v>
+        <v>557</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>550</v>
+        <v>558</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>551</v>
+        <v>559</v>
       </c>
     </row>
     <row r="197" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
-        <v>552</v>
+        <v>560</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>553</v>
+        <v>561</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>554</v>
+        <v>562</v>
       </c>
     </row>
     <row r="198" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>556</v>
+        <v>564</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>557</v>
+        <v>565</v>
       </c>
     </row>
     <row r="199" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>558</v>
+        <v>566</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>559</v>
+        <v>567</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>560</v>
+        <v>568</v>
       </c>
     </row>
     <row r="200" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
-        <v>561</v>
+        <v>569</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>562</v>
+        <v>81</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>563</v>
+        <v>82</v>
       </c>
     </row>
     <row r="201" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
     </row>
     <row r="202" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>568</v>
+        <v>87</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
     </row>
     <row r="203" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
-        <v>570</v>
+        <v>575</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>571</v>
+        <v>576</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
     </row>
     <row r="204" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
-        <v>573</v>
+        <v>578</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>575</v>
+        <v>580</v>
       </c>
     </row>
     <row r="205" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>577</v>
+        <v>582</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
     </row>
     <row r="206" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
-        <v>579</v>
+        <v>584</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>580</v>
+        <v>585</v>
       </c>
       <c r="C206" s="2" t="s">
-        <v>581</v>
+        <v>586</v>
       </c>
     </row>
     <row r="207" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
-        <v>582</v>
+        <v>587</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>584</v>
+        <v>589</v>
       </c>
     </row>
     <row r="208" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
-        <v>585</v>
+        <v>590</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>586</v>
+        <v>591</v>
       </c>
       <c r="C208" s="2" t="s">
-        <v>587</v>
+        <v>592</v>
       </c>
     </row>
     <row r="209" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
-        <v>588</v>
+        <v>593</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>589</v>
+        <v>594</v>
       </c>
       <c r="C209" s="2" t="s">
-        <v>590</v>
+        <v>595</v>
       </c>
     </row>
     <row r="210" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
-        <v>591</v>
+        <v>596</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>592</v>
+        <v>597</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>593</v>
+        <v>598</v>
       </c>
     </row>
     <row r="211" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
-        <v>594</v>
+        <v>599</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>595</v>
+        <v>600</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
     </row>
     <row r="212" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>598</v>
+        <v>603</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>599</v>
+        <v>604</v>
       </c>
     </row>
     <row r="213" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
-        <v>600</v>
+        <v>605</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>601</v>
+        <v>606</v>
       </c>
       <c r="C213" s="2" t="s">
-        <v>602</v>
+        <v>607</v>
       </c>
     </row>
     <row r="214" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
-        <v>603</v>
+        <v>608</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>604</v>
+        <v>609</v>
       </c>
       <c r="C214" s="2" t="s">
-        <v>605</v>
+        <v>610</v>
       </c>
     </row>
     <row r="215" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A215" s="2" t="s">
-        <v>606</v>
+        <v>611</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>607</v>
+        <v>612</v>
       </c>
       <c r="C215" s="2" t="s">
-        <v>608</v>
+        <v>613</v>
       </c>
     </row>
     <row r="216" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A216" s="2" t="s">
-        <v>609</v>
+        <v>614</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>610</v>
+        <v>615</v>
       </c>
       <c r="C216" s="2" t="s">
-        <v>611</v>
+        <v>616</v>
       </c>
     </row>
     <row r="217" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A217" s="2" t="s">
-        <v>612</v>
+        <v>617</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>613</v>
+        <v>618</v>
       </c>
       <c r="C217" s="2" t="s">
-        <v>614</v>
+        <v>619</v>
       </c>
     </row>
     <row r="218" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A218" s="2" t="s">
-        <v>615</v>
+        <v>620</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>81</v>
+        <v>621</v>
       </c>
       <c r="C218" s="2" t="s">
-        <v>82</v>
+        <v>622</v>
       </c>
     </row>
     <row r="219" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
-        <v>616</v>
+        <v>623</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>617</v>
+        <v>624</v>
       </c>
       <c r="C219" s="2" t="s">
-        <v>618</v>
+        <v>67</v>
       </c>
     </row>
     <row r="220" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A220" s="2" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>87</v>
+        <v>626</v>
       </c>
       <c r="C220" s="2" t="s">
-        <v>620</v>
+        <v>627</v>
       </c>
     </row>
     <row r="221" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A221" s="2" t="s">
-        <v>621</v>
+        <v>628</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>622</v>
+        <v>629</v>
       </c>
       <c r="C221" s="2" t="s">
-        <v>623</v>
+        <v>630</v>
       </c>
     </row>
     <row r="222" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A222" s="2" t="s">
-        <v>624</v>
+        <v>631</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>625</v>
+        <v>632</v>
       </c>
       <c r="C222" s="2" t="s">
-        <v>626</v>
+        <v>633</v>
       </c>
     </row>
     <row r="223" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A223" s="2" t="s">
-        <v>627</v>
+        <v>634</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>628</v>
+        <v>635</v>
       </c>
       <c r="C223" s="2" t="s">
-        <v>629</v>
+        <v>636</v>
       </c>
     </row>
     <row r="224" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A224" s="2" t="s">
-        <v>630</v>
+        <v>637</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>631</v>
+        <v>638</v>
       </c>
       <c r="C224" s="2" t="s">
-        <v>632</v>
+        <v>639</v>
       </c>
     </row>
     <row r="225" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A225" s="2" t="s">
-        <v>633</v>
+        <v>640</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>634</v>
+        <v>641</v>
       </c>
       <c r="C225" s="2" t="s">
-        <v>635</v>
+        <v>642</v>
       </c>
     </row>
     <row r="226" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A226" s="2" t="s">
-        <v>636</v>
+        <v>643</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>637</v>
+        <v>99</v>
       </c>
       <c r="C226" s="2" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
     </row>
     <row r="227" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A227" s="2" t="s">
-        <v>639</v>
+        <v>645</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
       <c r="C227" s="2" t="s">
-        <v>641</v>
+        <v>647</v>
       </c>
     </row>
     <row r="228" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A228" s="2" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
       <c r="C228" s="2" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
     </row>
     <row r="229" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A229" s="2" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
       <c r="B229" s="2" t="s">
-        <v>646</v>
+        <v>652</v>
       </c>
       <c r="C229" s="2" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
     </row>
     <row r="230" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A230" s="2" t="s">
-        <v>648</v>
+        <v>654</v>
       </c>
       <c r="B230" s="2" t="s">
-        <v>649</v>
+        <v>655</v>
       </c>
       <c r="C230" s="2" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
     </row>
     <row r="231" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A231" s="2" t="s">
-        <v>651</v>
+        <v>657</v>
       </c>
       <c r="B231" s="2" t="s">
-        <v>652</v>
+        <v>658</v>
       </c>
       <c r="C231" s="2" t="s">
-        <v>653</v>
+        <v>659</v>
       </c>
     </row>
     <row r="232" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A232" s="2" t="s">
-        <v>654</v>
+        <v>660</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
       <c r="C232" s="2" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
     </row>
     <row r="233" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A233" s="2" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
       <c r="C233" s="2" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
     </row>
     <row r="234" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A234" s="2" t="s">
-        <v>660</v>
+        <v>666</v>
       </c>
       <c r="B234" s="2" t="s">
-        <v>661</v>
+        <v>667</v>
       </c>
       <c r="C234" s="2" t="s">
-        <v>662</v>
+        <v>668</v>
       </c>
     </row>
     <row r="235" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A235" s="2" t="s">
-        <v>663</v>
+        <v>669</v>
       </c>
       <c r="B235" s="2" t="s">
-        <v>664</v>
+        <v>670</v>
       </c>
       <c r="C235" s="2" t="s">
-        <v>665</v>
+        <v>671</v>
       </c>
     </row>
     <row r="236" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A236" s="2" t="s">
-        <v>666</v>
+        <v>672</v>
       </c>
       <c r="B236" s="2" t="s">
-        <v>667</v>
+        <v>673</v>
       </c>
       <c r="C236" s="2" t="s">
-        <v>668</v>
+        <v>674</v>
       </c>
     </row>
     <row r="237" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A237" s="2" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="B237" s="2" t="s">
-        <v>670</v>
+        <v>676</v>
       </c>
       <c r="C237" s="2" t="s">
-        <v>67</v>
+        <v>677</v>
       </c>
     </row>
     <row r="238" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A238" s="2" t="s">
-        <v>671</v>
+        <v>678</v>
       </c>
       <c r="B238" s="2" t="s">
-        <v>672</v>
+        <v>679</v>
       </c>
       <c r="C238" s="2" t="s">
-        <v>673</v>
+        <v>680</v>
       </c>
     </row>
     <row r="239" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A239" s="2" t="s">
-        <v>674</v>
+        <v>681</v>
       </c>
       <c r="B239" s="2" t="s">
-        <v>675</v>
+        <v>682</v>
       </c>
       <c r="C239" s="2" t="s">
-        <v>676</v>
+        <v>683</v>
       </c>
     </row>
     <row r="240" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A240" s="2" t="s">
-        <v>677</v>
+        <v>684</v>
       </c>
       <c r="B240" s="2" t="s">
-        <v>678</v>
+        <v>685</v>
       </c>
       <c r="C240" s="2" t="s">
-        <v>679</v>
+        <v>686</v>
       </c>
     </row>
     <row r="241" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A241" s="2" t="s">
-        <v>680</v>
+        <v>687</v>
       </c>
       <c r="B241" s="2" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="C241" s="2" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
     </row>
     <row r="242" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A242" s="2" t="s">
-        <v>683</v>
+        <v>690</v>
       </c>
       <c r="B242" s="2" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
       <c r="C242" s="2" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
     </row>
     <row r="243" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A243" s="2" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
       <c r="B243" s="2" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="C243" s="2" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
     </row>
     <row r="244" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A244" s="2" t="s">
-        <v>689</v>
+        <v>696</v>
       </c>
       <c r="B244" s="2" t="s">
-        <v>99</v>
+        <v>697</v>
       </c>
       <c r="C244" s="2" t="s">
-        <v>690</v>
+        <v>698</v>
       </c>
     </row>
     <row r="245" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A245" s="2" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B245" s="2" t="s">
-        <v>692</v>
+        <v>700</v>
       </c>
       <c r="C245" s="2" t="s">
-        <v>693</v>
+        <v>701</v>
       </c>
     </row>
     <row r="246" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A246" s="2" t="s">
-        <v>694</v>
+        <v>702</v>
       </c>
       <c r="B246" s="2" t="s">
-        <v>695</v>
+        <v>703</v>
       </c>
       <c r="C246" s="2" t="s">
-        <v>696</v>
+        <v>704</v>
       </c>
     </row>
     <row r="247" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A247" s="2" t="s">
-        <v>697</v>
+        <v>705</v>
       </c>
       <c r="B247" s="2" t="s">
-        <v>698</v>
+        <v>706</v>
       </c>
       <c r="C247" s="2" t="s">
-        <v>699</v>
+        <v>707</v>
       </c>
     </row>
     <row r="248" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A248" s="2" t="s">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="B248" s="2" t="s">
-        <v>701</v>
+        <v>709</v>
       </c>
       <c r="C248" s="2" t="s">
-        <v>702</v>
+        <v>710</v>
       </c>
     </row>
     <row r="249" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A249" s="2" t="s">
-        <v>703</v>
+        <v>711</v>
       </c>
       <c r="B249" s="2" t="s">
-        <v>704</v>
+        <v>712</v>
       </c>
       <c r="C249" s="2" t="s">
-        <v>705</v>
+        <v>713</v>
       </c>
     </row>
     <row r="250" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A250" s="2" t="s">
-        <v>706</v>
+        <v>714</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>707</v>
+        <v>715</v>
       </c>
       <c r="C250" s="2" t="s">
-        <v>708</v>
+        <v>716</v>
       </c>
     </row>
     <row r="251" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A251" s="2" t="s">
-        <v>709</v>
+        <v>717</v>
       </c>
       <c r="B251" s="2" t="s">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="C251" s="2" t="s">
-        <v>711</v>
+        <v>719</v>
       </c>
     </row>
     <row r="252" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A252" s="2" t="s">
-        <v>712</v>
+        <v>720</v>
       </c>
       <c r="B252" s="2" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="C252" s="2" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
     </row>
     <row r="253" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A253" s="2" t="s">
-        <v>715</v>
+        <v>723</v>
       </c>
       <c r="B253" s="2" t="s">
-        <v>716</v>
+        <v>724</v>
       </c>
       <c r="C253" s="2" t="s">
-        <v>717</v>
+        <v>725</v>
       </c>
     </row>
     <row r="254" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A254" s="2" t="s">
-        <v>718</v>
+        <v>726</v>
       </c>
       <c r="B254" s="2" t="s">
-        <v>719</v>
+        <v>727</v>
       </c>
       <c r="C254" s="2" t="s">
-        <v>720</v>
+        <v>728</v>
       </c>
     </row>
     <row r="255" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A255" s="2" t="s">
-        <v>721</v>
+        <v>729</v>
       </c>
       <c r="B255" s="2" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="C255" s="2" t="s">
-        <v>723</v>
+        <v>731</v>
       </c>
     </row>
     <row r="256" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A256" s="2" t="s">
-        <v>724</v>
+        <v>732</v>
       </c>
       <c r="B256" s="2" t="s">
-        <v>725</v>
+        <v>733</v>
       </c>
       <c r="C256" s="2" t="s">
-        <v>726</v>
+        <v>734</v>
       </c>
     </row>
     <row r="257" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A257" s="2" t="s">
-        <v>727</v>
+        <v>735</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>728</v>
+        <v>736</v>
       </c>
       <c r="C257" s="2" t="s">
-        <v>729</v>
+        <v>737</v>
       </c>
     </row>
     <row r="258" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A258" s="2" t="s">
-        <v>730</v>
+        <v>738</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>731</v>
+        <v>652</v>
       </c>
       <c r="C258" s="2" t="s">
-        <v>732</v>
+        <v>739</v>
       </c>
     </row>
     <row r="259" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A259" s="2" t="s">
-        <v>733</v>
+        <v>740</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>734</v>
+        <v>655</v>
       </c>
       <c r="C259" s="2" t="s">
-        <v>735</v>
+        <v>741</v>
       </c>
     </row>
     <row r="260" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A260" s="2" t="s">
-        <v>736</v>
+        <v>742</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>737</v>
+        <v>658</v>
       </c>
       <c r="C260" s="2" t="s">
-        <v>738</v>
+        <v>658</v>
       </c>
     </row>
     <row r="261" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A261" s="2" t="s">
-        <v>739</v>
+        <v>743</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>740</v>
+        <v>661</v>
       </c>
       <c r="C261" s="2" t="s">
-        <v>741</v>
+        <v>661</v>
       </c>
     </row>
     <row r="262" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A262" s="2" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="C262" s="2" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
     </row>
     <row r="263" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A263" s="2" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="C263" s="2" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
     </row>
     <row r="264" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A264" s="2" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="C264" s="2" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
     </row>
     <row r="265" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A265" s="2" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="B265" s="2" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="C265" s="2" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
     </row>
     <row r="266" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A266" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="B266" s="2" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="C266" s="2" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
     </row>
     <row r="267" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A267" s="2" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="C267" s="2" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
     </row>
     <row r="268" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A268" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="C268" s="2" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
     </row>
     <row r="269" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A269" s="2" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
       <c r="B269" s="2" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="C269" s="2" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
     </row>
     <row r="270" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A270" s="2" t="s">
-        <v>766</v>
+        <v>768</v>
       </c>
       <c r="B270" s="2" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="C270" s="2" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
     </row>
     <row r="271" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A271" s="2" t="s">
-        <v>769</v>
+        <v>771</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="C271" s="2" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
     </row>
     <row r="272" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A272" s="2" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
       <c r="B272" s="2" t="s">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="C272" s="2" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
     </row>
     <row r="273" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A273" s="2" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>776</v>
+        <v>778</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
     </row>
     <row r="274" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A274" s="2" t="s">
-        <v>778</v>
+        <v>780</v>
       </c>
       <c r="B274" s="2" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
     </row>
     <row r="275" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A275" s="2" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>783</v>
+        <v>785</v>
       </c>
     </row>
     <row r="276" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A276" s="2" t="s">
-        <v>784</v>
+        <v>786</v>
       </c>
       <c r="B276" s="2" t="s">
-        <v>698</v>
+        <v>787</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>785</v>
+        <v>788</v>
       </c>
     </row>
     <row r="277" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A277" s="2" t="s">
-        <v>786</v>
+        <v>789</v>
       </c>
       <c r="B277" s="2" t="s">
-        <v>701</v>
+        <v>790</v>
       </c>
       <c r="C277" s="2" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
     </row>
     <row r="278" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A278" s="2" t="s">
-        <v>788</v>
+        <v>792</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>704</v>
+        <v>793</v>
       </c>
       <c r="C278" s="2" t="s">
-        <v>704</v>
+        <v>794</v>
       </c>
     </row>
     <row r="279" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A279" s="2" t="s">
-        <v>789</v>
+        <v>795</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>707</v>
+        <v>796</v>
       </c>
       <c r="C279" s="2" t="s">
-        <v>707</v>
+        <v>797</v>
       </c>
     </row>
     <row r="280" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A280" s="2" t="s">
-        <v>790</v>
+        <v>798</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>791</v>
+        <v>799</v>
       </c>
       <c r="C280" s="2" t="s">
-        <v>792</v>
+        <v>800</v>
       </c>
     </row>
     <row r="281" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A281" s="2" t="s">
-        <v>793</v>
+        <v>801</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="C281" s="2" t="s">
-        <v>795</v>
+        <v>802</v>
       </c>
     </row>
     <row r="282" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A282" s="2" t="s">
-        <v>796</v>
+        <v>803</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>797</v>
+        <v>87</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>798</v>
+        <v>804</v>
       </c>
     </row>
     <row r="283" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A283" s="2" t="s">
-        <v>799</v>
+        <v>805</v>
       </c>
       <c r="B283" s="2" t="s">
-        <v>800</v>
+        <v>576</v>
       </c>
       <c r="C283" s="2" t="s">
-        <v>801</v>
+        <v>806</v>
       </c>
     </row>
     <row r="284" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A284" s="2" t="s">
-        <v>802</v>
+        <v>807</v>
       </c>
       <c r="B284" s="2" t="s">
-        <v>803</v>
+        <v>579</v>
       </c>
       <c r="C284" s="2" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
     </row>
     <row r="285" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A285" s="2" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
       <c r="B285" s="2" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
       <c r="C285" s="2" t="s">
-        <v>807</v>
+        <v>811</v>
       </c>
     </row>
     <row r="286" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A286" s="2" t="s">
-        <v>808</v>
+        <v>812</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>809</v>
+        <v>813</v>
       </c>
       <c r="C286" s="2" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
     </row>
     <row r="287" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A287" s="2" t="s">
-        <v>811</v>
+        <v>815</v>
       </c>
       <c r="B287" s="2" t="s">
-        <v>812</v>
+        <v>60</v>
       </c>
       <c r="C287" s="2" t="s">
-        <v>813</v>
+        <v>61</v>
       </c>
     </row>
     <row r="288" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A288" s="2" t="s">
-        <v>814</v>
+        <v>816</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>815</v>
+        <v>817</v>
       </c>
       <c r="C288" s="2" t="s">
-        <v>816</v>
+        <v>818</v>
       </c>
     </row>
     <row r="289" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A289" s="2" t="s">
-        <v>817</v>
+        <v>819</v>
       </c>
       <c r="B289" s="2" t="s">
-        <v>818</v>
+        <v>820</v>
       </c>
       <c r="C289" s="2" t="s">
-        <v>819</v>
+        <v>821</v>
       </c>
     </row>
     <row r="290" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A290" s="2" t="s">
-        <v>820</v>
+        <v>822</v>
       </c>
       <c r="B290" s="2" t="s">
-        <v>821</v>
+        <v>823</v>
       </c>
       <c r="C290" s="2" t="s">
-        <v>822</v>
+        <v>824</v>
       </c>
     </row>
     <row r="291" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A291" s="2" t="s">
-        <v>823</v>
+        <v>825</v>
       </c>
       <c r="B291" s="2" t="s">
-        <v>824</v>
+        <v>826</v>
       </c>
       <c r="C291" s="2" t="s">
-        <v>825</v>
+        <v>827</v>
       </c>
     </row>
     <row r="292" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A292" s="2" t="s">
-        <v>826</v>
+        <v>828</v>
       </c>
       <c r="B292" s="2" t="s">
-        <v>827</v>
+        <v>829</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>828</v>
+        <v>830</v>
       </c>
     </row>
     <row r="293" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A293" s="2" t="s">
-        <v>829</v>
+        <v>831</v>
       </c>
       <c r="B293" s="2" t="s">
-        <v>830</v>
+        <v>832</v>
       </c>
       <c r="C293" s="2" t="s">
-        <v>831</v>
+        <v>833</v>
       </c>
     </row>
     <row r="294" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A294" s="2" t="s">
-        <v>832</v>
+        <v>834</v>
       </c>
       <c r="B294" s="2" t="s">
-        <v>833</v>
+        <v>835</v>
       </c>
       <c r="C294" s="2" t="s">
-        <v>834</v>
+        <v>836</v>
       </c>
     </row>
     <row r="295" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A295" s="2" t="s">
-        <v>835</v>
+        <v>837</v>
       </c>
       <c r="B295" s="2" t="s">
-        <v>836</v>
+        <v>838</v>
       </c>
       <c r="C295" s="2" t="s">
-        <v>837</v>
+        <v>839</v>
       </c>
     </row>
     <row r="296" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A296" s="2" t="s">
-        <v>838</v>
+        <v>840</v>
       </c>
       <c r="B296" s="2" t="s">
-        <v>839</v>
+        <v>841</v>
       </c>
       <c r="C296" s="2" t="s">
-        <v>840</v>
+        <v>842</v>
       </c>
     </row>
     <row r="297" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A297" s="2" t="s">
-        <v>841</v>
+        <v>843</v>
       </c>
       <c r="B297" s="2" t="s">
-        <v>842</v>
+        <v>844</v>
       </c>
       <c r="C297" s="2" t="s">
-        <v>843</v>
+        <v>845</v>
       </c>
     </row>
     <row r="298" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A298" s="2" t="s">
-        <v>844</v>
+        <v>846</v>
       </c>
       <c r="B298" s="2" t="s">
-        <v>845</v>
+        <v>847</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>846</v>
+        <v>848</v>
       </c>
     </row>
     <row r="299" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A299" s="2" t="s">
-        <v>847</v>
+        <v>849</v>
       </c>
       <c r="B299" s="2" t="s">
-        <v>848</v>
+        <v>850</v>
       </c>
       <c r="C299" s="2" t="s">
-        <v>848</v>
+        <v>851</v>
       </c>
     </row>
     <row r="300" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A300" s="2" t="s">
-        <v>849</v>
+        <v>852</v>
       </c>
       <c r="B300" s="2" t="s">
-        <v>87</v>
+        <v>853</v>
       </c>
       <c r="C300" s="2" t="s">
-        <v>850</v>
+        <v>854</v>
       </c>
     </row>
     <row r="301" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A301" s="2" t="s">
-        <v>851</v>
+        <v>855</v>
       </c>
       <c r="B301" s="2" t="s">
-        <v>622</v>
+        <v>856</v>
       </c>
       <c r="C301" s="2" t="s">
-        <v>852</v>
+        <v>857</v>
       </c>
     </row>
     <row r="302" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A302" s="2" t="s">
-        <v>853</v>
+        <v>858</v>
       </c>
       <c r="B302" s="2" t="s">
-        <v>625</v>
+        <v>859</v>
       </c>
       <c r="C302" s="2" t="s">
-        <v>854</v>
+        <v>860</v>
       </c>
     </row>
     <row r="303" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A303" s="2" t="s">
-        <v>855</v>
+        <v>861</v>
       </c>
       <c r="B303" s="2" t="s">
-        <v>856</v>
+        <v>862</v>
       </c>
       <c r="C303" s="2" t="s">
-        <v>857</v>
+        <v>863</v>
       </c>
     </row>
     <row r="304" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A304" s="2" t="s">
-        <v>858</v>
+        <v>864</v>
       </c>
       <c r="B304" s="2" t="s">
-        <v>859</v>
+        <v>865</v>
       </c>
       <c r="C304" s="2" t="s">
-        <v>860</v>
+        <v>866</v>
       </c>
     </row>
     <row r="305" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A305" s="2" t="s">
-        <v>861</v>
+        <v>867</v>
       </c>
       <c r="B305" s="2" t="s">
-        <v>60</v>
+        <v>868</v>
       </c>
       <c r="C305" s="2" t="s">
-        <v>61</v>
+        <v>869</v>
       </c>
     </row>
     <row r="306" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A306" s="2" t="s">
-        <v>862</v>
+        <v>870</v>
       </c>
       <c r="B306" s="2" t="s">
-        <v>863</v>
+        <v>871</v>
       </c>
       <c r="C306" s="2" t="s">
-        <v>864</v>
+        <v>872</v>
       </c>
     </row>
     <row r="307" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A307" s="2" t="s">
-        <v>865</v>
+        <v>873</v>
       </c>
       <c r="B307" s="2" t="s">
-        <v>866</v>
+        <v>874</v>
       </c>
       <c r="C307" s="2" t="s">
-        <v>867</v>
+        <v>875</v>
       </c>
     </row>
     <row r="308" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A308" s="2" t="s">
-        <v>868</v>
+        <v>876</v>
       </c>
       <c r="B308" s="2" t="s">
-        <v>869</v>
+        <v>877</v>
       </c>
       <c r="C308" s="2" t="s">
-        <v>870</v>
+        <v>878</v>
       </c>
     </row>
     <row r="309" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A309" s="2" t="s">
-        <v>871</v>
+        <v>879</v>
       </c>
       <c r="B309" s="2" t="s">
-        <v>872</v>
+        <v>880</v>
       </c>
       <c r="C309" s="2" t="s">
-        <v>873</v>
+        <v>881</v>
       </c>
     </row>
     <row r="310" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A310" s="2" t="s">
-        <v>874</v>
+        <v>882</v>
       </c>
       <c r="B310" s="2" t="s">
-        <v>875</v>
+        <v>883</v>
       </c>
       <c r="C310" s="2" t="s">
-        <v>876</v>
+        <v>884</v>
       </c>
     </row>
     <row r="311" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A311" s="2" t="s">
-        <v>877</v>
+        <v>885</v>
       </c>
       <c r="B311" s="2" t="s">
-        <v>878</v>
+        <v>886</v>
       </c>
       <c r="C311" s="2" t="s">
-        <v>879</v>
+        <v>887</v>
       </c>
     </row>
     <row r="312" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A312" s="2" t="s">
-        <v>880</v>
+        <v>888</v>
       </c>
       <c r="B312" s="2" t="s">
-        <v>881</v>
+        <v>889</v>
       </c>
       <c r="C312" s="2" t="s">
-        <v>882</v>
+        <v>890</v>
       </c>
     </row>
     <row r="313" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A313" s="2" t="s">
-        <v>883</v>
+        <v>891</v>
       </c>
       <c r="B313" s="2" t="s">
-        <v>884</v>
+        <v>892</v>
       </c>
       <c r="C313" s="2" t="s">
-        <v>885</v>
+        <v>893</v>
       </c>
     </row>
     <row r="314" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A314" s="2" t="s">
-        <v>886</v>
+        <v>894</v>
       </c>
       <c r="B314" s="2" t="s">
-        <v>887</v>
+        <v>496</v>
       </c>
       <c r="C314" s="2" t="s">
-        <v>888</v>
+        <v>497</v>
       </c>
     </row>
     <row r="315" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A315" s="2" t="s">
-        <v>889</v>
+        <v>895</v>
       </c>
       <c r="B315" s="2" t="s">
-        <v>890</v>
+        <v>896</v>
       </c>
       <c r="C315" s="2" t="s">
-        <v>891</v>
+        <v>897</v>
       </c>
     </row>
     <row r="316" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A316" s="2" t="s">
-        <v>892</v>
+        <v>898</v>
       </c>
       <c r="B316" s="2" t="s">
-        <v>893</v>
+        <v>899</v>
       </c>
       <c r="C316" s="2" t="s">
-        <v>894</v>
+        <v>900</v>
       </c>
     </row>
     <row r="317" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A317" s="2" t="s">
-        <v>895</v>
+        <v>901</v>
       </c>
       <c r="B317" s="2" t="s">
-        <v>896</v>
+        <v>902</v>
       </c>
       <c r="C317" s="2" t="s">
-        <v>897</v>
+        <v>902</v>
       </c>
     </row>
     <row r="318" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A318" s="2" t="s">
-        <v>898</v>
+        <v>903</v>
       </c>
       <c r="B318" s="2" t="s">
-        <v>899</v>
+        <v>904</v>
       </c>
       <c r="C318" s="2" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
     </row>
     <row r="319" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A319" s="2" t="s">
-        <v>901</v>
+        <v>905</v>
       </c>
       <c r="B319" s="2" t="s">
-        <v>902</v>
+        <v>906</v>
       </c>
       <c r="C319" s="2" t="s">
-        <v>903</v>
+        <v>907</v>
       </c>
     </row>
     <row r="320" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A320" s="2" t="s">
-        <v>904</v>
+        <v>908</v>
       </c>
       <c r="B320" s="2" t="s">
-        <v>905</v>
+        <v>909</v>
       </c>
       <c r="C320" s="2" t="s">
-        <v>906</v>
+        <v>910</v>
       </c>
     </row>
     <row r="321" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A321" s="2" t="s">
-        <v>907</v>
+        <v>911</v>
       </c>
       <c r="B321" s="2" t="s">
-        <v>908</v>
+        <v>904</v>
       </c>
       <c r="C321" s="2" t="s">
-        <v>909</v>
+        <v>904</v>
       </c>
     </row>
     <row r="322" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A322" s="2" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
       <c r="B322" s="2" t="s">
-        <v>911</v>
+        <v>913</v>
       </c>
       <c r="C322" s="2" t="s">
-        <v>912</v>
+        <v>914</v>
       </c>
     </row>
     <row r="323" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A323" s="2" t="s">
-        <v>913</v>
+        <v>915</v>
       </c>
       <c r="B323" s="2" t="s">
-        <v>914</v>
+        <v>916</v>
       </c>
       <c r="C323" s="2" t="s">
-        <v>915</v>
+        <v>917</v>
       </c>
     </row>
     <row r="324" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A324" s="2" t="s">
-        <v>916</v>
+        <v>918</v>
       </c>
       <c r="B324" s="2" t="s">
-        <v>917</v>
+        <v>904</v>
       </c>
       <c r="C324" s="2" t="s">
-        <v>918</v>
+        <v>904</v>
       </c>
     </row>
     <row r="325" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8063,700 +7925,700 @@
         <v>925</v>
       </c>
       <c r="B327" s="2" t="s">
-        <v>926</v>
+        <v>904</v>
       </c>
       <c r="C327" s="2" t="s">
-        <v>927</v>
+        <v>904</v>
       </c>
     </row>
     <row r="328" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A328" s="2" t="s">
+        <v>926</v>
+      </c>
+      <c r="B328" s="2" t="s">
+        <v>927</v>
+      </c>
+      <c r="C328" s="2" t="s">
         <v>928</v>
-      </c>
-      <c r="B328" s="2" t="s">
-        <v>929</v>
-      </c>
-      <c r="C328" s="2" t="s">
-        <v>930</v>
       </c>
     </row>
     <row r="329" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A329" s="2" t="s">
+        <v>929</v>
+      </c>
+      <c r="B329" s="2" t="s">
+        <v>930</v>
+      </c>
+      <c r="C329" s="2" t="s">
         <v>931</v>
-      </c>
-      <c r="B329" s="2" t="s">
-        <v>932</v>
-      </c>
-      <c r="C329" s="2" t="s">
-        <v>933</v>
       </c>
     </row>
     <row r="330" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A330" s="2" t="s">
-        <v>934</v>
+        <v>932</v>
       </c>
       <c r="B330" s="2" t="s">
-        <v>935</v>
+        <v>904</v>
       </c>
       <c r="C330" s="2" t="s">
-        <v>936</v>
+        <v>904</v>
       </c>
     </row>
     <row r="331" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A331" s="2" t="s">
-        <v>937</v>
+        <v>933</v>
       </c>
       <c r="B331" s="2" t="s">
-        <v>938</v>
+        <v>934</v>
       </c>
       <c r="C331" s="2" t="s">
-        <v>939</v>
+        <v>935</v>
       </c>
     </row>
     <row r="332" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A332" s="2" t="s">
-        <v>940</v>
+        <v>936</v>
       </c>
       <c r="B332" s="2" t="s">
-        <v>496</v>
+        <v>937</v>
       </c>
       <c r="C332" s="2" t="s">
-        <v>497</v>
+        <v>938</v>
       </c>
     </row>
     <row r="333" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A333" s="2" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
       <c r="B333" s="2" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
       <c r="C333" s="2" t="s">
-        <v>943</v>
+        <v>940</v>
       </c>
     </row>
     <row r="334" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A334" s="2" t="s">
-        <v>944</v>
+        <v>941</v>
       </c>
       <c r="B334" s="2" t="s">
-        <v>945</v>
+        <v>942</v>
       </c>
       <c r="C334" s="2" t="s">
-        <v>946</v>
+        <v>943</v>
       </c>
     </row>
     <row r="335" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A335" s="2" t="s">
-        <v>947</v>
+        <v>944</v>
       </c>
       <c r="B335" s="2" t="s">
-        <v>948</v>
+        <v>945</v>
       </c>
       <c r="C335" s="2" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
     </row>
     <row r="336" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A336" s="2" t="s">
-        <v>949</v>
+        <v>947</v>
       </c>
       <c r="B336" s="2" t="s">
-        <v>950</v>
+        <v>940</v>
       </c>
       <c r="C336" s="2" t="s">
-        <v>950</v>
+        <v>940</v>
       </c>
     </row>
     <row r="337" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A337" s="2" t="s">
-        <v>951</v>
+        <v>948</v>
       </c>
       <c r="B337" s="2" t="s">
-        <v>952</v>
+        <v>949</v>
       </c>
       <c r="C337" s="2" t="s">
-        <v>953</v>
+        <v>950</v>
       </c>
     </row>
     <row r="338" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A338" s="2" t="s">
-        <v>954</v>
+        <v>951</v>
       </c>
       <c r="B338" s="2" t="s">
-        <v>955</v>
+        <v>952</v>
       </c>
       <c r="C338" s="2" t="s">
-        <v>956</v>
+        <v>953</v>
       </c>
     </row>
     <row r="339" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A339" s="2" t="s">
-        <v>957</v>
+        <v>954</v>
       </c>
       <c r="B339" s="2" t="s">
-        <v>950</v>
+        <v>940</v>
       </c>
       <c r="C339" s="2" t="s">
-        <v>950</v>
+        <v>940</v>
       </c>
     </row>
     <row r="340" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A340" s="2" t="s">
-        <v>958</v>
+        <v>955</v>
       </c>
       <c r="B340" s="2" t="s">
-        <v>959</v>
+        <v>956</v>
       </c>
       <c r="C340" s="2" t="s">
-        <v>960</v>
+        <v>957</v>
       </c>
     </row>
     <row r="341" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A341" s="2" t="s">
-        <v>961</v>
+        <v>958</v>
       </c>
       <c r="B341" s="2" t="s">
-        <v>962</v>
+        <v>959</v>
       </c>
       <c r="C341" s="2" t="s">
-        <v>963</v>
+        <v>960</v>
       </c>
     </row>
     <row r="342" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A342" s="2" t="s">
-        <v>964</v>
+        <v>961</v>
       </c>
       <c r="B342" s="2" t="s">
-        <v>950</v>
+        <v>940</v>
       </c>
       <c r="C342" s="2" t="s">
-        <v>950</v>
+        <v>940</v>
       </c>
     </row>
     <row r="343" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A343" s="2" t="s">
-        <v>965</v>
+        <v>962</v>
       </c>
       <c r="B343" s="2" t="s">
-        <v>966</v>
+        <v>963</v>
       </c>
       <c r="C343" s="2" t="s">
-        <v>967</v>
+        <v>964</v>
       </c>
     </row>
     <row r="344" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A344" s="2" t="s">
-        <v>968</v>
+        <v>965</v>
       </c>
       <c r="B344" s="2" t="s">
-        <v>969</v>
+        <v>966</v>
       </c>
       <c r="C344" s="2" t="s">
-        <v>970</v>
+        <v>967</v>
       </c>
     </row>
     <row r="345" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A345" s="2" t="s">
-        <v>971</v>
+        <v>968</v>
       </c>
       <c r="B345" s="2" t="s">
-        <v>950</v>
+        <v>940</v>
       </c>
       <c r="C345" s="2" t="s">
-        <v>950</v>
+        <v>940</v>
       </c>
     </row>
     <row r="346" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A346" s="2" t="s">
-        <v>972</v>
+        <v>969</v>
       </c>
       <c r="B346" s="2" t="s">
-        <v>973</v>
+        <v>970</v>
       </c>
       <c r="C346" s="2" t="s">
-        <v>974</v>
+        <v>971</v>
       </c>
     </row>
     <row r="347" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A347" s="2" t="s">
-        <v>975</v>
+        <v>972</v>
       </c>
       <c r="B347" s="2" t="s">
-        <v>976</v>
+        <v>973</v>
       </c>
       <c r="C347" s="2" t="s">
-        <v>977</v>
+        <v>974</v>
       </c>
     </row>
     <row r="348" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A348" s="2" t="s">
-        <v>978</v>
+        <v>975</v>
       </c>
       <c r="B348" s="2" t="s">
-        <v>950</v>
+        <v>940</v>
       </c>
       <c r="C348" s="2" t="s">
-        <v>950</v>
+        <v>940</v>
       </c>
     </row>
     <row r="349" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A349" s="2" t="s">
-        <v>979</v>
+        <v>976</v>
       </c>
       <c r="B349" s="2" t="s">
-        <v>980</v>
+        <v>977</v>
       </c>
       <c r="C349" s="2" t="s">
-        <v>981</v>
+        <v>978</v>
       </c>
     </row>
     <row r="350" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A350" s="2" t="s">
-        <v>982</v>
+        <v>979</v>
       </c>
       <c r="B350" s="2" t="s">
-        <v>983</v>
+        <v>980</v>
       </c>
       <c r="C350" s="2" t="s">
-        <v>984</v>
+        <v>981</v>
       </c>
     </row>
     <row r="351" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A351" s="2" t="s">
-        <v>985</v>
+        <v>982</v>
       </c>
       <c r="B351" s="2" t="s">
-        <v>986</v>
+        <v>940</v>
       </c>
       <c r="C351" s="2" t="s">
-        <v>986</v>
+        <v>940</v>
       </c>
     </row>
     <row r="352" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A352" s="2" t="s">
-        <v>987</v>
+        <v>983</v>
       </c>
       <c r="B352" s="2" t="s">
-        <v>988</v>
+        <v>984</v>
       </c>
       <c r="C352" s="2" t="s">
-        <v>989</v>
+        <v>985</v>
       </c>
     </row>
     <row r="353" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A353" s="2" t="s">
-        <v>990</v>
+        <v>986</v>
       </c>
       <c r="B353" s="2" t="s">
-        <v>991</v>
+        <v>987</v>
       </c>
       <c r="C353" s="2" t="s">
-        <v>992</v>
+        <v>988</v>
       </c>
     </row>
     <row r="354" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A354" s="2" t="s">
-        <v>993</v>
+        <v>989</v>
       </c>
       <c r="B354" s="2" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
       <c r="C354" s="2" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
     </row>
     <row r="355" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A355" s="2" t="s">
-        <v>994</v>
+        <v>991</v>
       </c>
       <c r="B355" s="2" t="s">
-        <v>995</v>
+        <v>992</v>
       </c>
       <c r="C355" s="2" t="s">
-        <v>996</v>
+        <v>993</v>
       </c>
     </row>
     <row r="356" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A356" s="2" t="s">
-        <v>997</v>
+        <v>994</v>
       </c>
       <c r="B356" s="2" t="s">
-        <v>998</v>
+        <v>995</v>
       </c>
       <c r="C356" s="2" t="s">
-        <v>999</v>
+        <v>996</v>
       </c>
     </row>
     <row r="357" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A357" s="2" t="s">
-        <v>1000</v>
+        <v>997</v>
       </c>
       <c r="B357" s="2" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
       <c r="C357" s="2" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
     </row>
     <row r="358" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A358" s="2" t="s">
-        <v>1001</v>
+        <v>998</v>
       </c>
       <c r="B358" s="2" t="s">
-        <v>1002</v>
+        <v>999</v>
       </c>
       <c r="C358" s="2" t="s">
-        <v>1003</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="359" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A359" s="2" t="s">
-        <v>1004</v>
+        <v>1001</v>
       </c>
       <c r="B359" s="2" t="s">
-        <v>1005</v>
+        <v>1002</v>
       </c>
       <c r="C359" s="2" t="s">
-        <v>1006</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="360" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A360" s="2" t="s">
-        <v>1007</v>
+        <v>1004</v>
       </c>
       <c r="B360" s="2" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
       <c r="C360" s="2" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
     </row>
     <row r="361" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A361" s="2" t="s">
-        <v>1008</v>
+        <v>1005</v>
       </c>
       <c r="B361" s="2" t="s">
-        <v>1009</v>
+        <v>1006</v>
       </c>
       <c r="C361" s="2" t="s">
-        <v>1010</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="362" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A362" s="2" t="s">
-        <v>1011</v>
+        <v>1008</v>
       </c>
       <c r="B362" s="2" t="s">
-        <v>1012</v>
+        <v>1009</v>
       </c>
       <c r="C362" s="2" t="s">
-        <v>1013</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="363" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A363" s="2" t="s">
-        <v>1014</v>
+        <v>1011</v>
       </c>
       <c r="B363" s="2" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
       <c r="C363" s="2" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
     </row>
     <row r="364" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A364" s="2" t="s">
-        <v>1015</v>
+        <v>1012</v>
       </c>
       <c r="B364" s="2" t="s">
-        <v>1016</v>
+        <v>1013</v>
       </c>
       <c r="C364" s="2" t="s">
-        <v>1017</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="365" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A365" s="2" t="s">
-        <v>1018</v>
+        <v>1015</v>
       </c>
       <c r="B365" s="2" t="s">
-        <v>1019</v>
+        <v>1016</v>
       </c>
       <c r="C365" s="2" t="s">
-        <v>1020</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="366" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A366" s="2" t="s">
-        <v>1021</v>
+        <v>1018</v>
       </c>
       <c r="B366" s="2" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
       <c r="C366" s="2" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
     </row>
     <row r="367" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A367" s="2" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="B367" s="2" t="s">
-        <v>1023</v>
+        <v>1020</v>
       </c>
       <c r="C367" s="2" t="s">
-        <v>1024</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="368" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A368" s="2" t="s">
-        <v>1025</v>
+        <v>1022</v>
       </c>
       <c r="B368" s="2" t="s">
-        <v>1026</v>
+        <v>1023</v>
       </c>
       <c r="C368" s="2" t="s">
-        <v>1027</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="369" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A369" s="2" t="s">
-        <v>1028</v>
+        <v>1025</v>
       </c>
       <c r="B369" s="2" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
       <c r="C369" s="2" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
     </row>
     <row r="370" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A370" s="2" t="s">
-        <v>1029</v>
+        <v>1026</v>
       </c>
       <c r="B370" s="2" t="s">
-        <v>1030</v>
+        <v>1027</v>
       </c>
       <c r="C370" s="2" t="s">
-        <v>1031</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="371" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A371" s="2" t="s">
-        <v>1032</v>
+        <v>1029</v>
       </c>
       <c r="B371" s="2" t="s">
-        <v>1033</v>
+        <v>1030</v>
       </c>
       <c r="C371" s="2" t="s">
-        <v>1034</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="372" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A372" s="2" t="s">
-        <v>1035</v>
+        <v>1032</v>
       </c>
       <c r="B372" s="2" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="C372" s="2" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="373" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A373" s="2" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="B373" s="2" t="s">
-        <v>1038</v>
+        <v>1035</v>
       </c>
       <c r="C373" s="2" t="s">
-        <v>1039</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="374" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A374" s="2" t="s">
-        <v>1040</v>
+        <v>1037</v>
       </c>
       <c r="B374" s="2" t="s">
-        <v>1041</v>
+        <v>1038</v>
       </c>
       <c r="C374" s="2" t="s">
-        <v>1042</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="375" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A375" s="2" t="s">
-        <v>1043</v>
+        <v>1040</v>
       </c>
       <c r="B375" s="2" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="C375" s="2" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="376" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A376" s="2" t="s">
-        <v>1044</v>
+        <v>1041</v>
       </c>
       <c r="B376" s="2" t="s">
-        <v>1045</v>
+        <v>1042</v>
       </c>
       <c r="C376" s="2" t="s">
-        <v>1046</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="377" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A377" s="2" t="s">
-        <v>1047</v>
+        <v>1044</v>
       </c>
       <c r="B377" s="2" t="s">
-        <v>1048</v>
+        <v>1045</v>
       </c>
       <c r="C377" s="2" t="s">
-        <v>1049</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="378" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A378" s="2" t="s">
-        <v>1050</v>
+        <v>1047</v>
       </c>
       <c r="B378" s="2" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="C378" s="2" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="379" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A379" s="2" t="s">
-        <v>1051</v>
+        <v>1048</v>
       </c>
       <c r="B379" s="2" t="s">
-        <v>1052</v>
+        <v>1049</v>
       </c>
       <c r="C379" s="2" t="s">
-        <v>1053</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="380" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A380" s="2" t="s">
-        <v>1054</v>
+        <v>1051</v>
       </c>
       <c r="B380" s="2" t="s">
-        <v>1055</v>
+        <v>1052</v>
       </c>
       <c r="C380" s="2" t="s">
-        <v>1056</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="381" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A381" s="2" t="s">
-        <v>1057</v>
+        <v>1054</v>
       </c>
       <c r="B381" s="2" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="C381" s="2" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="382" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A382" s="2" t="s">
-        <v>1058</v>
+        <v>1055</v>
       </c>
       <c r="B382" s="2" t="s">
-        <v>1059</v>
+        <v>1056</v>
       </c>
       <c r="C382" s="2" t="s">
-        <v>1060</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="383" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A383" s="2" t="s">
-        <v>1061</v>
+        <v>1058</v>
       </c>
       <c r="B383" s="2" t="s">
-        <v>1062</v>
+        <v>1059</v>
       </c>
       <c r="C383" s="2" t="s">
-        <v>1063</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="384" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A384" s="2" t="s">
-        <v>1064</v>
+        <v>1061</v>
       </c>
       <c r="B384" s="2" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="C384" s="2" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="385" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A385" s="2" t="s">
-        <v>1065</v>
+        <v>1062</v>
       </c>
       <c r="B385" s="2" t="s">
-        <v>1066</v>
+        <v>1063</v>
       </c>
       <c r="C385" s="2" t="s">
-        <v>1067</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="386" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A386" s="2" t="s">
-        <v>1068</v>
+        <v>1065</v>
       </c>
       <c r="B386" s="2" t="s">
-        <v>1069</v>
+        <v>1066</v>
       </c>
       <c r="C386" s="2" t="s">
-        <v>1070</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="387" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A387" s="2" t="s">
-        <v>1071</v>
+        <v>1068</v>
       </c>
       <c r="B387" s="2" t="s">
-        <v>1036</v>
+        <v>1069</v>
       </c>
       <c r="C387" s="2" t="s">
-        <v>1036</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="388" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A388" s="2" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B388" s="2" t="s">
         <v>1072</v>
       </c>
-      <c r="B388" s="2" t="s">
+      <c r="C388" s="2" t="s">
         <v>1073</v>
-      </c>
-      <c r="C388" s="2" t="s">
-        <v>1074</v>
       </c>
     </row>
     <row r="389" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A389" s="2" t="s">
+        <v>1074</v>
+      </c>
+      <c r="B389" s="2" t="s">
         <v>1075</v>
       </c>
-      <c r="B389" s="2" t="s">
+      <c r="C389" s="2" t="s">
         <v>1076</v>
-      </c>
-      <c r="C389" s="2" t="s">
-        <v>1077</v>
       </c>
     </row>
     <row r="390" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A390" s="2" t="s">
+        <v>1077</v>
+      </c>
+      <c r="B390" s="2" t="s">
         <v>1078</v>
-      </c>
-      <c r="B390" s="2" t="s">
-        <v>1079</v>
       </c>
       <c r="C390" s="2" t="s">
         <v>1079</v>
@@ -8781,18 +8643,18 @@
         <v>1084</v>
       </c>
       <c r="C392" s="2" t="s">
-        <v>1085</v>
+        <v>500</v>
       </c>
     </row>
     <row r="393" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A393" s="2" t="s">
+        <v>1085</v>
+      </c>
+      <c r="B393" s="2" t="s">
         <v>1086</v>
       </c>
-      <c r="B393" s="2" t="s">
-        <v>1079</v>
-      </c>
       <c r="C393" s="2" t="s">
-        <v>1079</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="394" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8822,10 +8684,10 @@
         <v>1093</v>
       </c>
       <c r="B396" s="2" t="s">
-        <v>1079</v>
+        <v>600</v>
       </c>
       <c r="C396" s="2" t="s">
-        <v>1079</v>
+        <v>601</v>
       </c>
     </row>
     <row r="397" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8833,65 +8695,65 @@
         <v>1094</v>
       </c>
       <c r="B397" s="2" t="s">
-        <v>1095</v>
+        <v>624</v>
       </c>
       <c r="C397" s="2" t="s">
-        <v>1096</v>
+        <v>67</v>
       </c>
     </row>
     <row r="398" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A398" s="2" t="s">
-        <v>1097</v>
+        <v>1095</v>
       </c>
       <c r="B398" s="2" t="s">
-        <v>1098</v>
+        <v>99</v>
       </c>
       <c r="C398" s="2" t="s">
-        <v>1099</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="399" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A399" s="2" t="s">
-        <v>1100</v>
+        <v>1097</v>
       </c>
       <c r="B399" s="2" t="s">
-        <v>1079</v>
+        <v>1098</v>
       </c>
       <c r="C399" s="2" t="s">
-        <v>1079</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="400" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A400" s="2" t="s">
+        <v>1100</v>
+      </c>
+      <c r="B400" s="2" t="s">
         <v>1101</v>
       </c>
-      <c r="B400" s="2" t="s">
+      <c r="C400" s="2" t="s">
         <v>1102</v>
-      </c>
-      <c r="C400" s="2" t="s">
-        <v>1103</v>
       </c>
     </row>
     <row r="401" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A401" s="2" t="s">
+        <v>1103</v>
+      </c>
+      <c r="B401" s="2" t="s">
         <v>1104</v>
       </c>
-      <c r="B401" s="2" t="s">
-        <v>1105</v>
-      </c>
       <c r="C401" s="2" t="s">
-        <v>1106</v>
+        <v>82</v>
       </c>
     </row>
     <row r="402" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A402" s="2" t="s">
+        <v>1105</v>
+      </c>
+      <c r="B402" s="2" t="s">
+        <v>1106</v>
+      </c>
+      <c r="C402" s="2" t="s">
         <v>1107</v>
-      </c>
-      <c r="B402" s="2" t="s">
-        <v>1079</v>
-      </c>
-      <c r="C402" s="2" t="s">
-        <v>1079</v>
       </c>
     </row>
     <row r="403" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8935,356 +8797,356 @@
         <v>1118</v>
       </c>
       <c r="C406" s="2" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="407" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A407" s="2" t="s">
+        <v>1119</v>
+      </c>
+      <c r="B407" s="2" t="s">
         <v>1120</v>
       </c>
-      <c r="B407" s="2" t="s">
+      <c r="C407" s="2" t="s">
         <v>1121</v>
-      </c>
-      <c r="C407" s="2" t="s">
-        <v>1122</v>
       </c>
     </row>
     <row r="408" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A408" s="2" t="s">
+        <v>1122</v>
+      </c>
+      <c r="B408" s="2" t="s">
         <v>1123</v>
       </c>
-      <c r="B408" s="2" t="s">
-        <v>1124</v>
-      </c>
       <c r="C408" s="2" t="s">
-        <v>1125</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="409" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A409" s="2" t="s">
-        <v>1126</v>
+        <v>1124</v>
       </c>
       <c r="B409" s="2" t="s">
-        <v>1127</v>
+        <v>323</v>
       </c>
       <c r="C409" s="2" t="s">
-        <v>1128</v>
+        <v>324</v>
       </c>
     </row>
     <row r="410" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A410" s="2" t="s">
-        <v>1129</v>
+        <v>1125</v>
       </c>
       <c r="B410" s="2" t="s">
-        <v>1130</v>
+        <v>1126</v>
       </c>
       <c r="C410" s="2" t="s">
-        <v>500</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="411" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A411" s="2" t="s">
-        <v>1131</v>
+        <v>1127</v>
       </c>
       <c r="B411" s="2" t="s">
-        <v>1132</v>
+        <v>1128</v>
       </c>
       <c r="C411" s="2" t="s">
-        <v>1132</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="412" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A412" s="2" t="s">
-        <v>1133</v>
+        <v>1129</v>
       </c>
       <c r="B412" s="2" t="s">
-        <v>1134</v>
+        <v>1130</v>
       </c>
       <c r="C412" s="2" t="s">
-        <v>1135</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="413" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A413" s="2" t="s">
-        <v>1136</v>
+        <v>1131</v>
       </c>
       <c r="B413" s="2" t="s">
-        <v>1137</v>
+        <v>329</v>
       </c>
       <c r="C413" s="2" t="s">
-        <v>1138</v>
+        <v>330</v>
       </c>
     </row>
     <row r="414" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A414" s="2" t="s">
-        <v>1139</v>
+        <v>1132</v>
       </c>
       <c r="B414" s="2" t="s">
-        <v>646</v>
+        <v>1133</v>
       </c>
       <c r="C414" s="2" t="s">
-        <v>647</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="415" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A415" s="2" t="s">
-        <v>1140</v>
+        <v>1134</v>
       </c>
       <c r="B415" s="2" t="s">
-        <v>670</v>
+        <v>1135</v>
       </c>
       <c r="C415" s="2" t="s">
-        <v>67</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="416" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A416" s="2" t="s">
-        <v>1141</v>
+        <v>1136</v>
       </c>
       <c r="B416" s="2" t="s">
-        <v>99</v>
+        <v>1137</v>
       </c>
       <c r="C416" s="2" t="s">
-        <v>1142</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="417" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A417" s="2" t="s">
-        <v>1143</v>
+        <v>1138</v>
       </c>
       <c r="B417" s="2" t="s">
-        <v>1144</v>
+        <v>1139</v>
       </c>
       <c r="C417" s="2" t="s">
-        <v>1145</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="418" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A418" s="2" t="s">
-        <v>1146</v>
+        <v>1141</v>
       </c>
       <c r="B418" s="2" t="s">
-        <v>1147</v>
+        <v>7</v>
       </c>
       <c r="C418" s="2" t="s">
-        <v>1148</v>
+        <v>8</v>
       </c>
     </row>
     <row r="419" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A419" s="2" t="s">
-        <v>1149</v>
+        <v>1142</v>
       </c>
       <c r="B419" s="2" t="s">
-        <v>1150</v>
+        <v>1143</v>
       </c>
       <c r="C419" s="2" t="s">
-        <v>82</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="420" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A420" s="2" t="s">
-        <v>1151</v>
+        <v>1144</v>
       </c>
       <c r="B420" s="2" t="s">
-        <v>1152</v>
+        <v>1145</v>
       </c>
       <c r="C420" s="2" t="s">
-        <v>1153</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="421" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A421" s="2" t="s">
-        <v>1154</v>
+        <v>1146</v>
       </c>
       <c r="B421" s="2" t="s">
-        <v>1155</v>
+        <v>332</v>
       </c>
       <c r="C421" s="2" t="s">
-        <v>1156</v>
+        <v>333</v>
       </c>
     </row>
     <row r="422" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A422" s="2" t="s">
-        <v>1157</v>
+        <v>1147</v>
       </c>
       <c r="B422" s="2" t="s">
-        <v>1158</v>
+        <v>1148</v>
       </c>
       <c r="C422" s="2" t="s">
-        <v>1159</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="423" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A423" s="2" t="s">
-        <v>1160</v>
+        <v>1149</v>
       </c>
       <c r="B423" s="2" t="s">
-        <v>1161</v>
+        <v>1135</v>
       </c>
       <c r="C423" s="2" t="s">
-        <v>1162</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="424" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A424" s="2" t="s">
-        <v>1163</v>
+        <v>1150</v>
       </c>
       <c r="B424" s="2" t="s">
-        <v>1164</v>
+        <v>1151</v>
       </c>
       <c r="C424" s="2" t="s">
-        <v>1164</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="425" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A425" s="2" t="s">
-        <v>1165</v>
+        <v>1153</v>
       </c>
       <c r="B425" s="2" t="s">
-        <v>1166</v>
+        <v>1154</v>
       </c>
       <c r="C425" s="2" t="s">
-        <v>1167</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="426" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A426" s="2" t="s">
-        <v>1168</v>
+        <v>1156</v>
       </c>
       <c r="B426" s="2" t="s">
-        <v>1169</v>
+        <v>1157</v>
       </c>
       <c r="C426" s="2" t="s">
-        <v>1169</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="427" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A427" s="2" t="s">
-        <v>1170</v>
+        <v>1159</v>
       </c>
       <c r="B427" s="2" t="s">
-        <v>323</v>
+        <v>1160</v>
       </c>
       <c r="C427" s="2" t="s">
-        <v>324</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="428" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A428" s="2" t="s">
-        <v>1171</v>
+        <v>1162</v>
       </c>
       <c r="B428" s="2" t="s">
-        <v>1172</v>
+        <v>1163</v>
       </c>
       <c r="C428" s="2" t="s">
-        <v>1172</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="429" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A429" s="2" t="s">
-        <v>1173</v>
+        <v>1165</v>
       </c>
       <c r="B429" s="2" t="s">
-        <v>1174</v>
+        <v>1166</v>
       </c>
       <c r="C429" s="2" t="s">
-        <v>1174</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="430" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A430" s="2" t="s">
-        <v>1175</v>
+        <v>1168</v>
       </c>
       <c r="B430" s="2" t="s">
-        <v>1176</v>
+        <v>1169</v>
       </c>
       <c r="C430" s="2" t="s">
-        <v>1176</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="431" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A431" s="2" t="s">
-        <v>1177</v>
+        <v>1171</v>
       </c>
       <c r="B431" s="2" t="s">
-        <v>329</v>
+        <v>1172</v>
       </c>
       <c r="C431" s="2" t="s">
-        <v>330</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="432" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A432" s="2" t="s">
-        <v>1178</v>
+        <v>1174</v>
       </c>
       <c r="B432" s="2" t="s">
-        <v>1179</v>
+        <v>1175</v>
       </c>
       <c r="C432" s="2" t="s">
-        <v>1179</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="433" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A433" s="2" t="s">
-        <v>1180</v>
+        <v>1177</v>
       </c>
       <c r="B433" s="2" t="s">
-        <v>1181</v>
+        <v>1126</v>
       </c>
       <c r="C433" s="2" t="s">
-        <v>1181</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="434" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A434" s="2" t="s">
-        <v>1182</v>
+        <v>1178</v>
       </c>
       <c r="B434" s="2" t="s">
-        <v>1183</v>
+        <v>1179</v>
       </c>
       <c r="C434" s="2" t="s">
-        <v>1183</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="435" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A435" s="2" t="s">
-        <v>1184</v>
+        <v>1180</v>
       </c>
       <c r="B435" s="2" t="s">
-        <v>1185</v>
+        <v>1181</v>
       </c>
       <c r="C435" s="2" t="s">
-        <v>1186</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="436" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A436" s="2" t="s">
-        <v>1187</v>
+        <v>1183</v>
       </c>
       <c r="B436" s="2" t="s">
-        <v>7</v>
+        <v>1184</v>
       </c>
       <c r="C436" s="2" t="s">
-        <v>8</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="437" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A437" s="2" t="s">
+        <v>1186</v>
+      </c>
+      <c r="B437" s="2" t="s">
+        <v>1187</v>
+      </c>
+      <c r="C437" s="2" t="s">
         <v>1188</v>
-      </c>
-      <c r="B437" s="2" t="s">
-        <v>1189</v>
-      </c>
-      <c r="C437" s="2" t="s">
-        <v>1189</v>
       </c>
     </row>
     <row r="438" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A438" s="2" t="s">
+        <v>1189</v>
+      </c>
+      <c r="B438" s="2" t="s">
         <v>1190</v>
-      </c>
-      <c r="B438" s="2" t="s">
-        <v>1191</v>
       </c>
       <c r="C438" s="2" t="s">
         <v>1191</v>
@@ -9295,54 +9157,54 @@
         <v>1192</v>
       </c>
       <c r="B439" s="2" t="s">
-        <v>332</v>
+        <v>1193</v>
       </c>
       <c r="C439" s="2" t="s">
-        <v>333</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="440" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A440" s="2" t="s">
-        <v>1193</v>
+        <v>1195</v>
       </c>
       <c r="B440" s="2" t="s">
-        <v>1194</v>
+        <v>1196</v>
       </c>
       <c r="C440" s="2" t="s">
-        <v>1194</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="441" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A441" s="2" t="s">
-        <v>1195</v>
+        <v>1198</v>
       </c>
       <c r="B441" s="2" t="s">
-        <v>1181</v>
+        <v>1199</v>
       </c>
       <c r="C441" s="2" t="s">
-        <v>1181</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="442" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A442" s="2" t="s">
-        <v>1196</v>
+        <v>1200</v>
       </c>
       <c r="B442" s="2" t="s">
-        <v>1197</v>
+        <v>1133</v>
       </c>
       <c r="C442" s="2" t="s">
-        <v>1198</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="443" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A443" s="2" t="s">
-        <v>1199</v>
+        <v>1201</v>
       </c>
       <c r="B443" s="2" t="s">
-        <v>1200</v>
+        <v>329</v>
       </c>
       <c r="C443" s="2" t="s">
-        <v>1201</v>
+        <v>330</v>
       </c>
     </row>
     <row r="444" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9353,194 +9215,194 @@
         <v>1203</v>
       </c>
       <c r="C444" s="2" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="445" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A445" s="2" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
       <c r="B445" s="2" t="s">
-        <v>1206</v>
+        <v>1133</v>
       </c>
       <c r="C445" s="2" t="s">
-        <v>1207</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="446" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A446" s="2" t="s">
-        <v>1208</v>
+        <v>1205</v>
       </c>
       <c r="B446" s="2" t="s">
-        <v>1209</v>
+        <v>1206</v>
       </c>
       <c r="C446" s="2" t="s">
-        <v>1210</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="447" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A447" s="2" t="s">
-        <v>1211</v>
+        <v>1208</v>
       </c>
       <c r="B447" s="2" t="s">
-        <v>1212</v>
+        <v>1199</v>
       </c>
       <c r="C447" s="2" t="s">
-        <v>1213</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="448" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A448" s="2" t="s">
-        <v>1214</v>
+        <v>1209</v>
       </c>
       <c r="B448" s="2" t="s">
-        <v>1215</v>
+        <v>7</v>
       </c>
       <c r="C448" s="2" t="s">
-        <v>1216</v>
+        <v>8</v>
       </c>
     </row>
     <row r="449" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A449" s="2" t="s">
-        <v>1217</v>
+        <v>1210</v>
       </c>
       <c r="B449" s="2" t="s">
-        <v>1218</v>
+        <v>1211</v>
       </c>
       <c r="C449" s="2" t="s">
-        <v>1219</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="450" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A450" s="2" t="s">
-        <v>1220</v>
+        <v>1213</v>
       </c>
       <c r="B450" s="2" t="s">
-        <v>1221</v>
+        <v>1214</v>
       </c>
       <c r="C450" s="2" t="s">
-        <v>1222</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="451" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A451" s="2" t="s">
-        <v>1223</v>
+        <v>1216</v>
       </c>
       <c r="B451" s="2" t="s">
-        <v>1172</v>
+        <v>1217</v>
       </c>
       <c r="C451" s="2" t="s">
-        <v>1172</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="452" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A452" s="2" t="s">
-        <v>1224</v>
+        <v>1219</v>
       </c>
       <c r="B452" s="2" t="s">
-        <v>1225</v>
+        <v>1220</v>
       </c>
       <c r="C452" s="2" t="s">
-        <v>1225</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="453" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A453" s="2" t="s">
-        <v>1226</v>
+        <v>1222</v>
       </c>
       <c r="B453" s="2" t="s">
-        <v>1227</v>
+        <v>1223</v>
       </c>
       <c r="C453" s="2" t="s">
-        <v>1228</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="454" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A454" s="2" t="s">
-        <v>1229</v>
+        <v>1225</v>
       </c>
       <c r="B454" s="2" t="s">
-        <v>1230</v>
+        <v>1226</v>
       </c>
       <c r="C454" s="2" t="s">
-        <v>1231</v>
+        <v>1227</v>
       </c>
     </row>
     <row r="455" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A455" s="2" t="s">
-        <v>1232</v>
+        <v>1228</v>
       </c>
       <c r="B455" s="2" t="s">
-        <v>1233</v>
+        <v>1229</v>
       </c>
       <c r="C455" s="2" t="s">
-        <v>1234</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="456" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A456" s="2" t="s">
-        <v>1235</v>
+        <v>1231</v>
       </c>
       <c r="B456" s="2" t="s">
-        <v>1236</v>
+        <v>1232</v>
       </c>
       <c r="C456" s="2" t="s">
-        <v>1237</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="457" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A457" s="2" t="s">
-        <v>1238</v>
+        <v>1234</v>
       </c>
       <c r="B457" s="2" t="s">
-        <v>1239</v>
+        <v>1235</v>
       </c>
       <c r="C457" s="2" t="s">
-        <v>1240</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="458" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A458" s="2" t="s">
-        <v>1241</v>
+        <v>1236</v>
       </c>
       <c r="B458" s="2" t="s">
-        <v>1242</v>
+        <v>1237</v>
       </c>
       <c r="C458" s="2" t="s">
-        <v>1243</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="459" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A459" s="2" t="s">
-        <v>1244</v>
+        <v>1239</v>
       </c>
       <c r="B459" s="2" t="s">
-        <v>1245</v>
+        <v>1240</v>
       </c>
       <c r="C459" s="2" t="s">
-        <v>1245</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="460" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A460" s="2" t="s">
-        <v>1246</v>
+        <v>1242</v>
       </c>
       <c r="B460" s="2" t="s">
-        <v>1179</v>
+        <v>1243</v>
       </c>
       <c r="C460" s="2" t="s">
-        <v>1179</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="461" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A461" s="2" t="s">
+        <v>1245</v>
+      </c>
+      <c r="B461" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C461" s="2" t="s">
         <v>1247</v>
-      </c>
-      <c r="B461" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="C461" s="2" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="462" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9551,227 +9413,227 @@
         <v>1249</v>
       </c>
       <c r="C462" s="2" t="s">
-        <v>1249</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="463" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A463" s="2" t="s">
-        <v>1250</v>
+        <v>1251</v>
       </c>
       <c r="B463" s="2" t="s">
-        <v>1179</v>
+        <v>1252</v>
       </c>
       <c r="C463" s="2" t="s">
-        <v>1179</v>
+        <v>1253</v>
       </c>
     </row>
     <row r="464" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A464" s="2" t="s">
-        <v>1251</v>
+        <v>1254</v>
       </c>
       <c r="B464" s="2" t="s">
-        <v>1252</v>
+        <v>1255</v>
       </c>
       <c r="C464" s="2" t="s">
-        <v>1253</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="465" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A465" s="2" t="s">
-        <v>1254</v>
+        <v>1257</v>
       </c>
       <c r="B465" s="2" t="s">
-        <v>1245</v>
+        <v>1258</v>
       </c>
       <c r="C465" s="2" t="s">
-        <v>1245</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="466" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A466" s="2" t="s">
-        <v>1255</v>
+        <v>1260</v>
       </c>
       <c r="B466" s="2" t="s">
-        <v>7</v>
+        <v>1261</v>
       </c>
       <c r="C466" s="2" t="s">
-        <v>8</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="467" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A467" s="2" t="s">
-        <v>1256</v>
+        <v>1263</v>
       </c>
       <c r="B467" s="2" t="s">
-        <v>1257</v>
+        <v>1264</v>
       </c>
       <c r="C467" s="2" t="s">
-        <v>1258</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="468" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A468" s="2" t="s">
-        <v>1259</v>
+        <v>1266</v>
       </c>
       <c r="B468" s="2" t="s">
-        <v>1260</v>
+        <v>1267</v>
       </c>
       <c r="C468" s="2" t="s">
-        <v>1261</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="469" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A469" s="2" t="s">
-        <v>1262</v>
+        <v>1269</v>
       </c>
       <c r="B469" s="2" t="s">
-        <v>1263</v>
+        <v>1270</v>
       </c>
       <c r="C469" s="2" t="s">
-        <v>1264</v>
+        <v>1271</v>
       </c>
     </row>
     <row r="470" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A470" s="2" t="s">
-        <v>1265</v>
+        <v>1272</v>
       </c>
       <c r="B470" s="2" t="s">
-        <v>1266</v>
+        <v>1273</v>
       </c>
       <c r="C470" s="2" t="s">
-        <v>1267</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="471" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A471" s="2" t="s">
-        <v>1268</v>
+        <v>1275</v>
       </c>
       <c r="B471" s="2" t="s">
-        <v>1269</v>
+        <v>1276</v>
       </c>
       <c r="C471" s="2" t="s">
-        <v>1270</v>
+        <v>1277</v>
       </c>
     </row>
     <row r="472" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A472" s="2" t="s">
-        <v>1271</v>
+        <v>1278</v>
       </c>
       <c r="B472" s="2" t="s">
-        <v>1272</v>
+        <v>1279</v>
       </c>
       <c r="C472" s="2" t="s">
-        <v>1273</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="473" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A473" s="2" t="s">
-        <v>1274</v>
+        <v>1281</v>
       </c>
       <c r="B473" s="2" t="s">
-        <v>1275</v>
+        <v>1282</v>
       </c>
       <c r="C473" s="2" t="s">
-        <v>1276</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="474" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A474" s="2" t="s">
-        <v>1277</v>
+        <v>1284</v>
       </c>
       <c r="B474" s="2" t="s">
-        <v>1278</v>
+        <v>1285</v>
       </c>
       <c r="C474" s="2" t="s">
-        <v>1279</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="475" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A475" s="2" t="s">
-        <v>1280</v>
+        <v>1287</v>
       </c>
       <c r="B475" s="2" t="s">
-        <v>1281</v>
+        <v>1288</v>
       </c>
       <c r="C475" s="2" t="s">
-        <v>1281</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="476" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A476" s="2" t="s">
-        <v>1282</v>
+        <v>1290</v>
       </c>
       <c r="B476" s="2" t="s">
-        <v>1283</v>
+        <v>1291</v>
       </c>
       <c r="C476" s="2" t="s">
-        <v>1284</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="477" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A477" s="2" t="s">
-        <v>1285</v>
+        <v>1293</v>
       </c>
       <c r="B477" s="2" t="s">
-        <v>1286</v>
+        <v>1294</v>
       </c>
       <c r="C477" s="2" t="s">
-        <v>1287</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="478" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A478" s="2" t="s">
-        <v>1288</v>
+        <v>1296</v>
       </c>
       <c r="B478" s="2" t="s">
-        <v>1289</v>
+        <v>1297</v>
       </c>
       <c r="C478" s="2" t="s">
-        <v>1290</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="479" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A479" s="2" t="s">
-        <v>1291</v>
+        <v>1298</v>
       </c>
       <c r="B479" s="2" t="s">
-        <v>1292</v>
+        <v>1299</v>
       </c>
       <c r="C479" s="2" t="s">
-        <v>1293</v>
+        <v>1299</v>
       </c>
     </row>
     <row r="480" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A480" s="2" t="s">
-        <v>1294</v>
+        <v>1300</v>
       </c>
       <c r="B480" s="2" t="s">
-        <v>1295</v>
+        <v>1123</v>
       </c>
       <c r="C480" s="2" t="s">
-        <v>1296</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="481" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A481" s="2" t="s">
-        <v>1297</v>
+        <v>1301</v>
       </c>
       <c r="B481" s="2" t="s">
-        <v>1298</v>
+        <v>323</v>
       </c>
       <c r="C481" s="2" t="s">
-        <v>1299</v>
+        <v>324</v>
       </c>
     </row>
     <row r="482" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A482" s="2" t="s">
-        <v>1300</v>
+        <v>1302</v>
       </c>
       <c r="B482" s="2" t="s">
-        <v>1301</v>
+        <v>1126</v>
       </c>
       <c r="C482" s="2" t="s">
-        <v>1302</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="483" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9779,262 +9641,64 @@
         <v>1303</v>
       </c>
       <c r="B483" s="2" t="s">
-        <v>1304</v>
+        <v>1130</v>
       </c>
       <c r="C483" s="2" t="s">
-        <v>1305</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="484" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A484" s="2" t="s">
-        <v>1306</v>
+        <v>1304</v>
       </c>
       <c r="B484" s="2" t="s">
-        <v>1307</v>
+        <v>329</v>
       </c>
       <c r="C484" s="2" t="s">
-        <v>1308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="485" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A485" s="2" t="s">
-        <v>1309</v>
+        <v>1305</v>
       </c>
       <c r="B485" s="2" t="s">
-        <v>1310</v>
+        <v>1133</v>
       </c>
       <c r="C485" s="2" t="s">
-        <v>1311</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="486" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A486" s="2" t="s">
-        <v>1312</v>
+        <v>1306</v>
       </c>
       <c r="B486" s="2" t="s">
-        <v>1313</v>
+        <v>1137</v>
       </c>
       <c r="C486" s="2" t="s">
-        <v>1314</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="487" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A487" s="2" t="s">
-        <v>1315</v>
+        <v>1307</v>
       </c>
       <c r="B487" s="2" t="s">
-        <v>1316</v>
+        <v>1139</v>
       </c>
       <c r="C487" s="2" t="s">
-        <v>1317</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="488" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A488" s="2" t="s">
-        <v>1318</v>
+        <v>1308</v>
       </c>
       <c r="B488" s="2" t="s">
-        <v>1319</v>
+        <v>7</v>
       </c>
       <c r="C488" s="2" t="s">
-        <v>1320</v>
-      </c>
-    </row>
-    <row r="489" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A489" s="2" t="s">
-        <v>1321</v>
-      </c>
-      <c r="B489" s="2" t="s">
-        <v>1322</v>
-      </c>
-      <c r="C489" s="2" t="s">
-        <v>1323</v>
-      </c>
-    </row>
-    <row r="490" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A490" s="2" t="s">
-        <v>1324</v>
-      </c>
-      <c r="B490" s="2" t="s">
-        <v>1325</v>
-      </c>
-      <c r="C490" s="2" t="s">
-        <v>1326</v>
-      </c>
-    </row>
-    <row r="491" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A491" s="2" t="s">
-        <v>1327</v>
-      </c>
-      <c r="B491" s="2" t="s">
-        <v>1328</v>
-      </c>
-      <c r="C491" s="2" t="s">
-        <v>1329</v>
-      </c>
-    </row>
-    <row r="492" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A492" s="2" t="s">
-        <v>1330</v>
-      </c>
-      <c r="B492" s="2" t="s">
-        <v>1331</v>
-      </c>
-      <c r="C492" s="2" t="s">
-        <v>1332</v>
-      </c>
-    </row>
-    <row r="493" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A493" s="2" t="s">
-        <v>1333</v>
-      </c>
-      <c r="B493" s="2" t="s">
-        <v>1334</v>
-      </c>
-      <c r="C493" s="2" t="s">
-        <v>1335</v>
-      </c>
-    </row>
-    <row r="494" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A494" s="2" t="s">
-        <v>1336</v>
-      </c>
-      <c r="B494" s="2" t="s">
-        <v>1337</v>
-      </c>
-      <c r="C494" s="2" t="s">
-        <v>1338</v>
-      </c>
-    </row>
-    <row r="495" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A495" s="2" t="s">
-        <v>1339</v>
-      </c>
-      <c r="B495" s="2" t="s">
-        <v>1340</v>
-      </c>
-      <c r="C495" s="2" t="s">
-        <v>1341</v>
-      </c>
-    </row>
-    <row r="496" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A496" s="2" t="s">
-        <v>1342</v>
-      </c>
-      <c r="B496" s="2" t="s">
-        <v>1343</v>
-      </c>
-      <c r="C496" s="2" t="s">
-        <v>1148</v>
-      </c>
-    </row>
-    <row r="497" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A497" s="2" t="s">
-        <v>1344</v>
-      </c>
-      <c r="B497" s="2" t="s">
-        <v>1345</v>
-      </c>
-      <c r="C497" s="2" t="s">
-        <v>1345</v>
-      </c>
-    </row>
-    <row r="498" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A498" s="2" t="s">
-        <v>1346</v>
-      </c>
-      <c r="B498" s="2" t="s">
-        <v>1169</v>
-      </c>
-      <c r="C498" s="2" t="s">
-        <v>1169</v>
-      </c>
-    </row>
-    <row r="499" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A499" s="2" t="s">
-        <v>1347</v>
-      </c>
-      <c r="B499" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="C499" s="2" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="500" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A500" s="2" t="s">
-        <v>1348</v>
-      </c>
-      <c r="B500" s="2" t="s">
-        <v>1172</v>
-      </c>
-      <c r="C500" s="2" t="s">
-        <v>1172</v>
-      </c>
-    </row>
-    <row r="501" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A501" s="2" t="s">
-        <v>1349</v>
-      </c>
-      <c r="B501" s="2" t="s">
-        <v>1176</v>
-      </c>
-      <c r="C501" s="2" t="s">
-        <v>1176</v>
-      </c>
-    </row>
-    <row r="502" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A502" s="2" t="s">
-        <v>1350</v>
-      </c>
-      <c r="B502" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="C502" s="2" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="503" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A503" s="2" t="s">
-        <v>1351</v>
-      </c>
-      <c r="B503" s="2" t="s">
-        <v>1179</v>
-      </c>
-      <c r="C503" s="2" t="s">
-        <v>1179</v>
-      </c>
-    </row>
-    <row r="504" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A504" s="2" t="s">
-        <v>1352</v>
-      </c>
-      <c r="B504" s="2" t="s">
-        <v>1183</v>
-      </c>
-      <c r="C504" s="2" t="s">
-        <v>1183</v>
-      </c>
-    </row>
-    <row r="505" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A505" s="2" t="s">
-        <v>1353</v>
-      </c>
-      <c r="B505" s="2" t="s">
-        <v>1185</v>
-      </c>
-      <c r="C505" s="2" t="s">
-        <v>1186</v>
-      </c>
-    </row>
-    <row r="506" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A506" s="2" t="s">
-        <v>1354</v>
-      </c>
-      <c r="B506" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C506" s="2" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>